<commit_message>
Activos de Ciudad: cotejo con el plano de Verasol, «filtrante a» = simple, SISTEMA_VBC.bat abre el mapa CJB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DgLunmnneanaNJXpuCaofT
</commit_message>
<xml_diff>
--- a/Activos/PLANTILLA_ANALISIS_CHARCOS_CJB.xlsx
+++ b/Activos/PLANTILLA_ANALISIS_CHARCOS_CJB.xlsx
@@ -12800,7 +12800,7 @@
       </c>
       <c r="B172" s="22" t="inlineStr">
         <is>
-          <t>Filtrante tipo «A» (por confirmar)</t>
+          <t>Filtrante simple</t>
         </is>
       </c>
       <c r="C172" s="22" t="inlineStr">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="B173" s="22" t="inlineStr">
         <is>
-          <t>Filtrante tipo «A» (por confirmar)</t>
+          <t>Filtrante simple</t>
         </is>
       </c>
       <c r="C173" s="22" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="B174" s="22" t="inlineStr">
         <is>
-          <t>Filtrante tipo «A» (por confirmar)</t>
+          <t>Filtrante simple</t>
         </is>
       </c>
       <c r="C174" s="22" t="inlineStr">
@@ -12875,7 +12875,7 @@
       </c>
       <c r="B175" s="22" t="inlineStr">
         <is>
-          <t>Filtrante tipo «A» (por confirmar)</t>
+          <t>Filtrante simple</t>
         </is>
       </c>
       <c r="C175" s="22" t="inlineStr">
@@ -12900,7 +12900,7 @@
       </c>
       <c r="B176" s="22" t="inlineStr">
         <is>
-          <t>Filtrante tipo «A» (por confirmar)</t>
+          <t>Filtrante simple</t>
         </is>
       </c>
       <c r="C176" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Activos CJB: alto contraste, charcos animados con su extensión, leyenda de flujos y títulos por categoría
- Imbornales y charcos con colores vivos y doble contorno; calles translúcidas con satélite
- Charcos: mancha animada del largo × ancho, orientada según la calle (capa HTML animada por GPU)
- Pulso en el elemento seleccionado; leyenda «Cómo leer el mapa» en la ficha
- Plantilla de charcos: largo y ancho en metros
- Títulos del plano se ocultan cuando la categoría de su lote está apagada (sin tocar el SVG)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DgLunmnneanaNJXpuCaofT
</commit_message>
<xml_diff>
--- a/Activos/PLANTILLA_ANALISIS_CHARCOS_CJB.xlsx
+++ b/Activos/PLANTILLA_ANALISIS_CHARCOS_CJB.xlsx
@@ -18,7 +18,7 @@
     <definedName name="lst_origen">Listas!$B$2:$B$8</definedName>
     <definedName name="lst_causas">Listas!$C$2:$C$8</definedName>
     <definedName name="lst_afecta">Listas!$D$2:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Charcos'!$A$5:$R$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Charcos'!$A$5:$S$205</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lotes'!$A$5:$E$218</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -998,53 +998,65 @@
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Tamaño aproximado (m²)</t>
+          <t>Largo aproximado (m)</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Profundidad aproximada (cm)</t>
+          <t>Ancho aproximado (m)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="inlineStr">
         <is>
+          <t>Profundidad aproximada (cm)</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
           <t>Tiempo en secarse (horas)</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="5" t="inlineStr">
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>6. Al terminar</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="46" customHeight="1">
-      <c r="B40" s="6" t="inlineStr">
+    <row r="41" ht="46" customHeight="1">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Envío</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Guarde el archivo agregando su nombre y la fecha (por ejemplo «Charcos CJB - Delvinson - 2026-11-05») y envíelo al equipo de Data del Fideicomiso. Puede enviarlo por partes: se cargan todas las filas que estén completas.</t>
         </is>
@@ -1062,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R205"/>
+  <dimension ref="A1:S205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1079,10 +1091,11 @@
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="38" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="38" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1108,6 +1121,7 @@
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
       <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1132,6 +1146,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
     </row>
     <row r="3" ht="3" customHeight="1">
       <c r="A3" s="4" t="n"/>
@@ -1152,6 +1167,7 @@
       <c r="P3" s="4" t="n"/>
       <c r="Q3" s="4" t="n"/>
       <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
@@ -1221,25 +1237,30 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
+          <t>Metros, a lo largo de la calle</t>
+        </is>
+      </c>
+      <c r="O4" s="12" t="inlineStr">
+        <is>
+          <t>Metros, de lado a lado</t>
+        </is>
+      </c>
+      <c r="P4" s="12" t="inlineStr">
+        <is>
           <t>Número</t>
         </is>
       </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="Q4" s="12" t="inlineStr">
         <is>
           <t>Número</t>
         </is>
       </c>
-      <c r="P4" s="12" t="inlineStr">
-        <is>
-          <t>Número</t>
-        </is>
-      </c>
-      <c r="Q4" s="12" t="inlineStr">
+      <c r="R4" s="12" t="inlineStr">
         <is>
           <t>OneDrive, Drive o WhatsApp</t>
         </is>
       </c>
-      <c r="R4" s="12" t="inlineStr">
+      <c r="S4" s="12" t="inlineStr">
         <is>
           <t>Texto libre</t>
         </is>
@@ -1313,25 +1334,30 @@
       </c>
       <c r="N5" s="13" t="inlineStr">
         <is>
-          <t>Tamaño aproximado (m²)</t>
+          <t>Largo aproximado (m)</t>
         </is>
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
+          <t>Ancho aproximado (m)</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
           <t>Profundidad aproximada (cm)</t>
         </is>
       </c>
-      <c r="P5" s="13" t="inlineStr">
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>Tiempo en secarse (horas)</t>
         </is>
       </c>
-      <c r="Q5" s="13" t="inlineStr">
+      <c r="R5" s="13" t="inlineStr">
         <is>
           <t>Fotos o video (enlace)</t>
         </is>
       </c>
-      <c r="R5" s="13" t="inlineStr">
+      <c r="S5" s="13" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1344,7 +1370,7 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>IF(COUNTA(C6:R6)=0,"",IF(AND(C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",H6&lt;&gt;"",I6&lt;&gt;"",NOT(AND(LEFT(I6,7)="Sale de",J6="",K6=""))),"✔ Completa","Falta: "&amp;IF(C6="","fecha · ","")&amp;IF(D6="","ubicación · ","")&amp;IF(E6="","referencia · ","")&amp;IF(H6="","criticidad · ","")&amp;IF(I6="","origen del agua · ","")&amp;IF(AND(LEFT(I6,7)="Sale de",J6="",K6=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C6:S6)=0,"",IF(AND(C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",H6&lt;&gt;"",I6&lt;&gt;"",NOT(AND(LEFT(I6,7)="Sale de",J6="",K6=""))),"✔ Completa","Falta: "&amp;IF(C6="","fecha · ","")&amp;IF(D6="","ubicación · ","")&amp;IF(E6="","referencia · ","")&amp;IF(H6="","criticidad · ","")&amp;IF(I6="","origen del agua · ","")&amp;IF(AND(LEFT(I6,7)="Sale de",J6="",K6=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C6" s="17" t="n"/>
@@ -1361,8 +1387,9 @@
       <c r="N6" s="21" t="n"/>
       <c r="O6" s="21" t="n"/>
       <c r="P6" s="21" t="n"/>
-      <c r="Q6" s="18" t="n"/>
-      <c r="R6" s="19" t="n"/>
+      <c r="Q6" s="21" t="n"/>
+      <c r="R6" s="18" t="n"/>
+      <c r="S6" s="19" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
@@ -1371,7 +1398,7 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>IF(COUNTA(C7:R7)=0,"",IF(AND(C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",H7&lt;&gt;"",I7&lt;&gt;"",NOT(AND(LEFT(I7,7)="Sale de",J7="",K7=""))),"✔ Completa","Falta: "&amp;IF(C7="","fecha · ","")&amp;IF(D7="","ubicación · ","")&amp;IF(E7="","referencia · ","")&amp;IF(H7="","criticidad · ","")&amp;IF(I7="","origen del agua · ","")&amp;IF(AND(LEFT(I7,7)="Sale de",J7="",K7=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C7:S7)=0,"",IF(AND(C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",H7&lt;&gt;"",I7&lt;&gt;"",NOT(AND(LEFT(I7,7)="Sale de",J7="",K7=""))),"✔ Completa","Falta: "&amp;IF(C7="","fecha · ","")&amp;IF(D7="","ubicación · ","")&amp;IF(E7="","referencia · ","")&amp;IF(H7="","criticidad · ","")&amp;IF(I7="","origen del agua · ","")&amp;IF(AND(LEFT(I7,7)="Sale de",J7="",K7=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C7" s="17" t="n"/>
@@ -1388,8 +1415,9 @@
       <c r="N7" s="21" t="n"/>
       <c r="O7" s="21" t="n"/>
       <c r="P7" s="21" t="n"/>
-      <c r="Q7" s="18" t="n"/>
-      <c r="R7" s="19" t="n"/>
+      <c r="Q7" s="21" t="n"/>
+      <c r="R7" s="18" t="n"/>
+      <c r="S7" s="19" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
@@ -1398,7 +1426,7 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>IF(COUNTA(C8:R8)=0,"",IF(AND(C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",H8&lt;&gt;"",I8&lt;&gt;"",NOT(AND(LEFT(I8,7)="Sale de",J8="",K8=""))),"✔ Completa","Falta: "&amp;IF(C8="","fecha · ","")&amp;IF(D8="","ubicación · ","")&amp;IF(E8="","referencia · ","")&amp;IF(H8="","criticidad · ","")&amp;IF(I8="","origen del agua · ","")&amp;IF(AND(LEFT(I8,7)="Sale de",J8="",K8=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C8:S8)=0,"",IF(AND(C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",H8&lt;&gt;"",I8&lt;&gt;"",NOT(AND(LEFT(I8,7)="Sale de",J8="",K8=""))),"✔ Completa","Falta: "&amp;IF(C8="","fecha · ","")&amp;IF(D8="","ubicación · ","")&amp;IF(E8="","referencia · ","")&amp;IF(H8="","criticidad · ","")&amp;IF(I8="","origen del agua · ","")&amp;IF(AND(LEFT(I8,7)="Sale de",J8="",K8=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C8" s="17" t="n"/>
@@ -1415,8 +1443,9 @@
       <c r="N8" s="21" t="n"/>
       <c r="O8" s="21" t="n"/>
       <c r="P8" s="21" t="n"/>
-      <c r="Q8" s="18" t="n"/>
-      <c r="R8" s="19" t="n"/>
+      <c r="Q8" s="21" t="n"/>
+      <c r="R8" s="18" t="n"/>
+      <c r="S8" s="19" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
@@ -1425,7 +1454,7 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>IF(COUNTA(C9:R9)=0,"",IF(AND(C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",H9&lt;&gt;"",I9&lt;&gt;"",NOT(AND(LEFT(I9,7)="Sale de",J9="",K9=""))),"✔ Completa","Falta: "&amp;IF(C9="","fecha · ","")&amp;IF(D9="","ubicación · ","")&amp;IF(E9="","referencia · ","")&amp;IF(H9="","criticidad · ","")&amp;IF(I9="","origen del agua · ","")&amp;IF(AND(LEFT(I9,7)="Sale de",J9="",K9=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C9:S9)=0,"",IF(AND(C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",H9&lt;&gt;"",I9&lt;&gt;"",NOT(AND(LEFT(I9,7)="Sale de",J9="",K9=""))),"✔ Completa","Falta: "&amp;IF(C9="","fecha · ","")&amp;IF(D9="","ubicación · ","")&amp;IF(E9="","referencia · ","")&amp;IF(H9="","criticidad · ","")&amp;IF(I9="","origen del agua · ","")&amp;IF(AND(LEFT(I9,7)="Sale de",J9="",K9=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C9" s="17" t="n"/>
@@ -1442,8 +1471,9 @@
       <c r="N9" s="21" t="n"/>
       <c r="O9" s="21" t="n"/>
       <c r="P9" s="21" t="n"/>
-      <c r="Q9" s="18" t="n"/>
-      <c r="R9" s="19" t="n"/>
+      <c r="Q9" s="21" t="n"/>
+      <c r="R9" s="18" t="n"/>
+      <c r="S9" s="19" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="15" t="inlineStr">
@@ -1452,7 +1482,7 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>IF(COUNTA(C10:R10)=0,"",IF(AND(C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",H10&lt;&gt;"",I10&lt;&gt;"",NOT(AND(LEFT(I10,7)="Sale de",J10="",K10=""))),"✔ Completa","Falta: "&amp;IF(C10="","fecha · ","")&amp;IF(D10="","ubicación · ","")&amp;IF(E10="","referencia · ","")&amp;IF(H10="","criticidad · ","")&amp;IF(I10="","origen del agua · ","")&amp;IF(AND(LEFT(I10,7)="Sale de",J10="",K10=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C10:S10)=0,"",IF(AND(C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",H10&lt;&gt;"",I10&lt;&gt;"",NOT(AND(LEFT(I10,7)="Sale de",J10="",K10=""))),"✔ Completa","Falta: "&amp;IF(C10="","fecha · ","")&amp;IF(D10="","ubicación · ","")&amp;IF(E10="","referencia · ","")&amp;IF(H10="","criticidad · ","")&amp;IF(I10="","origen del agua · ","")&amp;IF(AND(LEFT(I10,7)="Sale de",J10="",K10=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C10" s="17" t="n"/>
@@ -1469,8 +1499,9 @@
       <c r="N10" s="21" t="n"/>
       <c r="O10" s="21" t="n"/>
       <c r="P10" s="21" t="n"/>
-      <c r="Q10" s="18" t="n"/>
-      <c r="R10" s="19" t="n"/>
+      <c r="Q10" s="21" t="n"/>
+      <c r="R10" s="18" t="n"/>
+      <c r="S10" s="19" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="15" t="inlineStr">
@@ -1479,7 +1510,7 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>IF(COUNTA(C11:R11)=0,"",IF(AND(C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",H11&lt;&gt;"",I11&lt;&gt;"",NOT(AND(LEFT(I11,7)="Sale de",J11="",K11=""))),"✔ Completa","Falta: "&amp;IF(C11="","fecha · ","")&amp;IF(D11="","ubicación · ","")&amp;IF(E11="","referencia · ","")&amp;IF(H11="","criticidad · ","")&amp;IF(I11="","origen del agua · ","")&amp;IF(AND(LEFT(I11,7)="Sale de",J11="",K11=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C11:S11)=0,"",IF(AND(C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",H11&lt;&gt;"",I11&lt;&gt;"",NOT(AND(LEFT(I11,7)="Sale de",J11="",K11=""))),"✔ Completa","Falta: "&amp;IF(C11="","fecha · ","")&amp;IF(D11="","ubicación · ","")&amp;IF(E11="","referencia · ","")&amp;IF(H11="","criticidad · ","")&amp;IF(I11="","origen del agua · ","")&amp;IF(AND(LEFT(I11,7)="Sale de",J11="",K11=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C11" s="17" t="n"/>
@@ -1496,8 +1527,9 @@
       <c r="N11" s="21" t="n"/>
       <c r="O11" s="21" t="n"/>
       <c r="P11" s="21" t="n"/>
-      <c r="Q11" s="18" t="n"/>
-      <c r="R11" s="19" t="n"/>
+      <c r="Q11" s="21" t="n"/>
+      <c r="R11" s="18" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
@@ -1506,7 +1538,7 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>IF(COUNTA(C12:R12)=0,"",IF(AND(C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",H12&lt;&gt;"",I12&lt;&gt;"",NOT(AND(LEFT(I12,7)="Sale de",J12="",K12=""))),"✔ Completa","Falta: "&amp;IF(C12="","fecha · ","")&amp;IF(D12="","ubicación · ","")&amp;IF(E12="","referencia · ","")&amp;IF(H12="","criticidad · ","")&amp;IF(I12="","origen del agua · ","")&amp;IF(AND(LEFT(I12,7)="Sale de",J12="",K12=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C12:S12)=0,"",IF(AND(C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",H12&lt;&gt;"",I12&lt;&gt;"",NOT(AND(LEFT(I12,7)="Sale de",J12="",K12=""))),"✔ Completa","Falta: "&amp;IF(C12="","fecha · ","")&amp;IF(D12="","ubicación · ","")&amp;IF(E12="","referencia · ","")&amp;IF(H12="","criticidad · ","")&amp;IF(I12="","origen del agua · ","")&amp;IF(AND(LEFT(I12,7)="Sale de",J12="",K12=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C12" s="17" t="n"/>
@@ -1523,8 +1555,9 @@
       <c r="N12" s="21" t="n"/>
       <c r="O12" s="21" t="n"/>
       <c r="P12" s="21" t="n"/>
-      <c r="Q12" s="18" t="n"/>
-      <c r="R12" s="19" t="n"/>
+      <c r="Q12" s="21" t="n"/>
+      <c r="R12" s="18" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="15" t="inlineStr">
@@ -1533,7 +1566,7 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>IF(COUNTA(C13:R13)=0,"",IF(AND(C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",H13&lt;&gt;"",I13&lt;&gt;"",NOT(AND(LEFT(I13,7)="Sale de",J13="",K13=""))),"✔ Completa","Falta: "&amp;IF(C13="","fecha · ","")&amp;IF(D13="","ubicación · ","")&amp;IF(E13="","referencia · ","")&amp;IF(H13="","criticidad · ","")&amp;IF(I13="","origen del agua · ","")&amp;IF(AND(LEFT(I13,7)="Sale de",J13="",K13=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C13:S13)=0,"",IF(AND(C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",H13&lt;&gt;"",I13&lt;&gt;"",NOT(AND(LEFT(I13,7)="Sale de",J13="",K13=""))),"✔ Completa","Falta: "&amp;IF(C13="","fecha · ","")&amp;IF(D13="","ubicación · ","")&amp;IF(E13="","referencia · ","")&amp;IF(H13="","criticidad · ","")&amp;IF(I13="","origen del agua · ","")&amp;IF(AND(LEFT(I13,7)="Sale de",J13="",K13=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C13" s="17" t="n"/>
@@ -1550,8 +1583,9 @@
       <c r="N13" s="21" t="n"/>
       <c r="O13" s="21" t="n"/>
       <c r="P13" s="21" t="n"/>
-      <c r="Q13" s="18" t="n"/>
-      <c r="R13" s="19" t="n"/>
+      <c r="Q13" s="21" t="n"/>
+      <c r="R13" s="18" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
@@ -1560,7 +1594,7 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>IF(COUNTA(C14:R14)=0,"",IF(AND(C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",H14&lt;&gt;"",I14&lt;&gt;"",NOT(AND(LEFT(I14,7)="Sale de",J14="",K14=""))),"✔ Completa","Falta: "&amp;IF(C14="","fecha · ","")&amp;IF(D14="","ubicación · ","")&amp;IF(E14="","referencia · ","")&amp;IF(H14="","criticidad · ","")&amp;IF(I14="","origen del agua · ","")&amp;IF(AND(LEFT(I14,7)="Sale de",J14="",K14=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C14:S14)=0,"",IF(AND(C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",H14&lt;&gt;"",I14&lt;&gt;"",NOT(AND(LEFT(I14,7)="Sale de",J14="",K14=""))),"✔ Completa","Falta: "&amp;IF(C14="","fecha · ","")&amp;IF(D14="","ubicación · ","")&amp;IF(E14="","referencia · ","")&amp;IF(H14="","criticidad · ","")&amp;IF(I14="","origen del agua · ","")&amp;IF(AND(LEFT(I14,7)="Sale de",J14="",K14=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C14" s="17" t="n"/>
@@ -1577,8 +1611,9 @@
       <c r="N14" s="21" t="n"/>
       <c r="O14" s="21" t="n"/>
       <c r="P14" s="21" t="n"/>
-      <c r="Q14" s="18" t="n"/>
-      <c r="R14" s="19" t="n"/>
+      <c r="Q14" s="21" t="n"/>
+      <c r="R14" s="18" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
@@ -1587,7 +1622,7 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>IF(COUNTA(C15:R15)=0,"",IF(AND(C15&lt;&gt;"",D15&lt;&gt;"",E15&lt;&gt;"",H15&lt;&gt;"",I15&lt;&gt;"",NOT(AND(LEFT(I15,7)="Sale de",J15="",K15=""))),"✔ Completa","Falta: "&amp;IF(C15="","fecha · ","")&amp;IF(D15="","ubicación · ","")&amp;IF(E15="","referencia · ","")&amp;IF(H15="","criticidad · ","")&amp;IF(I15="","origen del agua · ","")&amp;IF(AND(LEFT(I15,7)="Sale de",J15="",K15=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C15:S15)=0,"",IF(AND(C15&lt;&gt;"",D15&lt;&gt;"",E15&lt;&gt;"",H15&lt;&gt;"",I15&lt;&gt;"",NOT(AND(LEFT(I15,7)="Sale de",J15="",K15=""))),"✔ Completa","Falta: "&amp;IF(C15="","fecha · ","")&amp;IF(D15="","ubicación · ","")&amp;IF(E15="","referencia · ","")&amp;IF(H15="","criticidad · ","")&amp;IF(I15="","origen del agua · ","")&amp;IF(AND(LEFT(I15,7)="Sale de",J15="",K15=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C15" s="17" t="n"/>
@@ -1604,8 +1639,9 @@
       <c r="N15" s="21" t="n"/>
       <c r="O15" s="21" t="n"/>
       <c r="P15" s="21" t="n"/>
-      <c r="Q15" s="18" t="n"/>
-      <c r="R15" s="19" t="n"/>
+      <c r="Q15" s="21" t="n"/>
+      <c r="R15" s="18" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
@@ -1614,7 +1650,7 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>IF(COUNTA(C16:R16)=0,"",IF(AND(C16&lt;&gt;"",D16&lt;&gt;"",E16&lt;&gt;"",H16&lt;&gt;"",I16&lt;&gt;"",NOT(AND(LEFT(I16,7)="Sale de",J16="",K16=""))),"✔ Completa","Falta: "&amp;IF(C16="","fecha · ","")&amp;IF(D16="","ubicación · ","")&amp;IF(E16="","referencia · ","")&amp;IF(H16="","criticidad · ","")&amp;IF(I16="","origen del agua · ","")&amp;IF(AND(LEFT(I16,7)="Sale de",J16="",K16=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C16:S16)=0,"",IF(AND(C16&lt;&gt;"",D16&lt;&gt;"",E16&lt;&gt;"",H16&lt;&gt;"",I16&lt;&gt;"",NOT(AND(LEFT(I16,7)="Sale de",J16="",K16=""))),"✔ Completa","Falta: "&amp;IF(C16="","fecha · ","")&amp;IF(D16="","ubicación · ","")&amp;IF(E16="","referencia · ","")&amp;IF(H16="","criticidad · ","")&amp;IF(I16="","origen del agua · ","")&amp;IF(AND(LEFT(I16,7)="Sale de",J16="",K16=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C16" s="17" t="n"/>
@@ -1631,8 +1667,9 @@
       <c r="N16" s="21" t="n"/>
       <c r="O16" s="21" t="n"/>
       <c r="P16" s="21" t="n"/>
-      <c r="Q16" s="18" t="n"/>
-      <c r="R16" s="19" t="n"/>
+      <c r="Q16" s="21" t="n"/>
+      <c r="R16" s="18" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
@@ -1641,7 +1678,7 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>IF(COUNTA(C17:R17)=0,"",IF(AND(C17&lt;&gt;"",D17&lt;&gt;"",E17&lt;&gt;"",H17&lt;&gt;"",I17&lt;&gt;"",NOT(AND(LEFT(I17,7)="Sale de",J17="",K17=""))),"✔ Completa","Falta: "&amp;IF(C17="","fecha · ","")&amp;IF(D17="","ubicación · ","")&amp;IF(E17="","referencia · ","")&amp;IF(H17="","criticidad · ","")&amp;IF(I17="","origen del agua · ","")&amp;IF(AND(LEFT(I17,7)="Sale de",J17="",K17=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C17:S17)=0,"",IF(AND(C17&lt;&gt;"",D17&lt;&gt;"",E17&lt;&gt;"",H17&lt;&gt;"",I17&lt;&gt;"",NOT(AND(LEFT(I17,7)="Sale de",J17="",K17=""))),"✔ Completa","Falta: "&amp;IF(C17="","fecha · ","")&amp;IF(D17="","ubicación · ","")&amp;IF(E17="","referencia · ","")&amp;IF(H17="","criticidad · ","")&amp;IF(I17="","origen del agua · ","")&amp;IF(AND(LEFT(I17,7)="Sale de",J17="",K17=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C17" s="17" t="n"/>
@@ -1658,8 +1695,9 @@
       <c r="N17" s="21" t="n"/>
       <c r="O17" s="21" t="n"/>
       <c r="P17" s="21" t="n"/>
-      <c r="Q17" s="18" t="n"/>
-      <c r="R17" s="19" t="n"/>
+      <c r="Q17" s="21" t="n"/>
+      <c r="R17" s="18" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
@@ -1668,7 +1706,7 @@
         </is>
       </c>
       <c r="B18" s="16">
-        <f>IF(COUNTA(C18:R18)=0,"",IF(AND(C18&lt;&gt;"",D18&lt;&gt;"",E18&lt;&gt;"",H18&lt;&gt;"",I18&lt;&gt;"",NOT(AND(LEFT(I18,7)="Sale de",J18="",K18=""))),"✔ Completa","Falta: "&amp;IF(C18="","fecha · ","")&amp;IF(D18="","ubicación · ","")&amp;IF(E18="","referencia · ","")&amp;IF(H18="","criticidad · ","")&amp;IF(I18="","origen del agua · ","")&amp;IF(AND(LEFT(I18,7)="Sale de",J18="",K18=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C18:S18)=0,"",IF(AND(C18&lt;&gt;"",D18&lt;&gt;"",E18&lt;&gt;"",H18&lt;&gt;"",I18&lt;&gt;"",NOT(AND(LEFT(I18,7)="Sale de",J18="",K18=""))),"✔ Completa","Falta: "&amp;IF(C18="","fecha · ","")&amp;IF(D18="","ubicación · ","")&amp;IF(E18="","referencia · ","")&amp;IF(H18="","criticidad · ","")&amp;IF(I18="","origen del agua · ","")&amp;IF(AND(LEFT(I18,7)="Sale de",J18="",K18=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C18" s="17" t="n"/>
@@ -1685,8 +1723,9 @@
       <c r="N18" s="21" t="n"/>
       <c r="O18" s="21" t="n"/>
       <c r="P18" s="21" t="n"/>
-      <c r="Q18" s="18" t="n"/>
-      <c r="R18" s="19" t="n"/>
+      <c r="Q18" s="21" t="n"/>
+      <c r="R18" s="18" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
@@ -1695,7 +1734,7 @@
         </is>
       </c>
       <c r="B19" s="16">
-        <f>IF(COUNTA(C19:R19)=0,"",IF(AND(C19&lt;&gt;"",D19&lt;&gt;"",E19&lt;&gt;"",H19&lt;&gt;"",I19&lt;&gt;"",NOT(AND(LEFT(I19,7)="Sale de",J19="",K19=""))),"✔ Completa","Falta: "&amp;IF(C19="","fecha · ","")&amp;IF(D19="","ubicación · ","")&amp;IF(E19="","referencia · ","")&amp;IF(H19="","criticidad · ","")&amp;IF(I19="","origen del agua · ","")&amp;IF(AND(LEFT(I19,7)="Sale de",J19="",K19=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C19:S19)=0,"",IF(AND(C19&lt;&gt;"",D19&lt;&gt;"",E19&lt;&gt;"",H19&lt;&gt;"",I19&lt;&gt;"",NOT(AND(LEFT(I19,7)="Sale de",J19="",K19=""))),"✔ Completa","Falta: "&amp;IF(C19="","fecha · ","")&amp;IF(D19="","ubicación · ","")&amp;IF(E19="","referencia · ","")&amp;IF(H19="","criticidad · ","")&amp;IF(I19="","origen del agua · ","")&amp;IF(AND(LEFT(I19,7)="Sale de",J19="",K19=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C19" s="17" t="n"/>
@@ -1712,8 +1751,9 @@
       <c r="N19" s="21" t="n"/>
       <c r="O19" s="21" t="n"/>
       <c r="P19" s="21" t="n"/>
-      <c r="Q19" s="18" t="n"/>
-      <c r="R19" s="19" t="n"/>
+      <c r="Q19" s="21" t="n"/>
+      <c r="R19" s="18" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
@@ -1722,7 +1762,7 @@
         </is>
       </c>
       <c r="B20" s="16">
-        <f>IF(COUNTA(C20:R20)=0,"",IF(AND(C20&lt;&gt;"",D20&lt;&gt;"",E20&lt;&gt;"",H20&lt;&gt;"",I20&lt;&gt;"",NOT(AND(LEFT(I20,7)="Sale de",J20="",K20=""))),"✔ Completa","Falta: "&amp;IF(C20="","fecha · ","")&amp;IF(D20="","ubicación · ","")&amp;IF(E20="","referencia · ","")&amp;IF(H20="","criticidad · ","")&amp;IF(I20="","origen del agua · ","")&amp;IF(AND(LEFT(I20,7)="Sale de",J20="",K20=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C20:S20)=0,"",IF(AND(C20&lt;&gt;"",D20&lt;&gt;"",E20&lt;&gt;"",H20&lt;&gt;"",I20&lt;&gt;"",NOT(AND(LEFT(I20,7)="Sale de",J20="",K20=""))),"✔ Completa","Falta: "&amp;IF(C20="","fecha · ","")&amp;IF(D20="","ubicación · ","")&amp;IF(E20="","referencia · ","")&amp;IF(H20="","criticidad · ","")&amp;IF(I20="","origen del agua · ","")&amp;IF(AND(LEFT(I20,7)="Sale de",J20="",K20=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C20" s="17" t="n"/>
@@ -1739,8 +1779,9 @@
       <c r="N20" s="21" t="n"/>
       <c r="O20" s="21" t="n"/>
       <c r="P20" s="21" t="n"/>
-      <c r="Q20" s="18" t="n"/>
-      <c r="R20" s="19" t="n"/>
+      <c r="Q20" s="21" t="n"/>
+      <c r="R20" s="18" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
@@ -1749,7 +1790,7 @@
         </is>
       </c>
       <c r="B21" s="16">
-        <f>IF(COUNTA(C21:R21)=0,"",IF(AND(C21&lt;&gt;"",D21&lt;&gt;"",E21&lt;&gt;"",H21&lt;&gt;"",I21&lt;&gt;"",NOT(AND(LEFT(I21,7)="Sale de",J21="",K21=""))),"✔ Completa","Falta: "&amp;IF(C21="","fecha · ","")&amp;IF(D21="","ubicación · ","")&amp;IF(E21="","referencia · ","")&amp;IF(H21="","criticidad · ","")&amp;IF(I21="","origen del agua · ","")&amp;IF(AND(LEFT(I21,7)="Sale de",J21="",K21=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C21:S21)=0,"",IF(AND(C21&lt;&gt;"",D21&lt;&gt;"",E21&lt;&gt;"",H21&lt;&gt;"",I21&lt;&gt;"",NOT(AND(LEFT(I21,7)="Sale de",J21="",K21=""))),"✔ Completa","Falta: "&amp;IF(C21="","fecha · ","")&amp;IF(D21="","ubicación · ","")&amp;IF(E21="","referencia · ","")&amp;IF(H21="","criticidad · ","")&amp;IF(I21="","origen del agua · ","")&amp;IF(AND(LEFT(I21,7)="Sale de",J21="",K21=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C21" s="17" t="n"/>
@@ -1766,8 +1807,9 @@
       <c r="N21" s="21" t="n"/>
       <c r="O21" s="21" t="n"/>
       <c r="P21" s="21" t="n"/>
-      <c r="Q21" s="18" t="n"/>
-      <c r="R21" s="19" t="n"/>
+      <c r="Q21" s="21" t="n"/>
+      <c r="R21" s="18" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
@@ -1776,7 +1818,7 @@
         </is>
       </c>
       <c r="B22" s="16">
-        <f>IF(COUNTA(C22:R22)=0,"",IF(AND(C22&lt;&gt;"",D22&lt;&gt;"",E22&lt;&gt;"",H22&lt;&gt;"",I22&lt;&gt;"",NOT(AND(LEFT(I22,7)="Sale de",J22="",K22=""))),"✔ Completa","Falta: "&amp;IF(C22="","fecha · ","")&amp;IF(D22="","ubicación · ","")&amp;IF(E22="","referencia · ","")&amp;IF(H22="","criticidad · ","")&amp;IF(I22="","origen del agua · ","")&amp;IF(AND(LEFT(I22,7)="Sale de",J22="",K22=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C22:S22)=0,"",IF(AND(C22&lt;&gt;"",D22&lt;&gt;"",E22&lt;&gt;"",H22&lt;&gt;"",I22&lt;&gt;"",NOT(AND(LEFT(I22,7)="Sale de",J22="",K22=""))),"✔ Completa","Falta: "&amp;IF(C22="","fecha · ","")&amp;IF(D22="","ubicación · ","")&amp;IF(E22="","referencia · ","")&amp;IF(H22="","criticidad · ","")&amp;IF(I22="","origen del agua · ","")&amp;IF(AND(LEFT(I22,7)="Sale de",J22="",K22=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C22" s="17" t="n"/>
@@ -1793,8 +1835,9 @@
       <c r="N22" s="21" t="n"/>
       <c r="O22" s="21" t="n"/>
       <c r="P22" s="21" t="n"/>
-      <c r="Q22" s="18" t="n"/>
-      <c r="R22" s="19" t="n"/>
+      <c r="Q22" s="21" t="n"/>
+      <c r="R22" s="18" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
@@ -1803,7 +1846,7 @@
         </is>
       </c>
       <c r="B23" s="16">
-        <f>IF(COUNTA(C23:R23)=0,"",IF(AND(C23&lt;&gt;"",D23&lt;&gt;"",E23&lt;&gt;"",H23&lt;&gt;"",I23&lt;&gt;"",NOT(AND(LEFT(I23,7)="Sale de",J23="",K23=""))),"✔ Completa","Falta: "&amp;IF(C23="","fecha · ","")&amp;IF(D23="","ubicación · ","")&amp;IF(E23="","referencia · ","")&amp;IF(H23="","criticidad · ","")&amp;IF(I23="","origen del agua · ","")&amp;IF(AND(LEFT(I23,7)="Sale de",J23="",K23=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C23:S23)=0,"",IF(AND(C23&lt;&gt;"",D23&lt;&gt;"",E23&lt;&gt;"",H23&lt;&gt;"",I23&lt;&gt;"",NOT(AND(LEFT(I23,7)="Sale de",J23="",K23=""))),"✔ Completa","Falta: "&amp;IF(C23="","fecha · ","")&amp;IF(D23="","ubicación · ","")&amp;IF(E23="","referencia · ","")&amp;IF(H23="","criticidad · ","")&amp;IF(I23="","origen del agua · ","")&amp;IF(AND(LEFT(I23,7)="Sale de",J23="",K23=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C23" s="17" t="n"/>
@@ -1820,8 +1863,9 @@
       <c r="N23" s="21" t="n"/>
       <c r="O23" s="21" t="n"/>
       <c r="P23" s="21" t="n"/>
-      <c r="Q23" s="18" t="n"/>
-      <c r="R23" s="19" t="n"/>
+      <c r="Q23" s="21" t="n"/>
+      <c r="R23" s="18" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
@@ -1830,7 +1874,7 @@
         </is>
       </c>
       <c r="B24" s="16">
-        <f>IF(COUNTA(C24:R24)=0,"",IF(AND(C24&lt;&gt;"",D24&lt;&gt;"",E24&lt;&gt;"",H24&lt;&gt;"",I24&lt;&gt;"",NOT(AND(LEFT(I24,7)="Sale de",J24="",K24=""))),"✔ Completa","Falta: "&amp;IF(C24="","fecha · ","")&amp;IF(D24="","ubicación · ","")&amp;IF(E24="","referencia · ","")&amp;IF(H24="","criticidad · ","")&amp;IF(I24="","origen del agua · ","")&amp;IF(AND(LEFT(I24,7)="Sale de",J24="",K24=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C24:S24)=0,"",IF(AND(C24&lt;&gt;"",D24&lt;&gt;"",E24&lt;&gt;"",H24&lt;&gt;"",I24&lt;&gt;"",NOT(AND(LEFT(I24,7)="Sale de",J24="",K24=""))),"✔ Completa","Falta: "&amp;IF(C24="","fecha · ","")&amp;IF(D24="","ubicación · ","")&amp;IF(E24="","referencia · ","")&amp;IF(H24="","criticidad · ","")&amp;IF(I24="","origen del agua · ","")&amp;IF(AND(LEFT(I24,7)="Sale de",J24="",K24=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C24" s="17" t="n"/>
@@ -1847,8 +1891,9 @@
       <c r="N24" s="21" t="n"/>
       <c r="O24" s="21" t="n"/>
       <c r="P24" s="21" t="n"/>
-      <c r="Q24" s="18" t="n"/>
-      <c r="R24" s="19" t="n"/>
+      <c r="Q24" s="21" t="n"/>
+      <c r="R24" s="18" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
@@ -1857,7 +1902,7 @@
         </is>
       </c>
       <c r="B25" s="16">
-        <f>IF(COUNTA(C25:R25)=0,"",IF(AND(C25&lt;&gt;"",D25&lt;&gt;"",E25&lt;&gt;"",H25&lt;&gt;"",I25&lt;&gt;"",NOT(AND(LEFT(I25,7)="Sale de",J25="",K25=""))),"✔ Completa","Falta: "&amp;IF(C25="","fecha · ","")&amp;IF(D25="","ubicación · ","")&amp;IF(E25="","referencia · ","")&amp;IF(H25="","criticidad · ","")&amp;IF(I25="","origen del agua · ","")&amp;IF(AND(LEFT(I25,7)="Sale de",J25="",K25=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C25:S25)=0,"",IF(AND(C25&lt;&gt;"",D25&lt;&gt;"",E25&lt;&gt;"",H25&lt;&gt;"",I25&lt;&gt;"",NOT(AND(LEFT(I25,7)="Sale de",J25="",K25=""))),"✔ Completa","Falta: "&amp;IF(C25="","fecha · ","")&amp;IF(D25="","ubicación · ","")&amp;IF(E25="","referencia · ","")&amp;IF(H25="","criticidad · ","")&amp;IF(I25="","origen del agua · ","")&amp;IF(AND(LEFT(I25,7)="Sale de",J25="",K25=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C25" s="17" t="n"/>
@@ -1874,8 +1919,9 @@
       <c r="N25" s="21" t="n"/>
       <c r="O25" s="21" t="n"/>
       <c r="P25" s="21" t="n"/>
-      <c r="Q25" s="18" t="n"/>
-      <c r="R25" s="19" t="n"/>
+      <c r="Q25" s="21" t="n"/>
+      <c r="R25" s="18" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
@@ -1884,7 +1930,7 @@
         </is>
       </c>
       <c r="B26" s="16">
-        <f>IF(COUNTA(C26:R26)=0,"",IF(AND(C26&lt;&gt;"",D26&lt;&gt;"",E26&lt;&gt;"",H26&lt;&gt;"",I26&lt;&gt;"",NOT(AND(LEFT(I26,7)="Sale de",J26="",K26=""))),"✔ Completa","Falta: "&amp;IF(C26="","fecha · ","")&amp;IF(D26="","ubicación · ","")&amp;IF(E26="","referencia · ","")&amp;IF(H26="","criticidad · ","")&amp;IF(I26="","origen del agua · ","")&amp;IF(AND(LEFT(I26,7)="Sale de",J26="",K26=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C26:S26)=0,"",IF(AND(C26&lt;&gt;"",D26&lt;&gt;"",E26&lt;&gt;"",H26&lt;&gt;"",I26&lt;&gt;"",NOT(AND(LEFT(I26,7)="Sale de",J26="",K26=""))),"✔ Completa","Falta: "&amp;IF(C26="","fecha · ","")&amp;IF(D26="","ubicación · ","")&amp;IF(E26="","referencia · ","")&amp;IF(H26="","criticidad · ","")&amp;IF(I26="","origen del agua · ","")&amp;IF(AND(LEFT(I26,7)="Sale de",J26="",K26=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C26" s="17" t="n"/>
@@ -1901,8 +1947,9 @@
       <c r="N26" s="21" t="n"/>
       <c r="O26" s="21" t="n"/>
       <c r="P26" s="21" t="n"/>
-      <c r="Q26" s="18" t="n"/>
-      <c r="R26" s="19" t="n"/>
+      <c r="Q26" s="21" t="n"/>
+      <c r="R26" s="18" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
@@ -1911,7 +1958,7 @@
         </is>
       </c>
       <c r="B27" s="16">
-        <f>IF(COUNTA(C27:R27)=0,"",IF(AND(C27&lt;&gt;"",D27&lt;&gt;"",E27&lt;&gt;"",H27&lt;&gt;"",I27&lt;&gt;"",NOT(AND(LEFT(I27,7)="Sale de",J27="",K27=""))),"✔ Completa","Falta: "&amp;IF(C27="","fecha · ","")&amp;IF(D27="","ubicación · ","")&amp;IF(E27="","referencia · ","")&amp;IF(H27="","criticidad · ","")&amp;IF(I27="","origen del agua · ","")&amp;IF(AND(LEFT(I27,7)="Sale de",J27="",K27=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C27:S27)=0,"",IF(AND(C27&lt;&gt;"",D27&lt;&gt;"",E27&lt;&gt;"",H27&lt;&gt;"",I27&lt;&gt;"",NOT(AND(LEFT(I27,7)="Sale de",J27="",K27=""))),"✔ Completa","Falta: "&amp;IF(C27="","fecha · ","")&amp;IF(D27="","ubicación · ","")&amp;IF(E27="","referencia · ","")&amp;IF(H27="","criticidad · ","")&amp;IF(I27="","origen del agua · ","")&amp;IF(AND(LEFT(I27,7)="Sale de",J27="",K27=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C27" s="17" t="n"/>
@@ -1928,8 +1975,9 @@
       <c r="N27" s="21" t="n"/>
       <c r="O27" s="21" t="n"/>
       <c r="P27" s="21" t="n"/>
-      <c r="Q27" s="18" t="n"/>
-      <c r="R27" s="19" t="n"/>
+      <c r="Q27" s="21" t="n"/>
+      <c r="R27" s="18" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
@@ -1938,7 +1986,7 @@
         </is>
       </c>
       <c r="B28" s="16">
-        <f>IF(COUNTA(C28:R28)=0,"",IF(AND(C28&lt;&gt;"",D28&lt;&gt;"",E28&lt;&gt;"",H28&lt;&gt;"",I28&lt;&gt;"",NOT(AND(LEFT(I28,7)="Sale de",J28="",K28=""))),"✔ Completa","Falta: "&amp;IF(C28="","fecha · ","")&amp;IF(D28="","ubicación · ","")&amp;IF(E28="","referencia · ","")&amp;IF(H28="","criticidad · ","")&amp;IF(I28="","origen del agua · ","")&amp;IF(AND(LEFT(I28,7)="Sale de",J28="",K28=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C28:S28)=0,"",IF(AND(C28&lt;&gt;"",D28&lt;&gt;"",E28&lt;&gt;"",H28&lt;&gt;"",I28&lt;&gt;"",NOT(AND(LEFT(I28,7)="Sale de",J28="",K28=""))),"✔ Completa","Falta: "&amp;IF(C28="","fecha · ","")&amp;IF(D28="","ubicación · ","")&amp;IF(E28="","referencia · ","")&amp;IF(H28="","criticidad · ","")&amp;IF(I28="","origen del agua · ","")&amp;IF(AND(LEFT(I28,7)="Sale de",J28="",K28=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C28" s="17" t="n"/>
@@ -1955,8 +2003,9 @@
       <c r="N28" s="21" t="n"/>
       <c r="O28" s="21" t="n"/>
       <c r="P28" s="21" t="n"/>
-      <c r="Q28" s="18" t="n"/>
-      <c r="R28" s="19" t="n"/>
+      <c r="Q28" s="21" t="n"/>
+      <c r="R28" s="18" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
@@ -1965,7 +2014,7 @@
         </is>
       </c>
       <c r="B29" s="16">
-        <f>IF(COUNTA(C29:R29)=0,"",IF(AND(C29&lt;&gt;"",D29&lt;&gt;"",E29&lt;&gt;"",H29&lt;&gt;"",I29&lt;&gt;"",NOT(AND(LEFT(I29,7)="Sale de",J29="",K29=""))),"✔ Completa","Falta: "&amp;IF(C29="","fecha · ","")&amp;IF(D29="","ubicación · ","")&amp;IF(E29="","referencia · ","")&amp;IF(H29="","criticidad · ","")&amp;IF(I29="","origen del agua · ","")&amp;IF(AND(LEFT(I29,7)="Sale de",J29="",K29=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C29:S29)=0,"",IF(AND(C29&lt;&gt;"",D29&lt;&gt;"",E29&lt;&gt;"",H29&lt;&gt;"",I29&lt;&gt;"",NOT(AND(LEFT(I29,7)="Sale de",J29="",K29=""))),"✔ Completa","Falta: "&amp;IF(C29="","fecha · ","")&amp;IF(D29="","ubicación · ","")&amp;IF(E29="","referencia · ","")&amp;IF(H29="","criticidad · ","")&amp;IF(I29="","origen del agua · ","")&amp;IF(AND(LEFT(I29,7)="Sale de",J29="",K29=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C29" s="17" t="n"/>
@@ -1982,8 +2031,9 @@
       <c r="N29" s="21" t="n"/>
       <c r="O29" s="21" t="n"/>
       <c r="P29" s="21" t="n"/>
-      <c r="Q29" s="18" t="n"/>
-      <c r="R29" s="19" t="n"/>
+      <c r="Q29" s="21" t="n"/>
+      <c r="R29" s="18" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
@@ -1992,7 +2042,7 @@
         </is>
       </c>
       <c r="B30" s="16">
-        <f>IF(COUNTA(C30:R30)=0,"",IF(AND(C30&lt;&gt;"",D30&lt;&gt;"",E30&lt;&gt;"",H30&lt;&gt;"",I30&lt;&gt;"",NOT(AND(LEFT(I30,7)="Sale de",J30="",K30=""))),"✔ Completa","Falta: "&amp;IF(C30="","fecha · ","")&amp;IF(D30="","ubicación · ","")&amp;IF(E30="","referencia · ","")&amp;IF(H30="","criticidad · ","")&amp;IF(I30="","origen del agua · ","")&amp;IF(AND(LEFT(I30,7)="Sale de",J30="",K30=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C30:S30)=0,"",IF(AND(C30&lt;&gt;"",D30&lt;&gt;"",E30&lt;&gt;"",H30&lt;&gt;"",I30&lt;&gt;"",NOT(AND(LEFT(I30,7)="Sale de",J30="",K30=""))),"✔ Completa","Falta: "&amp;IF(C30="","fecha · ","")&amp;IF(D30="","ubicación · ","")&amp;IF(E30="","referencia · ","")&amp;IF(H30="","criticidad · ","")&amp;IF(I30="","origen del agua · ","")&amp;IF(AND(LEFT(I30,7)="Sale de",J30="",K30=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C30" s="17" t="n"/>
@@ -2009,8 +2059,9 @@
       <c r="N30" s="21" t="n"/>
       <c r="O30" s="21" t="n"/>
       <c r="P30" s="21" t="n"/>
-      <c r="Q30" s="18" t="n"/>
-      <c r="R30" s="19" t="n"/>
+      <c r="Q30" s="21" t="n"/>
+      <c r="R30" s="18" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
@@ -2019,7 +2070,7 @@
         </is>
       </c>
       <c r="B31" s="16">
-        <f>IF(COUNTA(C31:R31)=0,"",IF(AND(C31&lt;&gt;"",D31&lt;&gt;"",E31&lt;&gt;"",H31&lt;&gt;"",I31&lt;&gt;"",NOT(AND(LEFT(I31,7)="Sale de",J31="",K31=""))),"✔ Completa","Falta: "&amp;IF(C31="","fecha · ","")&amp;IF(D31="","ubicación · ","")&amp;IF(E31="","referencia · ","")&amp;IF(H31="","criticidad · ","")&amp;IF(I31="","origen del agua · ","")&amp;IF(AND(LEFT(I31,7)="Sale de",J31="",K31=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C31:S31)=0,"",IF(AND(C31&lt;&gt;"",D31&lt;&gt;"",E31&lt;&gt;"",H31&lt;&gt;"",I31&lt;&gt;"",NOT(AND(LEFT(I31,7)="Sale de",J31="",K31=""))),"✔ Completa","Falta: "&amp;IF(C31="","fecha · ","")&amp;IF(D31="","ubicación · ","")&amp;IF(E31="","referencia · ","")&amp;IF(H31="","criticidad · ","")&amp;IF(I31="","origen del agua · ","")&amp;IF(AND(LEFT(I31,7)="Sale de",J31="",K31=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C31" s="17" t="n"/>
@@ -2036,8 +2087,9 @@
       <c r="N31" s="21" t="n"/>
       <c r="O31" s="21" t="n"/>
       <c r="P31" s="21" t="n"/>
-      <c r="Q31" s="18" t="n"/>
-      <c r="R31" s="19" t="n"/>
+      <c r="Q31" s="21" t="n"/>
+      <c r="R31" s="18" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
@@ -2046,7 +2098,7 @@
         </is>
       </c>
       <c r="B32" s="16">
-        <f>IF(COUNTA(C32:R32)=0,"",IF(AND(C32&lt;&gt;"",D32&lt;&gt;"",E32&lt;&gt;"",H32&lt;&gt;"",I32&lt;&gt;"",NOT(AND(LEFT(I32,7)="Sale de",J32="",K32=""))),"✔ Completa","Falta: "&amp;IF(C32="","fecha · ","")&amp;IF(D32="","ubicación · ","")&amp;IF(E32="","referencia · ","")&amp;IF(H32="","criticidad · ","")&amp;IF(I32="","origen del agua · ","")&amp;IF(AND(LEFT(I32,7)="Sale de",J32="",K32=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C32:S32)=0,"",IF(AND(C32&lt;&gt;"",D32&lt;&gt;"",E32&lt;&gt;"",H32&lt;&gt;"",I32&lt;&gt;"",NOT(AND(LEFT(I32,7)="Sale de",J32="",K32=""))),"✔ Completa","Falta: "&amp;IF(C32="","fecha · ","")&amp;IF(D32="","ubicación · ","")&amp;IF(E32="","referencia · ","")&amp;IF(H32="","criticidad · ","")&amp;IF(I32="","origen del agua · ","")&amp;IF(AND(LEFT(I32,7)="Sale de",J32="",K32=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C32" s="17" t="n"/>
@@ -2063,8 +2115,9 @@
       <c r="N32" s="21" t="n"/>
       <c r="O32" s="21" t="n"/>
       <c r="P32" s="21" t="n"/>
-      <c r="Q32" s="18" t="n"/>
-      <c r="R32" s="19" t="n"/>
+      <c r="Q32" s="21" t="n"/>
+      <c r="R32" s="18" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
@@ -2073,7 +2126,7 @@
         </is>
       </c>
       <c r="B33" s="16">
-        <f>IF(COUNTA(C33:R33)=0,"",IF(AND(C33&lt;&gt;"",D33&lt;&gt;"",E33&lt;&gt;"",H33&lt;&gt;"",I33&lt;&gt;"",NOT(AND(LEFT(I33,7)="Sale de",J33="",K33=""))),"✔ Completa","Falta: "&amp;IF(C33="","fecha · ","")&amp;IF(D33="","ubicación · ","")&amp;IF(E33="","referencia · ","")&amp;IF(H33="","criticidad · ","")&amp;IF(I33="","origen del agua · ","")&amp;IF(AND(LEFT(I33,7)="Sale de",J33="",K33=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C33:S33)=0,"",IF(AND(C33&lt;&gt;"",D33&lt;&gt;"",E33&lt;&gt;"",H33&lt;&gt;"",I33&lt;&gt;"",NOT(AND(LEFT(I33,7)="Sale de",J33="",K33=""))),"✔ Completa","Falta: "&amp;IF(C33="","fecha · ","")&amp;IF(D33="","ubicación · ","")&amp;IF(E33="","referencia · ","")&amp;IF(H33="","criticidad · ","")&amp;IF(I33="","origen del agua · ","")&amp;IF(AND(LEFT(I33,7)="Sale de",J33="",K33=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C33" s="17" t="n"/>
@@ -2090,8 +2143,9 @@
       <c r="N33" s="21" t="n"/>
       <c r="O33" s="21" t="n"/>
       <c r="P33" s="21" t="n"/>
-      <c r="Q33" s="18" t="n"/>
-      <c r="R33" s="19" t="n"/>
+      <c r="Q33" s="21" t="n"/>
+      <c r="R33" s="18" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="15" t="inlineStr">
@@ -2100,7 +2154,7 @@
         </is>
       </c>
       <c r="B34" s="16">
-        <f>IF(COUNTA(C34:R34)=0,"",IF(AND(C34&lt;&gt;"",D34&lt;&gt;"",E34&lt;&gt;"",H34&lt;&gt;"",I34&lt;&gt;"",NOT(AND(LEFT(I34,7)="Sale de",J34="",K34=""))),"✔ Completa","Falta: "&amp;IF(C34="","fecha · ","")&amp;IF(D34="","ubicación · ","")&amp;IF(E34="","referencia · ","")&amp;IF(H34="","criticidad · ","")&amp;IF(I34="","origen del agua · ","")&amp;IF(AND(LEFT(I34,7)="Sale de",J34="",K34=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C34:S34)=0,"",IF(AND(C34&lt;&gt;"",D34&lt;&gt;"",E34&lt;&gt;"",H34&lt;&gt;"",I34&lt;&gt;"",NOT(AND(LEFT(I34,7)="Sale de",J34="",K34=""))),"✔ Completa","Falta: "&amp;IF(C34="","fecha · ","")&amp;IF(D34="","ubicación · ","")&amp;IF(E34="","referencia · ","")&amp;IF(H34="","criticidad · ","")&amp;IF(I34="","origen del agua · ","")&amp;IF(AND(LEFT(I34,7)="Sale de",J34="",K34=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C34" s="17" t="n"/>
@@ -2117,8 +2171,9 @@
       <c r="N34" s="21" t="n"/>
       <c r="O34" s="21" t="n"/>
       <c r="P34" s="21" t="n"/>
-      <c r="Q34" s="18" t="n"/>
-      <c r="R34" s="19" t="n"/>
+      <c r="Q34" s="21" t="n"/>
+      <c r="R34" s="18" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
@@ -2127,7 +2182,7 @@
         </is>
       </c>
       <c r="B35" s="16">
-        <f>IF(COUNTA(C35:R35)=0,"",IF(AND(C35&lt;&gt;"",D35&lt;&gt;"",E35&lt;&gt;"",H35&lt;&gt;"",I35&lt;&gt;"",NOT(AND(LEFT(I35,7)="Sale de",J35="",K35=""))),"✔ Completa","Falta: "&amp;IF(C35="","fecha · ","")&amp;IF(D35="","ubicación · ","")&amp;IF(E35="","referencia · ","")&amp;IF(H35="","criticidad · ","")&amp;IF(I35="","origen del agua · ","")&amp;IF(AND(LEFT(I35,7)="Sale de",J35="",K35=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C35:S35)=0,"",IF(AND(C35&lt;&gt;"",D35&lt;&gt;"",E35&lt;&gt;"",H35&lt;&gt;"",I35&lt;&gt;"",NOT(AND(LEFT(I35,7)="Sale de",J35="",K35=""))),"✔ Completa","Falta: "&amp;IF(C35="","fecha · ","")&amp;IF(D35="","ubicación · ","")&amp;IF(E35="","referencia · ","")&amp;IF(H35="","criticidad · ","")&amp;IF(I35="","origen del agua · ","")&amp;IF(AND(LEFT(I35,7)="Sale de",J35="",K35=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C35" s="17" t="n"/>
@@ -2144,8 +2199,9 @@
       <c r="N35" s="21" t="n"/>
       <c r="O35" s="21" t="n"/>
       <c r="P35" s="21" t="n"/>
-      <c r="Q35" s="18" t="n"/>
-      <c r="R35" s="19" t="n"/>
+      <c r="Q35" s="21" t="n"/>
+      <c r="R35" s="18" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="15" t="inlineStr">
@@ -2154,7 +2210,7 @@
         </is>
       </c>
       <c r="B36" s="16">
-        <f>IF(COUNTA(C36:R36)=0,"",IF(AND(C36&lt;&gt;"",D36&lt;&gt;"",E36&lt;&gt;"",H36&lt;&gt;"",I36&lt;&gt;"",NOT(AND(LEFT(I36,7)="Sale de",J36="",K36=""))),"✔ Completa","Falta: "&amp;IF(C36="","fecha · ","")&amp;IF(D36="","ubicación · ","")&amp;IF(E36="","referencia · ","")&amp;IF(H36="","criticidad · ","")&amp;IF(I36="","origen del agua · ","")&amp;IF(AND(LEFT(I36,7)="Sale de",J36="",K36=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C36:S36)=0,"",IF(AND(C36&lt;&gt;"",D36&lt;&gt;"",E36&lt;&gt;"",H36&lt;&gt;"",I36&lt;&gt;"",NOT(AND(LEFT(I36,7)="Sale de",J36="",K36=""))),"✔ Completa","Falta: "&amp;IF(C36="","fecha · ","")&amp;IF(D36="","ubicación · ","")&amp;IF(E36="","referencia · ","")&amp;IF(H36="","criticidad · ","")&amp;IF(I36="","origen del agua · ","")&amp;IF(AND(LEFT(I36,7)="Sale de",J36="",K36=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C36" s="17" t="n"/>
@@ -2171,8 +2227,9 @@
       <c r="N36" s="21" t="n"/>
       <c r="O36" s="21" t="n"/>
       <c r="P36" s="21" t="n"/>
-      <c r="Q36" s="18" t="n"/>
-      <c r="R36" s="19" t="n"/>
+      <c r="Q36" s="21" t="n"/>
+      <c r="R36" s="18" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="15" t="inlineStr">
@@ -2181,7 +2238,7 @@
         </is>
       </c>
       <c r="B37" s="16">
-        <f>IF(COUNTA(C37:R37)=0,"",IF(AND(C37&lt;&gt;"",D37&lt;&gt;"",E37&lt;&gt;"",H37&lt;&gt;"",I37&lt;&gt;"",NOT(AND(LEFT(I37,7)="Sale de",J37="",K37=""))),"✔ Completa","Falta: "&amp;IF(C37="","fecha · ","")&amp;IF(D37="","ubicación · ","")&amp;IF(E37="","referencia · ","")&amp;IF(H37="","criticidad · ","")&amp;IF(I37="","origen del agua · ","")&amp;IF(AND(LEFT(I37,7)="Sale de",J37="",K37=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C37:S37)=0,"",IF(AND(C37&lt;&gt;"",D37&lt;&gt;"",E37&lt;&gt;"",H37&lt;&gt;"",I37&lt;&gt;"",NOT(AND(LEFT(I37,7)="Sale de",J37="",K37=""))),"✔ Completa","Falta: "&amp;IF(C37="","fecha · ","")&amp;IF(D37="","ubicación · ","")&amp;IF(E37="","referencia · ","")&amp;IF(H37="","criticidad · ","")&amp;IF(I37="","origen del agua · ","")&amp;IF(AND(LEFT(I37,7)="Sale de",J37="",K37=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C37" s="17" t="n"/>
@@ -2198,8 +2255,9 @@
       <c r="N37" s="21" t="n"/>
       <c r="O37" s="21" t="n"/>
       <c r="P37" s="21" t="n"/>
-      <c r="Q37" s="18" t="n"/>
-      <c r="R37" s="19" t="n"/>
+      <c r="Q37" s="21" t="n"/>
+      <c r="R37" s="18" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="15" t="inlineStr">
@@ -2208,7 +2266,7 @@
         </is>
       </c>
       <c r="B38" s="16">
-        <f>IF(COUNTA(C38:R38)=0,"",IF(AND(C38&lt;&gt;"",D38&lt;&gt;"",E38&lt;&gt;"",H38&lt;&gt;"",I38&lt;&gt;"",NOT(AND(LEFT(I38,7)="Sale de",J38="",K38=""))),"✔ Completa","Falta: "&amp;IF(C38="","fecha · ","")&amp;IF(D38="","ubicación · ","")&amp;IF(E38="","referencia · ","")&amp;IF(H38="","criticidad · ","")&amp;IF(I38="","origen del agua · ","")&amp;IF(AND(LEFT(I38,7)="Sale de",J38="",K38=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C38:S38)=0,"",IF(AND(C38&lt;&gt;"",D38&lt;&gt;"",E38&lt;&gt;"",H38&lt;&gt;"",I38&lt;&gt;"",NOT(AND(LEFT(I38,7)="Sale de",J38="",K38=""))),"✔ Completa","Falta: "&amp;IF(C38="","fecha · ","")&amp;IF(D38="","ubicación · ","")&amp;IF(E38="","referencia · ","")&amp;IF(H38="","criticidad · ","")&amp;IF(I38="","origen del agua · ","")&amp;IF(AND(LEFT(I38,7)="Sale de",J38="",K38=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C38" s="17" t="n"/>
@@ -2225,8 +2283,9 @@
       <c r="N38" s="21" t="n"/>
       <c r="O38" s="21" t="n"/>
       <c r="P38" s="21" t="n"/>
-      <c r="Q38" s="18" t="n"/>
-      <c r="R38" s="19" t="n"/>
+      <c r="Q38" s="21" t="n"/>
+      <c r="R38" s="18" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="15" t="inlineStr">
@@ -2235,7 +2294,7 @@
         </is>
       </c>
       <c r="B39" s="16">
-        <f>IF(COUNTA(C39:R39)=0,"",IF(AND(C39&lt;&gt;"",D39&lt;&gt;"",E39&lt;&gt;"",H39&lt;&gt;"",I39&lt;&gt;"",NOT(AND(LEFT(I39,7)="Sale de",J39="",K39=""))),"✔ Completa","Falta: "&amp;IF(C39="","fecha · ","")&amp;IF(D39="","ubicación · ","")&amp;IF(E39="","referencia · ","")&amp;IF(H39="","criticidad · ","")&amp;IF(I39="","origen del agua · ","")&amp;IF(AND(LEFT(I39,7)="Sale de",J39="",K39=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C39:S39)=0,"",IF(AND(C39&lt;&gt;"",D39&lt;&gt;"",E39&lt;&gt;"",H39&lt;&gt;"",I39&lt;&gt;"",NOT(AND(LEFT(I39,7)="Sale de",J39="",K39=""))),"✔ Completa","Falta: "&amp;IF(C39="","fecha · ","")&amp;IF(D39="","ubicación · ","")&amp;IF(E39="","referencia · ","")&amp;IF(H39="","criticidad · ","")&amp;IF(I39="","origen del agua · ","")&amp;IF(AND(LEFT(I39,7)="Sale de",J39="",K39=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C39" s="17" t="n"/>
@@ -2252,8 +2311,9 @@
       <c r="N39" s="21" t="n"/>
       <c r="O39" s="21" t="n"/>
       <c r="P39" s="21" t="n"/>
-      <c r="Q39" s="18" t="n"/>
-      <c r="R39" s="19" t="n"/>
+      <c r="Q39" s="21" t="n"/>
+      <c r="R39" s="18" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="15" t="inlineStr">
@@ -2262,7 +2322,7 @@
         </is>
       </c>
       <c r="B40" s="16">
-        <f>IF(COUNTA(C40:R40)=0,"",IF(AND(C40&lt;&gt;"",D40&lt;&gt;"",E40&lt;&gt;"",H40&lt;&gt;"",I40&lt;&gt;"",NOT(AND(LEFT(I40,7)="Sale de",J40="",K40=""))),"✔ Completa","Falta: "&amp;IF(C40="","fecha · ","")&amp;IF(D40="","ubicación · ","")&amp;IF(E40="","referencia · ","")&amp;IF(H40="","criticidad · ","")&amp;IF(I40="","origen del agua · ","")&amp;IF(AND(LEFT(I40,7)="Sale de",J40="",K40=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C40:S40)=0,"",IF(AND(C40&lt;&gt;"",D40&lt;&gt;"",E40&lt;&gt;"",H40&lt;&gt;"",I40&lt;&gt;"",NOT(AND(LEFT(I40,7)="Sale de",J40="",K40=""))),"✔ Completa","Falta: "&amp;IF(C40="","fecha · ","")&amp;IF(D40="","ubicación · ","")&amp;IF(E40="","referencia · ","")&amp;IF(H40="","criticidad · ","")&amp;IF(I40="","origen del agua · ","")&amp;IF(AND(LEFT(I40,7)="Sale de",J40="",K40=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C40" s="17" t="n"/>
@@ -2279,8 +2339,9 @@
       <c r="N40" s="21" t="n"/>
       <c r="O40" s="21" t="n"/>
       <c r="P40" s="21" t="n"/>
-      <c r="Q40" s="18" t="n"/>
-      <c r="R40" s="19" t="n"/>
+      <c r="Q40" s="21" t="n"/>
+      <c r="R40" s="18" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="15" t="inlineStr">
@@ -2289,7 +2350,7 @@
         </is>
       </c>
       <c r="B41" s="16">
-        <f>IF(COUNTA(C41:R41)=0,"",IF(AND(C41&lt;&gt;"",D41&lt;&gt;"",E41&lt;&gt;"",H41&lt;&gt;"",I41&lt;&gt;"",NOT(AND(LEFT(I41,7)="Sale de",J41="",K41=""))),"✔ Completa","Falta: "&amp;IF(C41="","fecha · ","")&amp;IF(D41="","ubicación · ","")&amp;IF(E41="","referencia · ","")&amp;IF(H41="","criticidad · ","")&amp;IF(I41="","origen del agua · ","")&amp;IF(AND(LEFT(I41,7)="Sale de",J41="",K41=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C41:S41)=0,"",IF(AND(C41&lt;&gt;"",D41&lt;&gt;"",E41&lt;&gt;"",H41&lt;&gt;"",I41&lt;&gt;"",NOT(AND(LEFT(I41,7)="Sale de",J41="",K41=""))),"✔ Completa","Falta: "&amp;IF(C41="","fecha · ","")&amp;IF(D41="","ubicación · ","")&amp;IF(E41="","referencia · ","")&amp;IF(H41="","criticidad · ","")&amp;IF(I41="","origen del agua · ","")&amp;IF(AND(LEFT(I41,7)="Sale de",J41="",K41=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C41" s="17" t="n"/>
@@ -2306,8 +2367,9 @@
       <c r="N41" s="21" t="n"/>
       <c r="O41" s="21" t="n"/>
       <c r="P41" s="21" t="n"/>
-      <c r="Q41" s="18" t="n"/>
-      <c r="R41" s="19" t="n"/>
+      <c r="Q41" s="21" t="n"/>
+      <c r="R41" s="18" t="n"/>
+      <c r="S41" s="19" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="15" t="inlineStr">
@@ -2316,7 +2378,7 @@
         </is>
       </c>
       <c r="B42" s="16">
-        <f>IF(COUNTA(C42:R42)=0,"",IF(AND(C42&lt;&gt;"",D42&lt;&gt;"",E42&lt;&gt;"",H42&lt;&gt;"",I42&lt;&gt;"",NOT(AND(LEFT(I42,7)="Sale de",J42="",K42=""))),"✔ Completa","Falta: "&amp;IF(C42="","fecha · ","")&amp;IF(D42="","ubicación · ","")&amp;IF(E42="","referencia · ","")&amp;IF(H42="","criticidad · ","")&amp;IF(I42="","origen del agua · ","")&amp;IF(AND(LEFT(I42,7)="Sale de",J42="",K42=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C42:S42)=0,"",IF(AND(C42&lt;&gt;"",D42&lt;&gt;"",E42&lt;&gt;"",H42&lt;&gt;"",I42&lt;&gt;"",NOT(AND(LEFT(I42,7)="Sale de",J42="",K42=""))),"✔ Completa","Falta: "&amp;IF(C42="","fecha · ","")&amp;IF(D42="","ubicación · ","")&amp;IF(E42="","referencia · ","")&amp;IF(H42="","criticidad · ","")&amp;IF(I42="","origen del agua · ","")&amp;IF(AND(LEFT(I42,7)="Sale de",J42="",K42=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C42" s="17" t="n"/>
@@ -2333,8 +2395,9 @@
       <c r="N42" s="21" t="n"/>
       <c r="O42" s="21" t="n"/>
       <c r="P42" s="21" t="n"/>
-      <c r="Q42" s="18" t="n"/>
-      <c r="R42" s="19" t="n"/>
+      <c r="Q42" s="21" t="n"/>
+      <c r="R42" s="18" t="n"/>
+      <c r="S42" s="19" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="15" t="inlineStr">
@@ -2343,7 +2406,7 @@
         </is>
       </c>
       <c r="B43" s="16">
-        <f>IF(COUNTA(C43:R43)=0,"",IF(AND(C43&lt;&gt;"",D43&lt;&gt;"",E43&lt;&gt;"",H43&lt;&gt;"",I43&lt;&gt;"",NOT(AND(LEFT(I43,7)="Sale de",J43="",K43=""))),"✔ Completa","Falta: "&amp;IF(C43="","fecha · ","")&amp;IF(D43="","ubicación · ","")&amp;IF(E43="","referencia · ","")&amp;IF(H43="","criticidad · ","")&amp;IF(I43="","origen del agua · ","")&amp;IF(AND(LEFT(I43,7)="Sale de",J43="",K43=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C43:S43)=0,"",IF(AND(C43&lt;&gt;"",D43&lt;&gt;"",E43&lt;&gt;"",H43&lt;&gt;"",I43&lt;&gt;"",NOT(AND(LEFT(I43,7)="Sale de",J43="",K43=""))),"✔ Completa","Falta: "&amp;IF(C43="","fecha · ","")&amp;IF(D43="","ubicación · ","")&amp;IF(E43="","referencia · ","")&amp;IF(H43="","criticidad · ","")&amp;IF(I43="","origen del agua · ","")&amp;IF(AND(LEFT(I43,7)="Sale de",J43="",K43=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C43" s="17" t="n"/>
@@ -2360,8 +2423,9 @@
       <c r="N43" s="21" t="n"/>
       <c r="O43" s="21" t="n"/>
       <c r="P43" s="21" t="n"/>
-      <c r="Q43" s="18" t="n"/>
-      <c r="R43" s="19" t="n"/>
+      <c r="Q43" s="21" t="n"/>
+      <c r="R43" s="18" t="n"/>
+      <c r="S43" s="19" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="15" t="inlineStr">
@@ -2370,7 +2434,7 @@
         </is>
       </c>
       <c r="B44" s="16">
-        <f>IF(COUNTA(C44:R44)=0,"",IF(AND(C44&lt;&gt;"",D44&lt;&gt;"",E44&lt;&gt;"",H44&lt;&gt;"",I44&lt;&gt;"",NOT(AND(LEFT(I44,7)="Sale de",J44="",K44=""))),"✔ Completa","Falta: "&amp;IF(C44="","fecha · ","")&amp;IF(D44="","ubicación · ","")&amp;IF(E44="","referencia · ","")&amp;IF(H44="","criticidad · ","")&amp;IF(I44="","origen del agua · ","")&amp;IF(AND(LEFT(I44,7)="Sale de",J44="",K44=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C44:S44)=0,"",IF(AND(C44&lt;&gt;"",D44&lt;&gt;"",E44&lt;&gt;"",H44&lt;&gt;"",I44&lt;&gt;"",NOT(AND(LEFT(I44,7)="Sale de",J44="",K44=""))),"✔ Completa","Falta: "&amp;IF(C44="","fecha · ","")&amp;IF(D44="","ubicación · ","")&amp;IF(E44="","referencia · ","")&amp;IF(H44="","criticidad · ","")&amp;IF(I44="","origen del agua · ","")&amp;IF(AND(LEFT(I44,7)="Sale de",J44="",K44=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C44" s="17" t="n"/>
@@ -2387,8 +2451,9 @@
       <c r="N44" s="21" t="n"/>
       <c r="O44" s="21" t="n"/>
       <c r="P44" s="21" t="n"/>
-      <c r="Q44" s="18" t="n"/>
-      <c r="R44" s="19" t="n"/>
+      <c r="Q44" s="21" t="n"/>
+      <c r="R44" s="18" t="n"/>
+      <c r="S44" s="19" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="15" t="inlineStr">
@@ -2397,7 +2462,7 @@
         </is>
       </c>
       <c r="B45" s="16">
-        <f>IF(COUNTA(C45:R45)=0,"",IF(AND(C45&lt;&gt;"",D45&lt;&gt;"",E45&lt;&gt;"",H45&lt;&gt;"",I45&lt;&gt;"",NOT(AND(LEFT(I45,7)="Sale de",J45="",K45=""))),"✔ Completa","Falta: "&amp;IF(C45="","fecha · ","")&amp;IF(D45="","ubicación · ","")&amp;IF(E45="","referencia · ","")&amp;IF(H45="","criticidad · ","")&amp;IF(I45="","origen del agua · ","")&amp;IF(AND(LEFT(I45,7)="Sale de",J45="",K45=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C45:S45)=0,"",IF(AND(C45&lt;&gt;"",D45&lt;&gt;"",E45&lt;&gt;"",H45&lt;&gt;"",I45&lt;&gt;"",NOT(AND(LEFT(I45,7)="Sale de",J45="",K45=""))),"✔ Completa","Falta: "&amp;IF(C45="","fecha · ","")&amp;IF(D45="","ubicación · ","")&amp;IF(E45="","referencia · ","")&amp;IF(H45="","criticidad · ","")&amp;IF(I45="","origen del agua · ","")&amp;IF(AND(LEFT(I45,7)="Sale de",J45="",K45=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C45" s="17" t="n"/>
@@ -2414,8 +2479,9 @@
       <c r="N45" s="21" t="n"/>
       <c r="O45" s="21" t="n"/>
       <c r="P45" s="21" t="n"/>
-      <c r="Q45" s="18" t="n"/>
-      <c r="R45" s="19" t="n"/>
+      <c r="Q45" s="21" t="n"/>
+      <c r="R45" s="18" t="n"/>
+      <c r="S45" s="19" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="15" t="inlineStr">
@@ -2424,7 +2490,7 @@
         </is>
       </c>
       <c r="B46" s="16">
-        <f>IF(COUNTA(C46:R46)=0,"",IF(AND(C46&lt;&gt;"",D46&lt;&gt;"",E46&lt;&gt;"",H46&lt;&gt;"",I46&lt;&gt;"",NOT(AND(LEFT(I46,7)="Sale de",J46="",K46=""))),"✔ Completa","Falta: "&amp;IF(C46="","fecha · ","")&amp;IF(D46="","ubicación · ","")&amp;IF(E46="","referencia · ","")&amp;IF(H46="","criticidad · ","")&amp;IF(I46="","origen del agua · ","")&amp;IF(AND(LEFT(I46,7)="Sale de",J46="",K46=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C46:S46)=0,"",IF(AND(C46&lt;&gt;"",D46&lt;&gt;"",E46&lt;&gt;"",H46&lt;&gt;"",I46&lt;&gt;"",NOT(AND(LEFT(I46,7)="Sale de",J46="",K46=""))),"✔ Completa","Falta: "&amp;IF(C46="","fecha · ","")&amp;IF(D46="","ubicación · ","")&amp;IF(E46="","referencia · ","")&amp;IF(H46="","criticidad · ","")&amp;IF(I46="","origen del agua · ","")&amp;IF(AND(LEFT(I46,7)="Sale de",J46="",K46=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C46" s="17" t="n"/>
@@ -2441,8 +2507,9 @@
       <c r="N46" s="21" t="n"/>
       <c r="O46" s="21" t="n"/>
       <c r="P46" s="21" t="n"/>
-      <c r="Q46" s="18" t="n"/>
-      <c r="R46" s="19" t="n"/>
+      <c r="Q46" s="21" t="n"/>
+      <c r="R46" s="18" t="n"/>
+      <c r="S46" s="19" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="15" t="inlineStr">
@@ -2451,7 +2518,7 @@
         </is>
       </c>
       <c r="B47" s="16">
-        <f>IF(COUNTA(C47:R47)=0,"",IF(AND(C47&lt;&gt;"",D47&lt;&gt;"",E47&lt;&gt;"",H47&lt;&gt;"",I47&lt;&gt;"",NOT(AND(LEFT(I47,7)="Sale de",J47="",K47=""))),"✔ Completa","Falta: "&amp;IF(C47="","fecha · ","")&amp;IF(D47="","ubicación · ","")&amp;IF(E47="","referencia · ","")&amp;IF(H47="","criticidad · ","")&amp;IF(I47="","origen del agua · ","")&amp;IF(AND(LEFT(I47,7)="Sale de",J47="",K47=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C47:S47)=0,"",IF(AND(C47&lt;&gt;"",D47&lt;&gt;"",E47&lt;&gt;"",H47&lt;&gt;"",I47&lt;&gt;"",NOT(AND(LEFT(I47,7)="Sale de",J47="",K47=""))),"✔ Completa","Falta: "&amp;IF(C47="","fecha · ","")&amp;IF(D47="","ubicación · ","")&amp;IF(E47="","referencia · ","")&amp;IF(H47="","criticidad · ","")&amp;IF(I47="","origen del agua · ","")&amp;IF(AND(LEFT(I47,7)="Sale de",J47="",K47=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C47" s="17" t="n"/>
@@ -2468,8 +2535,9 @@
       <c r="N47" s="21" t="n"/>
       <c r="O47" s="21" t="n"/>
       <c r="P47" s="21" t="n"/>
-      <c r="Q47" s="18" t="n"/>
-      <c r="R47" s="19" t="n"/>
+      <c r="Q47" s="21" t="n"/>
+      <c r="R47" s="18" t="n"/>
+      <c r="S47" s="19" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="15" t="inlineStr">
@@ -2478,7 +2546,7 @@
         </is>
       </c>
       <c r="B48" s="16">
-        <f>IF(COUNTA(C48:R48)=0,"",IF(AND(C48&lt;&gt;"",D48&lt;&gt;"",E48&lt;&gt;"",H48&lt;&gt;"",I48&lt;&gt;"",NOT(AND(LEFT(I48,7)="Sale de",J48="",K48=""))),"✔ Completa","Falta: "&amp;IF(C48="","fecha · ","")&amp;IF(D48="","ubicación · ","")&amp;IF(E48="","referencia · ","")&amp;IF(H48="","criticidad · ","")&amp;IF(I48="","origen del agua · ","")&amp;IF(AND(LEFT(I48,7)="Sale de",J48="",K48=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C48:S48)=0,"",IF(AND(C48&lt;&gt;"",D48&lt;&gt;"",E48&lt;&gt;"",H48&lt;&gt;"",I48&lt;&gt;"",NOT(AND(LEFT(I48,7)="Sale de",J48="",K48=""))),"✔ Completa","Falta: "&amp;IF(C48="","fecha · ","")&amp;IF(D48="","ubicación · ","")&amp;IF(E48="","referencia · ","")&amp;IF(H48="","criticidad · ","")&amp;IF(I48="","origen del agua · ","")&amp;IF(AND(LEFT(I48,7)="Sale de",J48="",K48=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C48" s="17" t="n"/>
@@ -2495,8 +2563,9 @@
       <c r="N48" s="21" t="n"/>
       <c r="O48" s="21" t="n"/>
       <c r="P48" s="21" t="n"/>
-      <c r="Q48" s="18" t="n"/>
-      <c r="R48" s="19" t="n"/>
+      <c r="Q48" s="21" t="n"/>
+      <c r="R48" s="18" t="n"/>
+      <c r="S48" s="19" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="15" t="inlineStr">
@@ -2505,7 +2574,7 @@
         </is>
       </c>
       <c r="B49" s="16">
-        <f>IF(COUNTA(C49:R49)=0,"",IF(AND(C49&lt;&gt;"",D49&lt;&gt;"",E49&lt;&gt;"",H49&lt;&gt;"",I49&lt;&gt;"",NOT(AND(LEFT(I49,7)="Sale de",J49="",K49=""))),"✔ Completa","Falta: "&amp;IF(C49="","fecha · ","")&amp;IF(D49="","ubicación · ","")&amp;IF(E49="","referencia · ","")&amp;IF(H49="","criticidad · ","")&amp;IF(I49="","origen del agua · ","")&amp;IF(AND(LEFT(I49,7)="Sale de",J49="",K49=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C49:S49)=0,"",IF(AND(C49&lt;&gt;"",D49&lt;&gt;"",E49&lt;&gt;"",H49&lt;&gt;"",I49&lt;&gt;"",NOT(AND(LEFT(I49,7)="Sale de",J49="",K49=""))),"✔ Completa","Falta: "&amp;IF(C49="","fecha · ","")&amp;IF(D49="","ubicación · ","")&amp;IF(E49="","referencia · ","")&amp;IF(H49="","criticidad · ","")&amp;IF(I49="","origen del agua · ","")&amp;IF(AND(LEFT(I49,7)="Sale de",J49="",K49=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -2522,8 +2591,9 @@
       <c r="N49" s="21" t="n"/>
       <c r="O49" s="21" t="n"/>
       <c r="P49" s="21" t="n"/>
-      <c r="Q49" s="18" t="n"/>
-      <c r="R49" s="19" t="n"/>
+      <c r="Q49" s="21" t="n"/>
+      <c r="R49" s="18" t="n"/>
+      <c r="S49" s="19" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="15" t="inlineStr">
@@ -2532,7 +2602,7 @@
         </is>
       </c>
       <c r="B50" s="16">
-        <f>IF(COUNTA(C50:R50)=0,"",IF(AND(C50&lt;&gt;"",D50&lt;&gt;"",E50&lt;&gt;"",H50&lt;&gt;"",I50&lt;&gt;"",NOT(AND(LEFT(I50,7)="Sale de",J50="",K50=""))),"✔ Completa","Falta: "&amp;IF(C50="","fecha · ","")&amp;IF(D50="","ubicación · ","")&amp;IF(E50="","referencia · ","")&amp;IF(H50="","criticidad · ","")&amp;IF(I50="","origen del agua · ","")&amp;IF(AND(LEFT(I50,7)="Sale de",J50="",K50=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C50:S50)=0,"",IF(AND(C50&lt;&gt;"",D50&lt;&gt;"",E50&lt;&gt;"",H50&lt;&gt;"",I50&lt;&gt;"",NOT(AND(LEFT(I50,7)="Sale de",J50="",K50=""))),"✔ Completa","Falta: "&amp;IF(C50="","fecha · ","")&amp;IF(D50="","ubicación · ","")&amp;IF(E50="","referencia · ","")&amp;IF(H50="","criticidad · ","")&amp;IF(I50="","origen del agua · ","")&amp;IF(AND(LEFT(I50,7)="Sale de",J50="",K50=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C50" s="17" t="n"/>
@@ -2549,8 +2619,9 @@
       <c r="N50" s="21" t="n"/>
       <c r="O50" s="21" t="n"/>
       <c r="P50" s="21" t="n"/>
-      <c r="Q50" s="18" t="n"/>
-      <c r="R50" s="19" t="n"/>
+      <c r="Q50" s="21" t="n"/>
+      <c r="R50" s="18" t="n"/>
+      <c r="S50" s="19" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="15" t="inlineStr">
@@ -2559,7 +2630,7 @@
         </is>
       </c>
       <c r="B51" s="16">
-        <f>IF(COUNTA(C51:R51)=0,"",IF(AND(C51&lt;&gt;"",D51&lt;&gt;"",E51&lt;&gt;"",H51&lt;&gt;"",I51&lt;&gt;"",NOT(AND(LEFT(I51,7)="Sale de",J51="",K51=""))),"✔ Completa","Falta: "&amp;IF(C51="","fecha · ","")&amp;IF(D51="","ubicación · ","")&amp;IF(E51="","referencia · ","")&amp;IF(H51="","criticidad · ","")&amp;IF(I51="","origen del agua · ","")&amp;IF(AND(LEFT(I51,7)="Sale de",J51="",K51=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C51:S51)=0,"",IF(AND(C51&lt;&gt;"",D51&lt;&gt;"",E51&lt;&gt;"",H51&lt;&gt;"",I51&lt;&gt;"",NOT(AND(LEFT(I51,7)="Sale de",J51="",K51=""))),"✔ Completa","Falta: "&amp;IF(C51="","fecha · ","")&amp;IF(D51="","ubicación · ","")&amp;IF(E51="","referencia · ","")&amp;IF(H51="","criticidad · ","")&amp;IF(I51="","origen del agua · ","")&amp;IF(AND(LEFT(I51,7)="Sale de",J51="",K51=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C51" s="17" t="n"/>
@@ -2576,8 +2647,9 @@
       <c r="N51" s="21" t="n"/>
       <c r="O51" s="21" t="n"/>
       <c r="P51" s="21" t="n"/>
-      <c r="Q51" s="18" t="n"/>
-      <c r="R51" s="19" t="n"/>
+      <c r="Q51" s="21" t="n"/>
+      <c r="R51" s="18" t="n"/>
+      <c r="S51" s="19" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="15" t="inlineStr">
@@ -2586,7 +2658,7 @@
         </is>
       </c>
       <c r="B52" s="16">
-        <f>IF(COUNTA(C52:R52)=0,"",IF(AND(C52&lt;&gt;"",D52&lt;&gt;"",E52&lt;&gt;"",H52&lt;&gt;"",I52&lt;&gt;"",NOT(AND(LEFT(I52,7)="Sale de",J52="",K52=""))),"✔ Completa","Falta: "&amp;IF(C52="","fecha · ","")&amp;IF(D52="","ubicación · ","")&amp;IF(E52="","referencia · ","")&amp;IF(H52="","criticidad · ","")&amp;IF(I52="","origen del agua · ","")&amp;IF(AND(LEFT(I52,7)="Sale de",J52="",K52=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C52:S52)=0,"",IF(AND(C52&lt;&gt;"",D52&lt;&gt;"",E52&lt;&gt;"",H52&lt;&gt;"",I52&lt;&gt;"",NOT(AND(LEFT(I52,7)="Sale de",J52="",K52=""))),"✔ Completa","Falta: "&amp;IF(C52="","fecha · ","")&amp;IF(D52="","ubicación · ","")&amp;IF(E52="","referencia · ","")&amp;IF(H52="","criticidad · ","")&amp;IF(I52="","origen del agua · ","")&amp;IF(AND(LEFT(I52,7)="Sale de",J52="",K52=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C52" s="17" t="n"/>
@@ -2603,8 +2675,9 @@
       <c r="N52" s="21" t="n"/>
       <c r="O52" s="21" t="n"/>
       <c r="P52" s="21" t="n"/>
-      <c r="Q52" s="18" t="n"/>
-      <c r="R52" s="19" t="n"/>
+      <c r="Q52" s="21" t="n"/>
+      <c r="R52" s="18" t="n"/>
+      <c r="S52" s="19" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="15" t="inlineStr">
@@ -2613,7 +2686,7 @@
         </is>
       </c>
       <c r="B53" s="16">
-        <f>IF(COUNTA(C53:R53)=0,"",IF(AND(C53&lt;&gt;"",D53&lt;&gt;"",E53&lt;&gt;"",H53&lt;&gt;"",I53&lt;&gt;"",NOT(AND(LEFT(I53,7)="Sale de",J53="",K53=""))),"✔ Completa","Falta: "&amp;IF(C53="","fecha · ","")&amp;IF(D53="","ubicación · ","")&amp;IF(E53="","referencia · ","")&amp;IF(H53="","criticidad · ","")&amp;IF(I53="","origen del agua · ","")&amp;IF(AND(LEFT(I53,7)="Sale de",J53="",K53=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C53:S53)=0,"",IF(AND(C53&lt;&gt;"",D53&lt;&gt;"",E53&lt;&gt;"",H53&lt;&gt;"",I53&lt;&gt;"",NOT(AND(LEFT(I53,7)="Sale de",J53="",K53=""))),"✔ Completa","Falta: "&amp;IF(C53="","fecha · ","")&amp;IF(D53="","ubicación · ","")&amp;IF(E53="","referencia · ","")&amp;IF(H53="","criticidad · ","")&amp;IF(I53="","origen del agua · ","")&amp;IF(AND(LEFT(I53,7)="Sale de",J53="",K53=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C53" s="17" t="n"/>
@@ -2630,8 +2703,9 @@
       <c r="N53" s="21" t="n"/>
       <c r="O53" s="21" t="n"/>
       <c r="P53" s="21" t="n"/>
-      <c r="Q53" s="18" t="n"/>
-      <c r="R53" s="19" t="n"/>
+      <c r="Q53" s="21" t="n"/>
+      <c r="R53" s="18" t="n"/>
+      <c r="S53" s="19" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="15" t="inlineStr">
@@ -2640,7 +2714,7 @@
         </is>
       </c>
       <c r="B54" s="16">
-        <f>IF(COUNTA(C54:R54)=0,"",IF(AND(C54&lt;&gt;"",D54&lt;&gt;"",E54&lt;&gt;"",H54&lt;&gt;"",I54&lt;&gt;"",NOT(AND(LEFT(I54,7)="Sale de",J54="",K54=""))),"✔ Completa","Falta: "&amp;IF(C54="","fecha · ","")&amp;IF(D54="","ubicación · ","")&amp;IF(E54="","referencia · ","")&amp;IF(H54="","criticidad · ","")&amp;IF(I54="","origen del agua · ","")&amp;IF(AND(LEFT(I54,7)="Sale de",J54="",K54=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C54:S54)=0,"",IF(AND(C54&lt;&gt;"",D54&lt;&gt;"",E54&lt;&gt;"",H54&lt;&gt;"",I54&lt;&gt;"",NOT(AND(LEFT(I54,7)="Sale de",J54="",K54=""))),"✔ Completa","Falta: "&amp;IF(C54="","fecha · ","")&amp;IF(D54="","ubicación · ","")&amp;IF(E54="","referencia · ","")&amp;IF(H54="","criticidad · ","")&amp;IF(I54="","origen del agua · ","")&amp;IF(AND(LEFT(I54,7)="Sale de",J54="",K54=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C54" s="17" t="n"/>
@@ -2657,8 +2731,9 @@
       <c r="N54" s="21" t="n"/>
       <c r="O54" s="21" t="n"/>
       <c r="P54" s="21" t="n"/>
-      <c r="Q54" s="18" t="n"/>
-      <c r="R54" s="19" t="n"/>
+      <c r="Q54" s="21" t="n"/>
+      <c r="R54" s="18" t="n"/>
+      <c r="S54" s="19" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="15" t="inlineStr">
@@ -2667,7 +2742,7 @@
         </is>
       </c>
       <c r="B55" s="16">
-        <f>IF(COUNTA(C55:R55)=0,"",IF(AND(C55&lt;&gt;"",D55&lt;&gt;"",E55&lt;&gt;"",H55&lt;&gt;"",I55&lt;&gt;"",NOT(AND(LEFT(I55,7)="Sale de",J55="",K55=""))),"✔ Completa","Falta: "&amp;IF(C55="","fecha · ","")&amp;IF(D55="","ubicación · ","")&amp;IF(E55="","referencia · ","")&amp;IF(H55="","criticidad · ","")&amp;IF(I55="","origen del agua · ","")&amp;IF(AND(LEFT(I55,7)="Sale de",J55="",K55=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C55:S55)=0,"",IF(AND(C55&lt;&gt;"",D55&lt;&gt;"",E55&lt;&gt;"",H55&lt;&gt;"",I55&lt;&gt;"",NOT(AND(LEFT(I55,7)="Sale de",J55="",K55=""))),"✔ Completa","Falta: "&amp;IF(C55="","fecha · ","")&amp;IF(D55="","ubicación · ","")&amp;IF(E55="","referencia · ","")&amp;IF(H55="","criticidad · ","")&amp;IF(I55="","origen del agua · ","")&amp;IF(AND(LEFT(I55,7)="Sale de",J55="",K55=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C55" s="17" t="n"/>
@@ -2684,8 +2759,9 @@
       <c r="N55" s="21" t="n"/>
       <c r="O55" s="21" t="n"/>
       <c r="P55" s="21" t="n"/>
-      <c r="Q55" s="18" t="n"/>
-      <c r="R55" s="19" t="n"/>
+      <c r="Q55" s="21" t="n"/>
+      <c r="R55" s="18" t="n"/>
+      <c r="S55" s="19" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="15" t="inlineStr">
@@ -2694,7 +2770,7 @@
         </is>
       </c>
       <c r="B56" s="16">
-        <f>IF(COUNTA(C56:R56)=0,"",IF(AND(C56&lt;&gt;"",D56&lt;&gt;"",E56&lt;&gt;"",H56&lt;&gt;"",I56&lt;&gt;"",NOT(AND(LEFT(I56,7)="Sale de",J56="",K56=""))),"✔ Completa","Falta: "&amp;IF(C56="","fecha · ","")&amp;IF(D56="","ubicación · ","")&amp;IF(E56="","referencia · ","")&amp;IF(H56="","criticidad · ","")&amp;IF(I56="","origen del agua · ","")&amp;IF(AND(LEFT(I56,7)="Sale de",J56="",K56=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C56:S56)=0,"",IF(AND(C56&lt;&gt;"",D56&lt;&gt;"",E56&lt;&gt;"",H56&lt;&gt;"",I56&lt;&gt;"",NOT(AND(LEFT(I56,7)="Sale de",J56="",K56=""))),"✔ Completa","Falta: "&amp;IF(C56="","fecha · ","")&amp;IF(D56="","ubicación · ","")&amp;IF(E56="","referencia · ","")&amp;IF(H56="","criticidad · ","")&amp;IF(I56="","origen del agua · ","")&amp;IF(AND(LEFT(I56,7)="Sale de",J56="",K56=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C56" s="17" t="n"/>
@@ -2711,8 +2787,9 @@
       <c r="N56" s="21" t="n"/>
       <c r="O56" s="21" t="n"/>
       <c r="P56" s="21" t="n"/>
-      <c r="Q56" s="18" t="n"/>
-      <c r="R56" s="19" t="n"/>
+      <c r="Q56" s="21" t="n"/>
+      <c r="R56" s="18" t="n"/>
+      <c r="S56" s="19" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="15" t="inlineStr">
@@ -2721,7 +2798,7 @@
         </is>
       </c>
       <c r="B57" s="16">
-        <f>IF(COUNTA(C57:R57)=0,"",IF(AND(C57&lt;&gt;"",D57&lt;&gt;"",E57&lt;&gt;"",H57&lt;&gt;"",I57&lt;&gt;"",NOT(AND(LEFT(I57,7)="Sale de",J57="",K57=""))),"✔ Completa","Falta: "&amp;IF(C57="","fecha · ","")&amp;IF(D57="","ubicación · ","")&amp;IF(E57="","referencia · ","")&amp;IF(H57="","criticidad · ","")&amp;IF(I57="","origen del agua · ","")&amp;IF(AND(LEFT(I57,7)="Sale de",J57="",K57=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C57:S57)=0,"",IF(AND(C57&lt;&gt;"",D57&lt;&gt;"",E57&lt;&gt;"",H57&lt;&gt;"",I57&lt;&gt;"",NOT(AND(LEFT(I57,7)="Sale de",J57="",K57=""))),"✔ Completa","Falta: "&amp;IF(C57="","fecha · ","")&amp;IF(D57="","ubicación · ","")&amp;IF(E57="","referencia · ","")&amp;IF(H57="","criticidad · ","")&amp;IF(I57="","origen del agua · ","")&amp;IF(AND(LEFT(I57,7)="Sale de",J57="",K57=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C57" s="17" t="n"/>
@@ -2738,8 +2815,9 @@
       <c r="N57" s="21" t="n"/>
       <c r="O57" s="21" t="n"/>
       <c r="P57" s="21" t="n"/>
-      <c r="Q57" s="18" t="n"/>
-      <c r="R57" s="19" t="n"/>
+      <c r="Q57" s="21" t="n"/>
+      <c r="R57" s="18" t="n"/>
+      <c r="S57" s="19" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="15" t="inlineStr">
@@ -2748,7 +2826,7 @@
         </is>
       </c>
       <c r="B58" s="16">
-        <f>IF(COUNTA(C58:R58)=0,"",IF(AND(C58&lt;&gt;"",D58&lt;&gt;"",E58&lt;&gt;"",H58&lt;&gt;"",I58&lt;&gt;"",NOT(AND(LEFT(I58,7)="Sale de",J58="",K58=""))),"✔ Completa","Falta: "&amp;IF(C58="","fecha · ","")&amp;IF(D58="","ubicación · ","")&amp;IF(E58="","referencia · ","")&amp;IF(H58="","criticidad · ","")&amp;IF(I58="","origen del agua · ","")&amp;IF(AND(LEFT(I58,7)="Sale de",J58="",K58=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C58:S58)=0,"",IF(AND(C58&lt;&gt;"",D58&lt;&gt;"",E58&lt;&gt;"",H58&lt;&gt;"",I58&lt;&gt;"",NOT(AND(LEFT(I58,7)="Sale de",J58="",K58=""))),"✔ Completa","Falta: "&amp;IF(C58="","fecha · ","")&amp;IF(D58="","ubicación · ","")&amp;IF(E58="","referencia · ","")&amp;IF(H58="","criticidad · ","")&amp;IF(I58="","origen del agua · ","")&amp;IF(AND(LEFT(I58,7)="Sale de",J58="",K58=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C58" s="17" t="n"/>
@@ -2765,8 +2843,9 @@
       <c r="N58" s="21" t="n"/>
       <c r="O58" s="21" t="n"/>
       <c r="P58" s="21" t="n"/>
-      <c r="Q58" s="18" t="n"/>
-      <c r="R58" s="19" t="n"/>
+      <c r="Q58" s="21" t="n"/>
+      <c r="R58" s="18" t="n"/>
+      <c r="S58" s="19" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="15" t="inlineStr">
@@ -2775,7 +2854,7 @@
         </is>
       </c>
       <c r="B59" s="16">
-        <f>IF(COUNTA(C59:R59)=0,"",IF(AND(C59&lt;&gt;"",D59&lt;&gt;"",E59&lt;&gt;"",H59&lt;&gt;"",I59&lt;&gt;"",NOT(AND(LEFT(I59,7)="Sale de",J59="",K59=""))),"✔ Completa","Falta: "&amp;IF(C59="","fecha · ","")&amp;IF(D59="","ubicación · ","")&amp;IF(E59="","referencia · ","")&amp;IF(H59="","criticidad · ","")&amp;IF(I59="","origen del agua · ","")&amp;IF(AND(LEFT(I59,7)="Sale de",J59="",K59=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C59:S59)=0,"",IF(AND(C59&lt;&gt;"",D59&lt;&gt;"",E59&lt;&gt;"",H59&lt;&gt;"",I59&lt;&gt;"",NOT(AND(LEFT(I59,7)="Sale de",J59="",K59=""))),"✔ Completa","Falta: "&amp;IF(C59="","fecha · ","")&amp;IF(D59="","ubicación · ","")&amp;IF(E59="","referencia · ","")&amp;IF(H59="","criticidad · ","")&amp;IF(I59="","origen del agua · ","")&amp;IF(AND(LEFT(I59,7)="Sale de",J59="",K59=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C59" s="17" t="n"/>
@@ -2792,8 +2871,9 @@
       <c r="N59" s="21" t="n"/>
       <c r="O59" s="21" t="n"/>
       <c r="P59" s="21" t="n"/>
-      <c r="Q59" s="18" t="n"/>
-      <c r="R59" s="19" t="n"/>
+      <c r="Q59" s="21" t="n"/>
+      <c r="R59" s="18" t="n"/>
+      <c r="S59" s="19" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="15" t="inlineStr">
@@ -2802,7 +2882,7 @@
         </is>
       </c>
       <c r="B60" s="16">
-        <f>IF(COUNTA(C60:R60)=0,"",IF(AND(C60&lt;&gt;"",D60&lt;&gt;"",E60&lt;&gt;"",H60&lt;&gt;"",I60&lt;&gt;"",NOT(AND(LEFT(I60,7)="Sale de",J60="",K60=""))),"✔ Completa","Falta: "&amp;IF(C60="","fecha · ","")&amp;IF(D60="","ubicación · ","")&amp;IF(E60="","referencia · ","")&amp;IF(H60="","criticidad · ","")&amp;IF(I60="","origen del agua · ","")&amp;IF(AND(LEFT(I60,7)="Sale de",J60="",K60=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C60:S60)=0,"",IF(AND(C60&lt;&gt;"",D60&lt;&gt;"",E60&lt;&gt;"",H60&lt;&gt;"",I60&lt;&gt;"",NOT(AND(LEFT(I60,7)="Sale de",J60="",K60=""))),"✔ Completa","Falta: "&amp;IF(C60="","fecha · ","")&amp;IF(D60="","ubicación · ","")&amp;IF(E60="","referencia · ","")&amp;IF(H60="","criticidad · ","")&amp;IF(I60="","origen del agua · ","")&amp;IF(AND(LEFT(I60,7)="Sale de",J60="",K60=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C60" s="17" t="n"/>
@@ -2819,8 +2899,9 @@
       <c r="N60" s="21" t="n"/>
       <c r="O60" s="21" t="n"/>
       <c r="P60" s="21" t="n"/>
-      <c r="Q60" s="18" t="n"/>
-      <c r="R60" s="19" t="n"/>
+      <c r="Q60" s="21" t="n"/>
+      <c r="R60" s="18" t="n"/>
+      <c r="S60" s="19" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
@@ -2829,7 +2910,7 @@
         </is>
       </c>
       <c r="B61" s="16">
-        <f>IF(COUNTA(C61:R61)=0,"",IF(AND(C61&lt;&gt;"",D61&lt;&gt;"",E61&lt;&gt;"",H61&lt;&gt;"",I61&lt;&gt;"",NOT(AND(LEFT(I61,7)="Sale de",J61="",K61=""))),"✔ Completa","Falta: "&amp;IF(C61="","fecha · ","")&amp;IF(D61="","ubicación · ","")&amp;IF(E61="","referencia · ","")&amp;IF(H61="","criticidad · ","")&amp;IF(I61="","origen del agua · ","")&amp;IF(AND(LEFT(I61,7)="Sale de",J61="",K61=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C61:S61)=0,"",IF(AND(C61&lt;&gt;"",D61&lt;&gt;"",E61&lt;&gt;"",H61&lt;&gt;"",I61&lt;&gt;"",NOT(AND(LEFT(I61,7)="Sale de",J61="",K61=""))),"✔ Completa","Falta: "&amp;IF(C61="","fecha · ","")&amp;IF(D61="","ubicación · ","")&amp;IF(E61="","referencia · ","")&amp;IF(H61="","criticidad · ","")&amp;IF(I61="","origen del agua · ","")&amp;IF(AND(LEFT(I61,7)="Sale de",J61="",K61=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C61" s="17" t="n"/>
@@ -2846,8 +2927,9 @@
       <c r="N61" s="21" t="n"/>
       <c r="O61" s="21" t="n"/>
       <c r="P61" s="21" t="n"/>
-      <c r="Q61" s="18" t="n"/>
-      <c r="R61" s="19" t="n"/>
+      <c r="Q61" s="21" t="n"/>
+      <c r="R61" s="18" t="n"/>
+      <c r="S61" s="19" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="15" t="inlineStr">
@@ -2856,7 +2938,7 @@
         </is>
       </c>
       <c r="B62" s="16">
-        <f>IF(COUNTA(C62:R62)=0,"",IF(AND(C62&lt;&gt;"",D62&lt;&gt;"",E62&lt;&gt;"",H62&lt;&gt;"",I62&lt;&gt;"",NOT(AND(LEFT(I62,7)="Sale de",J62="",K62=""))),"✔ Completa","Falta: "&amp;IF(C62="","fecha · ","")&amp;IF(D62="","ubicación · ","")&amp;IF(E62="","referencia · ","")&amp;IF(H62="","criticidad · ","")&amp;IF(I62="","origen del agua · ","")&amp;IF(AND(LEFT(I62,7)="Sale de",J62="",K62=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C62:S62)=0,"",IF(AND(C62&lt;&gt;"",D62&lt;&gt;"",E62&lt;&gt;"",H62&lt;&gt;"",I62&lt;&gt;"",NOT(AND(LEFT(I62,7)="Sale de",J62="",K62=""))),"✔ Completa","Falta: "&amp;IF(C62="","fecha · ","")&amp;IF(D62="","ubicación · ","")&amp;IF(E62="","referencia · ","")&amp;IF(H62="","criticidad · ","")&amp;IF(I62="","origen del agua · ","")&amp;IF(AND(LEFT(I62,7)="Sale de",J62="",K62=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C62" s="17" t="n"/>
@@ -2873,8 +2955,9 @@
       <c r="N62" s="21" t="n"/>
       <c r="O62" s="21" t="n"/>
       <c r="P62" s="21" t="n"/>
-      <c r="Q62" s="18" t="n"/>
-      <c r="R62" s="19" t="n"/>
+      <c r="Q62" s="21" t="n"/>
+      <c r="R62" s="18" t="n"/>
+      <c r="S62" s="19" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="15" t="inlineStr">
@@ -2883,7 +2966,7 @@
         </is>
       </c>
       <c r="B63" s="16">
-        <f>IF(COUNTA(C63:R63)=0,"",IF(AND(C63&lt;&gt;"",D63&lt;&gt;"",E63&lt;&gt;"",H63&lt;&gt;"",I63&lt;&gt;"",NOT(AND(LEFT(I63,7)="Sale de",J63="",K63=""))),"✔ Completa","Falta: "&amp;IF(C63="","fecha · ","")&amp;IF(D63="","ubicación · ","")&amp;IF(E63="","referencia · ","")&amp;IF(H63="","criticidad · ","")&amp;IF(I63="","origen del agua · ","")&amp;IF(AND(LEFT(I63,7)="Sale de",J63="",K63=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C63:S63)=0,"",IF(AND(C63&lt;&gt;"",D63&lt;&gt;"",E63&lt;&gt;"",H63&lt;&gt;"",I63&lt;&gt;"",NOT(AND(LEFT(I63,7)="Sale de",J63="",K63=""))),"✔ Completa","Falta: "&amp;IF(C63="","fecha · ","")&amp;IF(D63="","ubicación · ","")&amp;IF(E63="","referencia · ","")&amp;IF(H63="","criticidad · ","")&amp;IF(I63="","origen del agua · ","")&amp;IF(AND(LEFT(I63,7)="Sale de",J63="",K63=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C63" s="17" t="n"/>
@@ -2900,8 +2983,9 @@
       <c r="N63" s="21" t="n"/>
       <c r="O63" s="21" t="n"/>
       <c r="P63" s="21" t="n"/>
-      <c r="Q63" s="18" t="n"/>
-      <c r="R63" s="19" t="n"/>
+      <c r="Q63" s="21" t="n"/>
+      <c r="R63" s="18" t="n"/>
+      <c r="S63" s="19" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="15" t="inlineStr">
@@ -2910,7 +2994,7 @@
         </is>
       </c>
       <c r="B64" s="16">
-        <f>IF(COUNTA(C64:R64)=0,"",IF(AND(C64&lt;&gt;"",D64&lt;&gt;"",E64&lt;&gt;"",H64&lt;&gt;"",I64&lt;&gt;"",NOT(AND(LEFT(I64,7)="Sale de",J64="",K64=""))),"✔ Completa","Falta: "&amp;IF(C64="","fecha · ","")&amp;IF(D64="","ubicación · ","")&amp;IF(E64="","referencia · ","")&amp;IF(H64="","criticidad · ","")&amp;IF(I64="","origen del agua · ","")&amp;IF(AND(LEFT(I64,7)="Sale de",J64="",K64=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C64:S64)=0,"",IF(AND(C64&lt;&gt;"",D64&lt;&gt;"",E64&lt;&gt;"",H64&lt;&gt;"",I64&lt;&gt;"",NOT(AND(LEFT(I64,7)="Sale de",J64="",K64=""))),"✔ Completa","Falta: "&amp;IF(C64="","fecha · ","")&amp;IF(D64="","ubicación · ","")&amp;IF(E64="","referencia · ","")&amp;IF(H64="","criticidad · ","")&amp;IF(I64="","origen del agua · ","")&amp;IF(AND(LEFT(I64,7)="Sale de",J64="",K64=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C64" s="17" t="n"/>
@@ -2927,8 +3011,9 @@
       <c r="N64" s="21" t="n"/>
       <c r="O64" s="21" t="n"/>
       <c r="P64" s="21" t="n"/>
-      <c r="Q64" s="18" t="n"/>
-      <c r="R64" s="19" t="n"/>
+      <c r="Q64" s="21" t="n"/>
+      <c r="R64" s="18" t="n"/>
+      <c r="S64" s="19" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
@@ -2937,7 +3022,7 @@
         </is>
       </c>
       <c r="B65" s="16">
-        <f>IF(COUNTA(C65:R65)=0,"",IF(AND(C65&lt;&gt;"",D65&lt;&gt;"",E65&lt;&gt;"",H65&lt;&gt;"",I65&lt;&gt;"",NOT(AND(LEFT(I65,7)="Sale de",J65="",K65=""))),"✔ Completa","Falta: "&amp;IF(C65="","fecha · ","")&amp;IF(D65="","ubicación · ","")&amp;IF(E65="","referencia · ","")&amp;IF(H65="","criticidad · ","")&amp;IF(I65="","origen del agua · ","")&amp;IF(AND(LEFT(I65,7)="Sale de",J65="",K65=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C65:S65)=0,"",IF(AND(C65&lt;&gt;"",D65&lt;&gt;"",E65&lt;&gt;"",H65&lt;&gt;"",I65&lt;&gt;"",NOT(AND(LEFT(I65,7)="Sale de",J65="",K65=""))),"✔ Completa","Falta: "&amp;IF(C65="","fecha · ","")&amp;IF(D65="","ubicación · ","")&amp;IF(E65="","referencia · ","")&amp;IF(H65="","criticidad · ","")&amp;IF(I65="","origen del agua · ","")&amp;IF(AND(LEFT(I65,7)="Sale de",J65="",K65=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C65" s="17" t="n"/>
@@ -2954,8 +3039,9 @@
       <c r="N65" s="21" t="n"/>
       <c r="O65" s="21" t="n"/>
       <c r="P65" s="21" t="n"/>
-      <c r="Q65" s="18" t="n"/>
-      <c r="R65" s="19" t="n"/>
+      <c r="Q65" s="21" t="n"/>
+      <c r="R65" s="18" t="n"/>
+      <c r="S65" s="19" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="15" t="inlineStr">
@@ -2964,7 +3050,7 @@
         </is>
       </c>
       <c r="B66" s="16">
-        <f>IF(COUNTA(C66:R66)=0,"",IF(AND(C66&lt;&gt;"",D66&lt;&gt;"",E66&lt;&gt;"",H66&lt;&gt;"",I66&lt;&gt;"",NOT(AND(LEFT(I66,7)="Sale de",J66="",K66=""))),"✔ Completa","Falta: "&amp;IF(C66="","fecha · ","")&amp;IF(D66="","ubicación · ","")&amp;IF(E66="","referencia · ","")&amp;IF(H66="","criticidad · ","")&amp;IF(I66="","origen del agua · ","")&amp;IF(AND(LEFT(I66,7)="Sale de",J66="",K66=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C66:S66)=0,"",IF(AND(C66&lt;&gt;"",D66&lt;&gt;"",E66&lt;&gt;"",H66&lt;&gt;"",I66&lt;&gt;"",NOT(AND(LEFT(I66,7)="Sale de",J66="",K66=""))),"✔ Completa","Falta: "&amp;IF(C66="","fecha · ","")&amp;IF(D66="","ubicación · ","")&amp;IF(E66="","referencia · ","")&amp;IF(H66="","criticidad · ","")&amp;IF(I66="","origen del agua · ","")&amp;IF(AND(LEFT(I66,7)="Sale de",J66="",K66=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C66" s="17" t="n"/>
@@ -2981,8 +3067,9 @@
       <c r="N66" s="21" t="n"/>
       <c r="O66" s="21" t="n"/>
       <c r="P66" s="21" t="n"/>
-      <c r="Q66" s="18" t="n"/>
-      <c r="R66" s="19" t="n"/>
+      <c r="Q66" s="21" t="n"/>
+      <c r="R66" s="18" t="n"/>
+      <c r="S66" s="19" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="15" t="inlineStr">
@@ -2991,7 +3078,7 @@
         </is>
       </c>
       <c r="B67" s="16">
-        <f>IF(COUNTA(C67:R67)=0,"",IF(AND(C67&lt;&gt;"",D67&lt;&gt;"",E67&lt;&gt;"",H67&lt;&gt;"",I67&lt;&gt;"",NOT(AND(LEFT(I67,7)="Sale de",J67="",K67=""))),"✔ Completa","Falta: "&amp;IF(C67="","fecha · ","")&amp;IF(D67="","ubicación · ","")&amp;IF(E67="","referencia · ","")&amp;IF(H67="","criticidad · ","")&amp;IF(I67="","origen del agua · ","")&amp;IF(AND(LEFT(I67,7)="Sale de",J67="",K67=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C67:S67)=0,"",IF(AND(C67&lt;&gt;"",D67&lt;&gt;"",E67&lt;&gt;"",H67&lt;&gt;"",I67&lt;&gt;"",NOT(AND(LEFT(I67,7)="Sale de",J67="",K67=""))),"✔ Completa","Falta: "&amp;IF(C67="","fecha · ","")&amp;IF(D67="","ubicación · ","")&amp;IF(E67="","referencia · ","")&amp;IF(H67="","criticidad · ","")&amp;IF(I67="","origen del agua · ","")&amp;IF(AND(LEFT(I67,7)="Sale de",J67="",K67=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C67" s="17" t="n"/>
@@ -3008,8 +3095,9 @@
       <c r="N67" s="21" t="n"/>
       <c r="O67" s="21" t="n"/>
       <c r="P67" s="21" t="n"/>
-      <c r="Q67" s="18" t="n"/>
-      <c r="R67" s="19" t="n"/>
+      <c r="Q67" s="21" t="n"/>
+      <c r="R67" s="18" t="n"/>
+      <c r="S67" s="19" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="15" t="inlineStr">
@@ -3018,7 +3106,7 @@
         </is>
       </c>
       <c r="B68" s="16">
-        <f>IF(COUNTA(C68:R68)=0,"",IF(AND(C68&lt;&gt;"",D68&lt;&gt;"",E68&lt;&gt;"",H68&lt;&gt;"",I68&lt;&gt;"",NOT(AND(LEFT(I68,7)="Sale de",J68="",K68=""))),"✔ Completa","Falta: "&amp;IF(C68="","fecha · ","")&amp;IF(D68="","ubicación · ","")&amp;IF(E68="","referencia · ","")&amp;IF(H68="","criticidad · ","")&amp;IF(I68="","origen del agua · ","")&amp;IF(AND(LEFT(I68,7)="Sale de",J68="",K68=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C68:S68)=0,"",IF(AND(C68&lt;&gt;"",D68&lt;&gt;"",E68&lt;&gt;"",H68&lt;&gt;"",I68&lt;&gt;"",NOT(AND(LEFT(I68,7)="Sale de",J68="",K68=""))),"✔ Completa","Falta: "&amp;IF(C68="","fecha · ","")&amp;IF(D68="","ubicación · ","")&amp;IF(E68="","referencia · ","")&amp;IF(H68="","criticidad · ","")&amp;IF(I68="","origen del agua · ","")&amp;IF(AND(LEFT(I68,7)="Sale de",J68="",K68=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C68" s="17" t="n"/>
@@ -3035,8 +3123,9 @@
       <c r="N68" s="21" t="n"/>
       <c r="O68" s="21" t="n"/>
       <c r="P68" s="21" t="n"/>
-      <c r="Q68" s="18" t="n"/>
-      <c r="R68" s="19" t="n"/>
+      <c r="Q68" s="21" t="n"/>
+      <c r="R68" s="18" t="n"/>
+      <c r="S68" s="19" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
@@ -3045,7 +3134,7 @@
         </is>
       </c>
       <c r="B69" s="16">
-        <f>IF(COUNTA(C69:R69)=0,"",IF(AND(C69&lt;&gt;"",D69&lt;&gt;"",E69&lt;&gt;"",H69&lt;&gt;"",I69&lt;&gt;"",NOT(AND(LEFT(I69,7)="Sale de",J69="",K69=""))),"✔ Completa","Falta: "&amp;IF(C69="","fecha · ","")&amp;IF(D69="","ubicación · ","")&amp;IF(E69="","referencia · ","")&amp;IF(H69="","criticidad · ","")&amp;IF(I69="","origen del agua · ","")&amp;IF(AND(LEFT(I69,7)="Sale de",J69="",K69=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C69:S69)=0,"",IF(AND(C69&lt;&gt;"",D69&lt;&gt;"",E69&lt;&gt;"",H69&lt;&gt;"",I69&lt;&gt;"",NOT(AND(LEFT(I69,7)="Sale de",J69="",K69=""))),"✔ Completa","Falta: "&amp;IF(C69="","fecha · ","")&amp;IF(D69="","ubicación · ","")&amp;IF(E69="","referencia · ","")&amp;IF(H69="","criticidad · ","")&amp;IF(I69="","origen del agua · ","")&amp;IF(AND(LEFT(I69,7)="Sale de",J69="",K69=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C69" s="17" t="n"/>
@@ -3062,8 +3151,9 @@
       <c r="N69" s="21" t="n"/>
       <c r="O69" s="21" t="n"/>
       <c r="P69" s="21" t="n"/>
-      <c r="Q69" s="18" t="n"/>
-      <c r="R69" s="19" t="n"/>
+      <c r="Q69" s="21" t="n"/>
+      <c r="R69" s="18" t="n"/>
+      <c r="S69" s="19" t="n"/>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="15" t="inlineStr">
@@ -3072,7 +3162,7 @@
         </is>
       </c>
       <c r="B70" s="16">
-        <f>IF(COUNTA(C70:R70)=0,"",IF(AND(C70&lt;&gt;"",D70&lt;&gt;"",E70&lt;&gt;"",H70&lt;&gt;"",I70&lt;&gt;"",NOT(AND(LEFT(I70,7)="Sale de",J70="",K70=""))),"✔ Completa","Falta: "&amp;IF(C70="","fecha · ","")&amp;IF(D70="","ubicación · ","")&amp;IF(E70="","referencia · ","")&amp;IF(H70="","criticidad · ","")&amp;IF(I70="","origen del agua · ","")&amp;IF(AND(LEFT(I70,7)="Sale de",J70="",K70=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C70:S70)=0,"",IF(AND(C70&lt;&gt;"",D70&lt;&gt;"",E70&lt;&gt;"",H70&lt;&gt;"",I70&lt;&gt;"",NOT(AND(LEFT(I70,7)="Sale de",J70="",K70=""))),"✔ Completa","Falta: "&amp;IF(C70="","fecha · ","")&amp;IF(D70="","ubicación · ","")&amp;IF(E70="","referencia · ","")&amp;IF(H70="","criticidad · ","")&amp;IF(I70="","origen del agua · ","")&amp;IF(AND(LEFT(I70,7)="Sale de",J70="",K70=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C70" s="17" t="n"/>
@@ -3089,8 +3179,9 @@
       <c r="N70" s="21" t="n"/>
       <c r="O70" s="21" t="n"/>
       <c r="P70" s="21" t="n"/>
-      <c r="Q70" s="18" t="n"/>
-      <c r="R70" s="19" t="n"/>
+      <c r="Q70" s="21" t="n"/>
+      <c r="R70" s="18" t="n"/>
+      <c r="S70" s="19" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="15" t="inlineStr">
@@ -3099,7 +3190,7 @@
         </is>
       </c>
       <c r="B71" s="16">
-        <f>IF(COUNTA(C71:R71)=0,"",IF(AND(C71&lt;&gt;"",D71&lt;&gt;"",E71&lt;&gt;"",H71&lt;&gt;"",I71&lt;&gt;"",NOT(AND(LEFT(I71,7)="Sale de",J71="",K71=""))),"✔ Completa","Falta: "&amp;IF(C71="","fecha · ","")&amp;IF(D71="","ubicación · ","")&amp;IF(E71="","referencia · ","")&amp;IF(H71="","criticidad · ","")&amp;IF(I71="","origen del agua · ","")&amp;IF(AND(LEFT(I71,7)="Sale de",J71="",K71=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C71:S71)=0,"",IF(AND(C71&lt;&gt;"",D71&lt;&gt;"",E71&lt;&gt;"",H71&lt;&gt;"",I71&lt;&gt;"",NOT(AND(LEFT(I71,7)="Sale de",J71="",K71=""))),"✔ Completa","Falta: "&amp;IF(C71="","fecha · ","")&amp;IF(D71="","ubicación · ","")&amp;IF(E71="","referencia · ","")&amp;IF(H71="","criticidad · ","")&amp;IF(I71="","origen del agua · ","")&amp;IF(AND(LEFT(I71,7)="Sale de",J71="",K71=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C71" s="17" t="n"/>
@@ -3116,8 +3207,9 @@
       <c r="N71" s="21" t="n"/>
       <c r="O71" s="21" t="n"/>
       <c r="P71" s="21" t="n"/>
-      <c r="Q71" s="18" t="n"/>
-      <c r="R71" s="19" t="n"/>
+      <c r="Q71" s="21" t="n"/>
+      <c r="R71" s="18" t="n"/>
+      <c r="S71" s="19" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="15" t="inlineStr">
@@ -3126,7 +3218,7 @@
         </is>
       </c>
       <c r="B72" s="16">
-        <f>IF(COUNTA(C72:R72)=0,"",IF(AND(C72&lt;&gt;"",D72&lt;&gt;"",E72&lt;&gt;"",H72&lt;&gt;"",I72&lt;&gt;"",NOT(AND(LEFT(I72,7)="Sale de",J72="",K72=""))),"✔ Completa","Falta: "&amp;IF(C72="","fecha · ","")&amp;IF(D72="","ubicación · ","")&amp;IF(E72="","referencia · ","")&amp;IF(H72="","criticidad · ","")&amp;IF(I72="","origen del agua · ","")&amp;IF(AND(LEFT(I72,7)="Sale de",J72="",K72=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C72:S72)=0,"",IF(AND(C72&lt;&gt;"",D72&lt;&gt;"",E72&lt;&gt;"",H72&lt;&gt;"",I72&lt;&gt;"",NOT(AND(LEFT(I72,7)="Sale de",J72="",K72=""))),"✔ Completa","Falta: "&amp;IF(C72="","fecha · ","")&amp;IF(D72="","ubicación · ","")&amp;IF(E72="","referencia · ","")&amp;IF(H72="","criticidad · ","")&amp;IF(I72="","origen del agua · ","")&amp;IF(AND(LEFT(I72,7)="Sale de",J72="",K72=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C72" s="17" t="n"/>
@@ -3143,8 +3235,9 @@
       <c r="N72" s="21" t="n"/>
       <c r="O72" s="21" t="n"/>
       <c r="P72" s="21" t="n"/>
-      <c r="Q72" s="18" t="n"/>
-      <c r="R72" s="19" t="n"/>
+      <c r="Q72" s="21" t="n"/>
+      <c r="R72" s="18" t="n"/>
+      <c r="S72" s="19" t="n"/>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="15" t="inlineStr">
@@ -3153,7 +3246,7 @@
         </is>
       </c>
       <c r="B73" s="16">
-        <f>IF(COUNTA(C73:R73)=0,"",IF(AND(C73&lt;&gt;"",D73&lt;&gt;"",E73&lt;&gt;"",H73&lt;&gt;"",I73&lt;&gt;"",NOT(AND(LEFT(I73,7)="Sale de",J73="",K73=""))),"✔ Completa","Falta: "&amp;IF(C73="","fecha · ","")&amp;IF(D73="","ubicación · ","")&amp;IF(E73="","referencia · ","")&amp;IF(H73="","criticidad · ","")&amp;IF(I73="","origen del agua · ","")&amp;IF(AND(LEFT(I73,7)="Sale de",J73="",K73=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C73:S73)=0,"",IF(AND(C73&lt;&gt;"",D73&lt;&gt;"",E73&lt;&gt;"",H73&lt;&gt;"",I73&lt;&gt;"",NOT(AND(LEFT(I73,7)="Sale de",J73="",K73=""))),"✔ Completa","Falta: "&amp;IF(C73="","fecha · ","")&amp;IF(D73="","ubicación · ","")&amp;IF(E73="","referencia · ","")&amp;IF(H73="","criticidad · ","")&amp;IF(I73="","origen del agua · ","")&amp;IF(AND(LEFT(I73,7)="Sale de",J73="",K73=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C73" s="17" t="n"/>
@@ -3170,8 +3263,9 @@
       <c r="N73" s="21" t="n"/>
       <c r="O73" s="21" t="n"/>
       <c r="P73" s="21" t="n"/>
-      <c r="Q73" s="18" t="n"/>
-      <c r="R73" s="19" t="n"/>
+      <c r="Q73" s="21" t="n"/>
+      <c r="R73" s="18" t="n"/>
+      <c r="S73" s="19" t="n"/>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="15" t="inlineStr">
@@ -3180,7 +3274,7 @@
         </is>
       </c>
       <c r="B74" s="16">
-        <f>IF(COUNTA(C74:R74)=0,"",IF(AND(C74&lt;&gt;"",D74&lt;&gt;"",E74&lt;&gt;"",H74&lt;&gt;"",I74&lt;&gt;"",NOT(AND(LEFT(I74,7)="Sale de",J74="",K74=""))),"✔ Completa","Falta: "&amp;IF(C74="","fecha · ","")&amp;IF(D74="","ubicación · ","")&amp;IF(E74="","referencia · ","")&amp;IF(H74="","criticidad · ","")&amp;IF(I74="","origen del agua · ","")&amp;IF(AND(LEFT(I74,7)="Sale de",J74="",K74=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C74:S74)=0,"",IF(AND(C74&lt;&gt;"",D74&lt;&gt;"",E74&lt;&gt;"",H74&lt;&gt;"",I74&lt;&gt;"",NOT(AND(LEFT(I74,7)="Sale de",J74="",K74=""))),"✔ Completa","Falta: "&amp;IF(C74="","fecha · ","")&amp;IF(D74="","ubicación · ","")&amp;IF(E74="","referencia · ","")&amp;IF(H74="","criticidad · ","")&amp;IF(I74="","origen del agua · ","")&amp;IF(AND(LEFT(I74,7)="Sale de",J74="",K74=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C74" s="17" t="n"/>
@@ -3197,8 +3291,9 @@
       <c r="N74" s="21" t="n"/>
       <c r="O74" s="21" t="n"/>
       <c r="P74" s="21" t="n"/>
-      <c r="Q74" s="18" t="n"/>
-      <c r="R74" s="19" t="n"/>
+      <c r="Q74" s="21" t="n"/>
+      <c r="R74" s="18" t="n"/>
+      <c r="S74" s="19" t="n"/>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="15" t="inlineStr">
@@ -3207,7 +3302,7 @@
         </is>
       </c>
       <c r="B75" s="16">
-        <f>IF(COUNTA(C75:R75)=0,"",IF(AND(C75&lt;&gt;"",D75&lt;&gt;"",E75&lt;&gt;"",H75&lt;&gt;"",I75&lt;&gt;"",NOT(AND(LEFT(I75,7)="Sale de",J75="",K75=""))),"✔ Completa","Falta: "&amp;IF(C75="","fecha · ","")&amp;IF(D75="","ubicación · ","")&amp;IF(E75="","referencia · ","")&amp;IF(H75="","criticidad · ","")&amp;IF(I75="","origen del agua · ","")&amp;IF(AND(LEFT(I75,7)="Sale de",J75="",K75=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C75:S75)=0,"",IF(AND(C75&lt;&gt;"",D75&lt;&gt;"",E75&lt;&gt;"",H75&lt;&gt;"",I75&lt;&gt;"",NOT(AND(LEFT(I75,7)="Sale de",J75="",K75=""))),"✔ Completa","Falta: "&amp;IF(C75="","fecha · ","")&amp;IF(D75="","ubicación · ","")&amp;IF(E75="","referencia · ","")&amp;IF(H75="","criticidad · ","")&amp;IF(I75="","origen del agua · ","")&amp;IF(AND(LEFT(I75,7)="Sale de",J75="",K75=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C75" s="17" t="n"/>
@@ -3224,8 +3319,9 @@
       <c r="N75" s="21" t="n"/>
       <c r="O75" s="21" t="n"/>
       <c r="P75" s="21" t="n"/>
-      <c r="Q75" s="18" t="n"/>
-      <c r="R75" s="19" t="n"/>
+      <c r="Q75" s="21" t="n"/>
+      <c r="R75" s="18" t="n"/>
+      <c r="S75" s="19" t="n"/>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="15" t="inlineStr">
@@ -3234,7 +3330,7 @@
         </is>
       </c>
       <c r="B76" s="16">
-        <f>IF(COUNTA(C76:R76)=0,"",IF(AND(C76&lt;&gt;"",D76&lt;&gt;"",E76&lt;&gt;"",H76&lt;&gt;"",I76&lt;&gt;"",NOT(AND(LEFT(I76,7)="Sale de",J76="",K76=""))),"✔ Completa","Falta: "&amp;IF(C76="","fecha · ","")&amp;IF(D76="","ubicación · ","")&amp;IF(E76="","referencia · ","")&amp;IF(H76="","criticidad · ","")&amp;IF(I76="","origen del agua · ","")&amp;IF(AND(LEFT(I76,7)="Sale de",J76="",K76=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C76:S76)=0,"",IF(AND(C76&lt;&gt;"",D76&lt;&gt;"",E76&lt;&gt;"",H76&lt;&gt;"",I76&lt;&gt;"",NOT(AND(LEFT(I76,7)="Sale de",J76="",K76=""))),"✔ Completa","Falta: "&amp;IF(C76="","fecha · ","")&amp;IF(D76="","ubicación · ","")&amp;IF(E76="","referencia · ","")&amp;IF(H76="","criticidad · ","")&amp;IF(I76="","origen del agua · ","")&amp;IF(AND(LEFT(I76,7)="Sale de",J76="",K76=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C76" s="17" t="n"/>
@@ -3251,8 +3347,9 @@
       <c r="N76" s="21" t="n"/>
       <c r="O76" s="21" t="n"/>
       <c r="P76" s="21" t="n"/>
-      <c r="Q76" s="18" t="n"/>
-      <c r="R76" s="19" t="n"/>
+      <c r="Q76" s="21" t="n"/>
+      <c r="R76" s="18" t="n"/>
+      <c r="S76" s="19" t="n"/>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="15" t="inlineStr">
@@ -3261,7 +3358,7 @@
         </is>
       </c>
       <c r="B77" s="16">
-        <f>IF(COUNTA(C77:R77)=0,"",IF(AND(C77&lt;&gt;"",D77&lt;&gt;"",E77&lt;&gt;"",H77&lt;&gt;"",I77&lt;&gt;"",NOT(AND(LEFT(I77,7)="Sale de",J77="",K77=""))),"✔ Completa","Falta: "&amp;IF(C77="","fecha · ","")&amp;IF(D77="","ubicación · ","")&amp;IF(E77="","referencia · ","")&amp;IF(H77="","criticidad · ","")&amp;IF(I77="","origen del agua · ","")&amp;IF(AND(LEFT(I77,7)="Sale de",J77="",K77=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C77:S77)=0,"",IF(AND(C77&lt;&gt;"",D77&lt;&gt;"",E77&lt;&gt;"",H77&lt;&gt;"",I77&lt;&gt;"",NOT(AND(LEFT(I77,7)="Sale de",J77="",K77=""))),"✔ Completa","Falta: "&amp;IF(C77="","fecha · ","")&amp;IF(D77="","ubicación · ","")&amp;IF(E77="","referencia · ","")&amp;IF(H77="","criticidad · ","")&amp;IF(I77="","origen del agua · ","")&amp;IF(AND(LEFT(I77,7)="Sale de",J77="",K77=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C77" s="17" t="n"/>
@@ -3278,8 +3375,9 @@
       <c r="N77" s="21" t="n"/>
       <c r="O77" s="21" t="n"/>
       <c r="P77" s="21" t="n"/>
-      <c r="Q77" s="18" t="n"/>
-      <c r="R77" s="19" t="n"/>
+      <c r="Q77" s="21" t="n"/>
+      <c r="R77" s="18" t="n"/>
+      <c r="S77" s="19" t="n"/>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="15" t="inlineStr">
@@ -3288,7 +3386,7 @@
         </is>
       </c>
       <c r="B78" s="16">
-        <f>IF(COUNTA(C78:R78)=0,"",IF(AND(C78&lt;&gt;"",D78&lt;&gt;"",E78&lt;&gt;"",H78&lt;&gt;"",I78&lt;&gt;"",NOT(AND(LEFT(I78,7)="Sale de",J78="",K78=""))),"✔ Completa","Falta: "&amp;IF(C78="","fecha · ","")&amp;IF(D78="","ubicación · ","")&amp;IF(E78="","referencia · ","")&amp;IF(H78="","criticidad · ","")&amp;IF(I78="","origen del agua · ","")&amp;IF(AND(LEFT(I78,7)="Sale de",J78="",K78=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C78:S78)=0,"",IF(AND(C78&lt;&gt;"",D78&lt;&gt;"",E78&lt;&gt;"",H78&lt;&gt;"",I78&lt;&gt;"",NOT(AND(LEFT(I78,7)="Sale de",J78="",K78=""))),"✔ Completa","Falta: "&amp;IF(C78="","fecha · ","")&amp;IF(D78="","ubicación · ","")&amp;IF(E78="","referencia · ","")&amp;IF(H78="","criticidad · ","")&amp;IF(I78="","origen del agua · ","")&amp;IF(AND(LEFT(I78,7)="Sale de",J78="",K78=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C78" s="17" t="n"/>
@@ -3305,8 +3403,9 @@
       <c r="N78" s="21" t="n"/>
       <c r="O78" s="21" t="n"/>
       <c r="P78" s="21" t="n"/>
-      <c r="Q78" s="18" t="n"/>
-      <c r="R78" s="19" t="n"/>
+      <c r="Q78" s="21" t="n"/>
+      <c r="R78" s="18" t="n"/>
+      <c r="S78" s="19" t="n"/>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="15" t="inlineStr">
@@ -3315,7 +3414,7 @@
         </is>
       </c>
       <c r="B79" s="16">
-        <f>IF(COUNTA(C79:R79)=0,"",IF(AND(C79&lt;&gt;"",D79&lt;&gt;"",E79&lt;&gt;"",H79&lt;&gt;"",I79&lt;&gt;"",NOT(AND(LEFT(I79,7)="Sale de",J79="",K79=""))),"✔ Completa","Falta: "&amp;IF(C79="","fecha · ","")&amp;IF(D79="","ubicación · ","")&amp;IF(E79="","referencia · ","")&amp;IF(H79="","criticidad · ","")&amp;IF(I79="","origen del agua · ","")&amp;IF(AND(LEFT(I79,7)="Sale de",J79="",K79=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C79:S79)=0,"",IF(AND(C79&lt;&gt;"",D79&lt;&gt;"",E79&lt;&gt;"",H79&lt;&gt;"",I79&lt;&gt;"",NOT(AND(LEFT(I79,7)="Sale de",J79="",K79=""))),"✔ Completa","Falta: "&amp;IF(C79="","fecha · ","")&amp;IF(D79="","ubicación · ","")&amp;IF(E79="","referencia · ","")&amp;IF(H79="","criticidad · ","")&amp;IF(I79="","origen del agua · ","")&amp;IF(AND(LEFT(I79,7)="Sale de",J79="",K79=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C79" s="17" t="n"/>
@@ -3332,8 +3431,9 @@
       <c r="N79" s="21" t="n"/>
       <c r="O79" s="21" t="n"/>
       <c r="P79" s="21" t="n"/>
-      <c r="Q79" s="18" t="n"/>
-      <c r="R79" s="19" t="n"/>
+      <c r="Q79" s="21" t="n"/>
+      <c r="R79" s="18" t="n"/>
+      <c r="S79" s="19" t="n"/>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="15" t="inlineStr">
@@ -3342,7 +3442,7 @@
         </is>
       </c>
       <c r="B80" s="16">
-        <f>IF(COUNTA(C80:R80)=0,"",IF(AND(C80&lt;&gt;"",D80&lt;&gt;"",E80&lt;&gt;"",H80&lt;&gt;"",I80&lt;&gt;"",NOT(AND(LEFT(I80,7)="Sale de",J80="",K80=""))),"✔ Completa","Falta: "&amp;IF(C80="","fecha · ","")&amp;IF(D80="","ubicación · ","")&amp;IF(E80="","referencia · ","")&amp;IF(H80="","criticidad · ","")&amp;IF(I80="","origen del agua · ","")&amp;IF(AND(LEFT(I80,7)="Sale de",J80="",K80=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C80:S80)=0,"",IF(AND(C80&lt;&gt;"",D80&lt;&gt;"",E80&lt;&gt;"",H80&lt;&gt;"",I80&lt;&gt;"",NOT(AND(LEFT(I80,7)="Sale de",J80="",K80=""))),"✔ Completa","Falta: "&amp;IF(C80="","fecha · ","")&amp;IF(D80="","ubicación · ","")&amp;IF(E80="","referencia · ","")&amp;IF(H80="","criticidad · ","")&amp;IF(I80="","origen del agua · ","")&amp;IF(AND(LEFT(I80,7)="Sale de",J80="",K80=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C80" s="17" t="n"/>
@@ -3359,8 +3459,9 @@
       <c r="N80" s="21" t="n"/>
       <c r="O80" s="21" t="n"/>
       <c r="P80" s="21" t="n"/>
-      <c r="Q80" s="18" t="n"/>
-      <c r="R80" s="19" t="n"/>
+      <c r="Q80" s="21" t="n"/>
+      <c r="R80" s="18" t="n"/>
+      <c r="S80" s="19" t="n"/>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="15" t="inlineStr">
@@ -3369,7 +3470,7 @@
         </is>
       </c>
       <c r="B81" s="16">
-        <f>IF(COUNTA(C81:R81)=0,"",IF(AND(C81&lt;&gt;"",D81&lt;&gt;"",E81&lt;&gt;"",H81&lt;&gt;"",I81&lt;&gt;"",NOT(AND(LEFT(I81,7)="Sale de",J81="",K81=""))),"✔ Completa","Falta: "&amp;IF(C81="","fecha · ","")&amp;IF(D81="","ubicación · ","")&amp;IF(E81="","referencia · ","")&amp;IF(H81="","criticidad · ","")&amp;IF(I81="","origen del agua · ","")&amp;IF(AND(LEFT(I81,7)="Sale de",J81="",K81=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C81:S81)=0,"",IF(AND(C81&lt;&gt;"",D81&lt;&gt;"",E81&lt;&gt;"",H81&lt;&gt;"",I81&lt;&gt;"",NOT(AND(LEFT(I81,7)="Sale de",J81="",K81=""))),"✔ Completa","Falta: "&amp;IF(C81="","fecha · ","")&amp;IF(D81="","ubicación · ","")&amp;IF(E81="","referencia · ","")&amp;IF(H81="","criticidad · ","")&amp;IF(I81="","origen del agua · ","")&amp;IF(AND(LEFT(I81,7)="Sale de",J81="",K81=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C81" s="17" t="n"/>
@@ -3386,8 +3487,9 @@
       <c r="N81" s="21" t="n"/>
       <c r="O81" s="21" t="n"/>
       <c r="P81" s="21" t="n"/>
-      <c r="Q81" s="18" t="n"/>
-      <c r="R81" s="19" t="n"/>
+      <c r="Q81" s="21" t="n"/>
+      <c r="R81" s="18" t="n"/>
+      <c r="S81" s="19" t="n"/>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="15" t="inlineStr">
@@ -3396,7 +3498,7 @@
         </is>
       </c>
       <c r="B82" s="16">
-        <f>IF(COUNTA(C82:R82)=0,"",IF(AND(C82&lt;&gt;"",D82&lt;&gt;"",E82&lt;&gt;"",H82&lt;&gt;"",I82&lt;&gt;"",NOT(AND(LEFT(I82,7)="Sale de",J82="",K82=""))),"✔ Completa","Falta: "&amp;IF(C82="","fecha · ","")&amp;IF(D82="","ubicación · ","")&amp;IF(E82="","referencia · ","")&amp;IF(H82="","criticidad · ","")&amp;IF(I82="","origen del agua · ","")&amp;IF(AND(LEFT(I82,7)="Sale de",J82="",K82=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C82:S82)=0,"",IF(AND(C82&lt;&gt;"",D82&lt;&gt;"",E82&lt;&gt;"",H82&lt;&gt;"",I82&lt;&gt;"",NOT(AND(LEFT(I82,7)="Sale de",J82="",K82=""))),"✔ Completa","Falta: "&amp;IF(C82="","fecha · ","")&amp;IF(D82="","ubicación · ","")&amp;IF(E82="","referencia · ","")&amp;IF(H82="","criticidad · ","")&amp;IF(I82="","origen del agua · ","")&amp;IF(AND(LEFT(I82,7)="Sale de",J82="",K82=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C82" s="17" t="n"/>
@@ -3413,8 +3515,9 @@
       <c r="N82" s="21" t="n"/>
       <c r="O82" s="21" t="n"/>
       <c r="P82" s="21" t="n"/>
-      <c r="Q82" s="18" t="n"/>
-      <c r="R82" s="19" t="n"/>
+      <c r="Q82" s="21" t="n"/>
+      <c r="R82" s="18" t="n"/>
+      <c r="S82" s="19" t="n"/>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="15" t="inlineStr">
@@ -3423,7 +3526,7 @@
         </is>
       </c>
       <c r="B83" s="16">
-        <f>IF(COUNTA(C83:R83)=0,"",IF(AND(C83&lt;&gt;"",D83&lt;&gt;"",E83&lt;&gt;"",H83&lt;&gt;"",I83&lt;&gt;"",NOT(AND(LEFT(I83,7)="Sale de",J83="",K83=""))),"✔ Completa","Falta: "&amp;IF(C83="","fecha · ","")&amp;IF(D83="","ubicación · ","")&amp;IF(E83="","referencia · ","")&amp;IF(H83="","criticidad · ","")&amp;IF(I83="","origen del agua · ","")&amp;IF(AND(LEFT(I83,7)="Sale de",J83="",K83=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C83:S83)=0,"",IF(AND(C83&lt;&gt;"",D83&lt;&gt;"",E83&lt;&gt;"",H83&lt;&gt;"",I83&lt;&gt;"",NOT(AND(LEFT(I83,7)="Sale de",J83="",K83=""))),"✔ Completa","Falta: "&amp;IF(C83="","fecha · ","")&amp;IF(D83="","ubicación · ","")&amp;IF(E83="","referencia · ","")&amp;IF(H83="","criticidad · ","")&amp;IF(I83="","origen del agua · ","")&amp;IF(AND(LEFT(I83,7)="Sale de",J83="",K83=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C83" s="17" t="n"/>
@@ -3440,8 +3543,9 @@
       <c r="N83" s="21" t="n"/>
       <c r="O83" s="21" t="n"/>
       <c r="P83" s="21" t="n"/>
-      <c r="Q83" s="18" t="n"/>
-      <c r="R83" s="19" t="n"/>
+      <c r="Q83" s="21" t="n"/>
+      <c r="R83" s="18" t="n"/>
+      <c r="S83" s="19" t="n"/>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="15" t="inlineStr">
@@ -3450,7 +3554,7 @@
         </is>
       </c>
       <c r="B84" s="16">
-        <f>IF(COUNTA(C84:R84)=0,"",IF(AND(C84&lt;&gt;"",D84&lt;&gt;"",E84&lt;&gt;"",H84&lt;&gt;"",I84&lt;&gt;"",NOT(AND(LEFT(I84,7)="Sale de",J84="",K84=""))),"✔ Completa","Falta: "&amp;IF(C84="","fecha · ","")&amp;IF(D84="","ubicación · ","")&amp;IF(E84="","referencia · ","")&amp;IF(H84="","criticidad · ","")&amp;IF(I84="","origen del agua · ","")&amp;IF(AND(LEFT(I84,7)="Sale de",J84="",K84=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C84:S84)=0,"",IF(AND(C84&lt;&gt;"",D84&lt;&gt;"",E84&lt;&gt;"",H84&lt;&gt;"",I84&lt;&gt;"",NOT(AND(LEFT(I84,7)="Sale de",J84="",K84=""))),"✔ Completa","Falta: "&amp;IF(C84="","fecha · ","")&amp;IF(D84="","ubicación · ","")&amp;IF(E84="","referencia · ","")&amp;IF(H84="","criticidad · ","")&amp;IF(I84="","origen del agua · ","")&amp;IF(AND(LEFT(I84,7)="Sale de",J84="",K84=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C84" s="17" t="n"/>
@@ -3467,8 +3571,9 @@
       <c r="N84" s="21" t="n"/>
       <c r="O84" s="21" t="n"/>
       <c r="P84" s="21" t="n"/>
-      <c r="Q84" s="18" t="n"/>
-      <c r="R84" s="19" t="n"/>
+      <c r="Q84" s="21" t="n"/>
+      <c r="R84" s="18" t="n"/>
+      <c r="S84" s="19" t="n"/>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="15" t="inlineStr">
@@ -3477,7 +3582,7 @@
         </is>
       </c>
       <c r="B85" s="16">
-        <f>IF(COUNTA(C85:R85)=0,"",IF(AND(C85&lt;&gt;"",D85&lt;&gt;"",E85&lt;&gt;"",H85&lt;&gt;"",I85&lt;&gt;"",NOT(AND(LEFT(I85,7)="Sale de",J85="",K85=""))),"✔ Completa","Falta: "&amp;IF(C85="","fecha · ","")&amp;IF(D85="","ubicación · ","")&amp;IF(E85="","referencia · ","")&amp;IF(H85="","criticidad · ","")&amp;IF(I85="","origen del agua · ","")&amp;IF(AND(LEFT(I85,7)="Sale de",J85="",K85=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C85:S85)=0,"",IF(AND(C85&lt;&gt;"",D85&lt;&gt;"",E85&lt;&gt;"",H85&lt;&gt;"",I85&lt;&gt;"",NOT(AND(LEFT(I85,7)="Sale de",J85="",K85=""))),"✔ Completa","Falta: "&amp;IF(C85="","fecha · ","")&amp;IF(D85="","ubicación · ","")&amp;IF(E85="","referencia · ","")&amp;IF(H85="","criticidad · ","")&amp;IF(I85="","origen del agua · ","")&amp;IF(AND(LEFT(I85,7)="Sale de",J85="",K85=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C85" s="17" t="n"/>
@@ -3494,8 +3599,9 @@
       <c r="N85" s="21" t="n"/>
       <c r="O85" s="21" t="n"/>
       <c r="P85" s="21" t="n"/>
-      <c r="Q85" s="18" t="n"/>
-      <c r="R85" s="19" t="n"/>
+      <c r="Q85" s="21" t="n"/>
+      <c r="R85" s="18" t="n"/>
+      <c r="S85" s="19" t="n"/>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="15" t="inlineStr">
@@ -3504,7 +3610,7 @@
         </is>
       </c>
       <c r="B86" s="16">
-        <f>IF(COUNTA(C86:R86)=0,"",IF(AND(C86&lt;&gt;"",D86&lt;&gt;"",E86&lt;&gt;"",H86&lt;&gt;"",I86&lt;&gt;"",NOT(AND(LEFT(I86,7)="Sale de",J86="",K86=""))),"✔ Completa","Falta: "&amp;IF(C86="","fecha · ","")&amp;IF(D86="","ubicación · ","")&amp;IF(E86="","referencia · ","")&amp;IF(H86="","criticidad · ","")&amp;IF(I86="","origen del agua · ","")&amp;IF(AND(LEFT(I86,7)="Sale de",J86="",K86=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C86:S86)=0,"",IF(AND(C86&lt;&gt;"",D86&lt;&gt;"",E86&lt;&gt;"",H86&lt;&gt;"",I86&lt;&gt;"",NOT(AND(LEFT(I86,7)="Sale de",J86="",K86=""))),"✔ Completa","Falta: "&amp;IF(C86="","fecha · ","")&amp;IF(D86="","ubicación · ","")&amp;IF(E86="","referencia · ","")&amp;IF(H86="","criticidad · ","")&amp;IF(I86="","origen del agua · ","")&amp;IF(AND(LEFT(I86,7)="Sale de",J86="",K86=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C86" s="17" t="n"/>
@@ -3521,8 +3627,9 @@
       <c r="N86" s="21" t="n"/>
       <c r="O86" s="21" t="n"/>
       <c r="P86" s="21" t="n"/>
-      <c r="Q86" s="18" t="n"/>
-      <c r="R86" s="19" t="n"/>
+      <c r="Q86" s="21" t="n"/>
+      <c r="R86" s="18" t="n"/>
+      <c r="S86" s="19" t="n"/>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="15" t="inlineStr">
@@ -3531,7 +3638,7 @@
         </is>
       </c>
       <c r="B87" s="16">
-        <f>IF(COUNTA(C87:R87)=0,"",IF(AND(C87&lt;&gt;"",D87&lt;&gt;"",E87&lt;&gt;"",H87&lt;&gt;"",I87&lt;&gt;"",NOT(AND(LEFT(I87,7)="Sale de",J87="",K87=""))),"✔ Completa","Falta: "&amp;IF(C87="","fecha · ","")&amp;IF(D87="","ubicación · ","")&amp;IF(E87="","referencia · ","")&amp;IF(H87="","criticidad · ","")&amp;IF(I87="","origen del agua · ","")&amp;IF(AND(LEFT(I87,7)="Sale de",J87="",K87=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C87:S87)=0,"",IF(AND(C87&lt;&gt;"",D87&lt;&gt;"",E87&lt;&gt;"",H87&lt;&gt;"",I87&lt;&gt;"",NOT(AND(LEFT(I87,7)="Sale de",J87="",K87=""))),"✔ Completa","Falta: "&amp;IF(C87="","fecha · ","")&amp;IF(D87="","ubicación · ","")&amp;IF(E87="","referencia · ","")&amp;IF(H87="","criticidad · ","")&amp;IF(I87="","origen del agua · ","")&amp;IF(AND(LEFT(I87,7)="Sale de",J87="",K87=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C87" s="17" t="n"/>
@@ -3548,8 +3655,9 @@
       <c r="N87" s="21" t="n"/>
       <c r="O87" s="21" t="n"/>
       <c r="P87" s="21" t="n"/>
-      <c r="Q87" s="18" t="n"/>
-      <c r="R87" s="19" t="n"/>
+      <c r="Q87" s="21" t="n"/>
+      <c r="R87" s="18" t="n"/>
+      <c r="S87" s="19" t="n"/>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="15" t="inlineStr">
@@ -3558,7 +3666,7 @@
         </is>
       </c>
       <c r="B88" s="16">
-        <f>IF(COUNTA(C88:R88)=0,"",IF(AND(C88&lt;&gt;"",D88&lt;&gt;"",E88&lt;&gt;"",H88&lt;&gt;"",I88&lt;&gt;"",NOT(AND(LEFT(I88,7)="Sale de",J88="",K88=""))),"✔ Completa","Falta: "&amp;IF(C88="","fecha · ","")&amp;IF(D88="","ubicación · ","")&amp;IF(E88="","referencia · ","")&amp;IF(H88="","criticidad · ","")&amp;IF(I88="","origen del agua · ","")&amp;IF(AND(LEFT(I88,7)="Sale de",J88="",K88=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C88:S88)=0,"",IF(AND(C88&lt;&gt;"",D88&lt;&gt;"",E88&lt;&gt;"",H88&lt;&gt;"",I88&lt;&gt;"",NOT(AND(LEFT(I88,7)="Sale de",J88="",K88=""))),"✔ Completa","Falta: "&amp;IF(C88="","fecha · ","")&amp;IF(D88="","ubicación · ","")&amp;IF(E88="","referencia · ","")&amp;IF(H88="","criticidad · ","")&amp;IF(I88="","origen del agua · ","")&amp;IF(AND(LEFT(I88,7)="Sale de",J88="",K88=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C88" s="17" t="n"/>
@@ -3575,8 +3683,9 @@
       <c r="N88" s="21" t="n"/>
       <c r="O88" s="21" t="n"/>
       <c r="P88" s="21" t="n"/>
-      <c r="Q88" s="18" t="n"/>
-      <c r="R88" s="19" t="n"/>
+      <c r="Q88" s="21" t="n"/>
+      <c r="R88" s="18" t="n"/>
+      <c r="S88" s="19" t="n"/>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="15" t="inlineStr">
@@ -3585,7 +3694,7 @@
         </is>
       </c>
       <c r="B89" s="16">
-        <f>IF(COUNTA(C89:R89)=0,"",IF(AND(C89&lt;&gt;"",D89&lt;&gt;"",E89&lt;&gt;"",H89&lt;&gt;"",I89&lt;&gt;"",NOT(AND(LEFT(I89,7)="Sale de",J89="",K89=""))),"✔ Completa","Falta: "&amp;IF(C89="","fecha · ","")&amp;IF(D89="","ubicación · ","")&amp;IF(E89="","referencia · ","")&amp;IF(H89="","criticidad · ","")&amp;IF(I89="","origen del agua · ","")&amp;IF(AND(LEFT(I89,7)="Sale de",J89="",K89=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C89:S89)=0,"",IF(AND(C89&lt;&gt;"",D89&lt;&gt;"",E89&lt;&gt;"",H89&lt;&gt;"",I89&lt;&gt;"",NOT(AND(LEFT(I89,7)="Sale de",J89="",K89=""))),"✔ Completa","Falta: "&amp;IF(C89="","fecha · ","")&amp;IF(D89="","ubicación · ","")&amp;IF(E89="","referencia · ","")&amp;IF(H89="","criticidad · ","")&amp;IF(I89="","origen del agua · ","")&amp;IF(AND(LEFT(I89,7)="Sale de",J89="",K89=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C89" s="17" t="n"/>
@@ -3602,8 +3711,9 @@
       <c r="N89" s="21" t="n"/>
       <c r="O89" s="21" t="n"/>
       <c r="P89" s="21" t="n"/>
-      <c r="Q89" s="18" t="n"/>
-      <c r="R89" s="19" t="n"/>
+      <c r="Q89" s="21" t="n"/>
+      <c r="R89" s="18" t="n"/>
+      <c r="S89" s="19" t="n"/>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="15" t="inlineStr">
@@ -3612,7 +3722,7 @@
         </is>
       </c>
       <c r="B90" s="16">
-        <f>IF(COUNTA(C90:R90)=0,"",IF(AND(C90&lt;&gt;"",D90&lt;&gt;"",E90&lt;&gt;"",H90&lt;&gt;"",I90&lt;&gt;"",NOT(AND(LEFT(I90,7)="Sale de",J90="",K90=""))),"✔ Completa","Falta: "&amp;IF(C90="","fecha · ","")&amp;IF(D90="","ubicación · ","")&amp;IF(E90="","referencia · ","")&amp;IF(H90="","criticidad · ","")&amp;IF(I90="","origen del agua · ","")&amp;IF(AND(LEFT(I90,7)="Sale de",J90="",K90=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C90:S90)=0,"",IF(AND(C90&lt;&gt;"",D90&lt;&gt;"",E90&lt;&gt;"",H90&lt;&gt;"",I90&lt;&gt;"",NOT(AND(LEFT(I90,7)="Sale de",J90="",K90=""))),"✔ Completa","Falta: "&amp;IF(C90="","fecha · ","")&amp;IF(D90="","ubicación · ","")&amp;IF(E90="","referencia · ","")&amp;IF(H90="","criticidad · ","")&amp;IF(I90="","origen del agua · ","")&amp;IF(AND(LEFT(I90,7)="Sale de",J90="",K90=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C90" s="17" t="n"/>
@@ -3629,8 +3739,9 @@
       <c r="N90" s="21" t="n"/>
       <c r="O90" s="21" t="n"/>
       <c r="P90" s="21" t="n"/>
-      <c r="Q90" s="18" t="n"/>
-      <c r="R90" s="19" t="n"/>
+      <c r="Q90" s="21" t="n"/>
+      <c r="R90" s="18" t="n"/>
+      <c r="S90" s="19" t="n"/>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="15" t="inlineStr">
@@ -3639,7 +3750,7 @@
         </is>
       </c>
       <c r="B91" s="16">
-        <f>IF(COUNTA(C91:R91)=0,"",IF(AND(C91&lt;&gt;"",D91&lt;&gt;"",E91&lt;&gt;"",H91&lt;&gt;"",I91&lt;&gt;"",NOT(AND(LEFT(I91,7)="Sale de",J91="",K91=""))),"✔ Completa","Falta: "&amp;IF(C91="","fecha · ","")&amp;IF(D91="","ubicación · ","")&amp;IF(E91="","referencia · ","")&amp;IF(H91="","criticidad · ","")&amp;IF(I91="","origen del agua · ","")&amp;IF(AND(LEFT(I91,7)="Sale de",J91="",K91=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C91:S91)=0,"",IF(AND(C91&lt;&gt;"",D91&lt;&gt;"",E91&lt;&gt;"",H91&lt;&gt;"",I91&lt;&gt;"",NOT(AND(LEFT(I91,7)="Sale de",J91="",K91=""))),"✔ Completa","Falta: "&amp;IF(C91="","fecha · ","")&amp;IF(D91="","ubicación · ","")&amp;IF(E91="","referencia · ","")&amp;IF(H91="","criticidad · ","")&amp;IF(I91="","origen del agua · ","")&amp;IF(AND(LEFT(I91,7)="Sale de",J91="",K91=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C91" s="17" t="n"/>
@@ -3656,8 +3767,9 @@
       <c r="N91" s="21" t="n"/>
       <c r="O91" s="21" t="n"/>
       <c r="P91" s="21" t="n"/>
-      <c r="Q91" s="18" t="n"/>
-      <c r="R91" s="19" t="n"/>
+      <c r="Q91" s="21" t="n"/>
+      <c r="R91" s="18" t="n"/>
+      <c r="S91" s="19" t="n"/>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="15" t="inlineStr">
@@ -3666,7 +3778,7 @@
         </is>
       </c>
       <c r="B92" s="16">
-        <f>IF(COUNTA(C92:R92)=0,"",IF(AND(C92&lt;&gt;"",D92&lt;&gt;"",E92&lt;&gt;"",H92&lt;&gt;"",I92&lt;&gt;"",NOT(AND(LEFT(I92,7)="Sale de",J92="",K92=""))),"✔ Completa","Falta: "&amp;IF(C92="","fecha · ","")&amp;IF(D92="","ubicación · ","")&amp;IF(E92="","referencia · ","")&amp;IF(H92="","criticidad · ","")&amp;IF(I92="","origen del agua · ","")&amp;IF(AND(LEFT(I92,7)="Sale de",J92="",K92=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C92:S92)=0,"",IF(AND(C92&lt;&gt;"",D92&lt;&gt;"",E92&lt;&gt;"",H92&lt;&gt;"",I92&lt;&gt;"",NOT(AND(LEFT(I92,7)="Sale de",J92="",K92=""))),"✔ Completa","Falta: "&amp;IF(C92="","fecha · ","")&amp;IF(D92="","ubicación · ","")&amp;IF(E92="","referencia · ","")&amp;IF(H92="","criticidad · ","")&amp;IF(I92="","origen del agua · ","")&amp;IF(AND(LEFT(I92,7)="Sale de",J92="",K92=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C92" s="17" t="n"/>
@@ -3683,8 +3795,9 @@
       <c r="N92" s="21" t="n"/>
       <c r="O92" s="21" t="n"/>
       <c r="P92" s="21" t="n"/>
-      <c r="Q92" s="18" t="n"/>
-      <c r="R92" s="19" t="n"/>
+      <c r="Q92" s="21" t="n"/>
+      <c r="R92" s="18" t="n"/>
+      <c r="S92" s="19" t="n"/>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="15" t="inlineStr">
@@ -3693,7 +3806,7 @@
         </is>
       </c>
       <c r="B93" s="16">
-        <f>IF(COUNTA(C93:R93)=0,"",IF(AND(C93&lt;&gt;"",D93&lt;&gt;"",E93&lt;&gt;"",H93&lt;&gt;"",I93&lt;&gt;"",NOT(AND(LEFT(I93,7)="Sale de",J93="",K93=""))),"✔ Completa","Falta: "&amp;IF(C93="","fecha · ","")&amp;IF(D93="","ubicación · ","")&amp;IF(E93="","referencia · ","")&amp;IF(H93="","criticidad · ","")&amp;IF(I93="","origen del agua · ","")&amp;IF(AND(LEFT(I93,7)="Sale de",J93="",K93=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C93:S93)=0,"",IF(AND(C93&lt;&gt;"",D93&lt;&gt;"",E93&lt;&gt;"",H93&lt;&gt;"",I93&lt;&gt;"",NOT(AND(LEFT(I93,7)="Sale de",J93="",K93=""))),"✔ Completa","Falta: "&amp;IF(C93="","fecha · ","")&amp;IF(D93="","ubicación · ","")&amp;IF(E93="","referencia · ","")&amp;IF(H93="","criticidad · ","")&amp;IF(I93="","origen del agua · ","")&amp;IF(AND(LEFT(I93,7)="Sale de",J93="",K93=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C93" s="17" t="n"/>
@@ -3710,8 +3823,9 @@
       <c r="N93" s="21" t="n"/>
       <c r="O93" s="21" t="n"/>
       <c r="P93" s="21" t="n"/>
-      <c r="Q93" s="18" t="n"/>
-      <c r="R93" s="19" t="n"/>
+      <c r="Q93" s="21" t="n"/>
+      <c r="R93" s="18" t="n"/>
+      <c r="S93" s="19" t="n"/>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="15" t="inlineStr">
@@ -3720,7 +3834,7 @@
         </is>
       </c>
       <c r="B94" s="16">
-        <f>IF(COUNTA(C94:R94)=0,"",IF(AND(C94&lt;&gt;"",D94&lt;&gt;"",E94&lt;&gt;"",H94&lt;&gt;"",I94&lt;&gt;"",NOT(AND(LEFT(I94,7)="Sale de",J94="",K94=""))),"✔ Completa","Falta: "&amp;IF(C94="","fecha · ","")&amp;IF(D94="","ubicación · ","")&amp;IF(E94="","referencia · ","")&amp;IF(H94="","criticidad · ","")&amp;IF(I94="","origen del agua · ","")&amp;IF(AND(LEFT(I94,7)="Sale de",J94="",K94=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C94:S94)=0,"",IF(AND(C94&lt;&gt;"",D94&lt;&gt;"",E94&lt;&gt;"",H94&lt;&gt;"",I94&lt;&gt;"",NOT(AND(LEFT(I94,7)="Sale de",J94="",K94=""))),"✔ Completa","Falta: "&amp;IF(C94="","fecha · ","")&amp;IF(D94="","ubicación · ","")&amp;IF(E94="","referencia · ","")&amp;IF(H94="","criticidad · ","")&amp;IF(I94="","origen del agua · ","")&amp;IF(AND(LEFT(I94,7)="Sale de",J94="",K94=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C94" s="17" t="n"/>
@@ -3737,8 +3851,9 @@
       <c r="N94" s="21" t="n"/>
       <c r="O94" s="21" t="n"/>
       <c r="P94" s="21" t="n"/>
-      <c r="Q94" s="18" t="n"/>
-      <c r="R94" s="19" t="n"/>
+      <c r="Q94" s="21" t="n"/>
+      <c r="R94" s="18" t="n"/>
+      <c r="S94" s="19" t="n"/>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="15" t="inlineStr">
@@ -3747,7 +3862,7 @@
         </is>
       </c>
       <c r="B95" s="16">
-        <f>IF(COUNTA(C95:R95)=0,"",IF(AND(C95&lt;&gt;"",D95&lt;&gt;"",E95&lt;&gt;"",H95&lt;&gt;"",I95&lt;&gt;"",NOT(AND(LEFT(I95,7)="Sale de",J95="",K95=""))),"✔ Completa","Falta: "&amp;IF(C95="","fecha · ","")&amp;IF(D95="","ubicación · ","")&amp;IF(E95="","referencia · ","")&amp;IF(H95="","criticidad · ","")&amp;IF(I95="","origen del agua · ","")&amp;IF(AND(LEFT(I95,7)="Sale de",J95="",K95=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C95:S95)=0,"",IF(AND(C95&lt;&gt;"",D95&lt;&gt;"",E95&lt;&gt;"",H95&lt;&gt;"",I95&lt;&gt;"",NOT(AND(LEFT(I95,7)="Sale de",J95="",K95=""))),"✔ Completa","Falta: "&amp;IF(C95="","fecha · ","")&amp;IF(D95="","ubicación · ","")&amp;IF(E95="","referencia · ","")&amp;IF(H95="","criticidad · ","")&amp;IF(I95="","origen del agua · ","")&amp;IF(AND(LEFT(I95,7)="Sale de",J95="",K95=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C95" s="17" t="n"/>
@@ -3764,8 +3879,9 @@
       <c r="N95" s="21" t="n"/>
       <c r="O95" s="21" t="n"/>
       <c r="P95" s="21" t="n"/>
-      <c r="Q95" s="18" t="n"/>
-      <c r="R95" s="19" t="n"/>
+      <c r="Q95" s="21" t="n"/>
+      <c r="R95" s="18" t="n"/>
+      <c r="S95" s="19" t="n"/>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="15" t="inlineStr">
@@ -3774,7 +3890,7 @@
         </is>
       </c>
       <c r="B96" s="16">
-        <f>IF(COUNTA(C96:R96)=0,"",IF(AND(C96&lt;&gt;"",D96&lt;&gt;"",E96&lt;&gt;"",H96&lt;&gt;"",I96&lt;&gt;"",NOT(AND(LEFT(I96,7)="Sale de",J96="",K96=""))),"✔ Completa","Falta: "&amp;IF(C96="","fecha · ","")&amp;IF(D96="","ubicación · ","")&amp;IF(E96="","referencia · ","")&amp;IF(H96="","criticidad · ","")&amp;IF(I96="","origen del agua · ","")&amp;IF(AND(LEFT(I96,7)="Sale de",J96="",K96=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C96:S96)=0,"",IF(AND(C96&lt;&gt;"",D96&lt;&gt;"",E96&lt;&gt;"",H96&lt;&gt;"",I96&lt;&gt;"",NOT(AND(LEFT(I96,7)="Sale de",J96="",K96=""))),"✔ Completa","Falta: "&amp;IF(C96="","fecha · ","")&amp;IF(D96="","ubicación · ","")&amp;IF(E96="","referencia · ","")&amp;IF(H96="","criticidad · ","")&amp;IF(I96="","origen del agua · ","")&amp;IF(AND(LEFT(I96,7)="Sale de",J96="",K96=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C96" s="17" t="n"/>
@@ -3791,8 +3907,9 @@
       <c r="N96" s="21" t="n"/>
       <c r="O96" s="21" t="n"/>
       <c r="P96" s="21" t="n"/>
-      <c r="Q96" s="18" t="n"/>
-      <c r="R96" s="19" t="n"/>
+      <c r="Q96" s="21" t="n"/>
+      <c r="R96" s="18" t="n"/>
+      <c r="S96" s="19" t="n"/>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="15" t="inlineStr">
@@ -3801,7 +3918,7 @@
         </is>
       </c>
       <c r="B97" s="16">
-        <f>IF(COUNTA(C97:R97)=0,"",IF(AND(C97&lt;&gt;"",D97&lt;&gt;"",E97&lt;&gt;"",H97&lt;&gt;"",I97&lt;&gt;"",NOT(AND(LEFT(I97,7)="Sale de",J97="",K97=""))),"✔ Completa","Falta: "&amp;IF(C97="","fecha · ","")&amp;IF(D97="","ubicación · ","")&amp;IF(E97="","referencia · ","")&amp;IF(H97="","criticidad · ","")&amp;IF(I97="","origen del agua · ","")&amp;IF(AND(LEFT(I97,7)="Sale de",J97="",K97=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C97:S97)=0,"",IF(AND(C97&lt;&gt;"",D97&lt;&gt;"",E97&lt;&gt;"",H97&lt;&gt;"",I97&lt;&gt;"",NOT(AND(LEFT(I97,7)="Sale de",J97="",K97=""))),"✔ Completa","Falta: "&amp;IF(C97="","fecha · ","")&amp;IF(D97="","ubicación · ","")&amp;IF(E97="","referencia · ","")&amp;IF(H97="","criticidad · ","")&amp;IF(I97="","origen del agua · ","")&amp;IF(AND(LEFT(I97,7)="Sale de",J97="",K97=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C97" s="17" t="n"/>
@@ -3818,8 +3935,9 @@
       <c r="N97" s="21" t="n"/>
       <c r="O97" s="21" t="n"/>
       <c r="P97" s="21" t="n"/>
-      <c r="Q97" s="18" t="n"/>
-      <c r="R97" s="19" t="n"/>
+      <c r="Q97" s="21" t="n"/>
+      <c r="R97" s="18" t="n"/>
+      <c r="S97" s="19" t="n"/>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="15" t="inlineStr">
@@ -3828,7 +3946,7 @@
         </is>
       </c>
       <c r="B98" s="16">
-        <f>IF(COUNTA(C98:R98)=0,"",IF(AND(C98&lt;&gt;"",D98&lt;&gt;"",E98&lt;&gt;"",H98&lt;&gt;"",I98&lt;&gt;"",NOT(AND(LEFT(I98,7)="Sale de",J98="",K98=""))),"✔ Completa","Falta: "&amp;IF(C98="","fecha · ","")&amp;IF(D98="","ubicación · ","")&amp;IF(E98="","referencia · ","")&amp;IF(H98="","criticidad · ","")&amp;IF(I98="","origen del agua · ","")&amp;IF(AND(LEFT(I98,7)="Sale de",J98="",K98=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C98:S98)=0,"",IF(AND(C98&lt;&gt;"",D98&lt;&gt;"",E98&lt;&gt;"",H98&lt;&gt;"",I98&lt;&gt;"",NOT(AND(LEFT(I98,7)="Sale de",J98="",K98=""))),"✔ Completa","Falta: "&amp;IF(C98="","fecha · ","")&amp;IF(D98="","ubicación · ","")&amp;IF(E98="","referencia · ","")&amp;IF(H98="","criticidad · ","")&amp;IF(I98="","origen del agua · ","")&amp;IF(AND(LEFT(I98,7)="Sale de",J98="",K98=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C98" s="17" t="n"/>
@@ -3845,8 +3963,9 @@
       <c r="N98" s="21" t="n"/>
       <c r="O98" s="21" t="n"/>
       <c r="P98" s="21" t="n"/>
-      <c r="Q98" s="18" t="n"/>
-      <c r="R98" s="19" t="n"/>
+      <c r="Q98" s="21" t="n"/>
+      <c r="R98" s="18" t="n"/>
+      <c r="S98" s="19" t="n"/>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="15" t="inlineStr">
@@ -3855,7 +3974,7 @@
         </is>
       </c>
       <c r="B99" s="16">
-        <f>IF(COUNTA(C99:R99)=0,"",IF(AND(C99&lt;&gt;"",D99&lt;&gt;"",E99&lt;&gt;"",H99&lt;&gt;"",I99&lt;&gt;"",NOT(AND(LEFT(I99,7)="Sale de",J99="",K99=""))),"✔ Completa","Falta: "&amp;IF(C99="","fecha · ","")&amp;IF(D99="","ubicación · ","")&amp;IF(E99="","referencia · ","")&amp;IF(H99="","criticidad · ","")&amp;IF(I99="","origen del agua · ","")&amp;IF(AND(LEFT(I99,7)="Sale de",J99="",K99=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C99:S99)=0,"",IF(AND(C99&lt;&gt;"",D99&lt;&gt;"",E99&lt;&gt;"",H99&lt;&gt;"",I99&lt;&gt;"",NOT(AND(LEFT(I99,7)="Sale de",J99="",K99=""))),"✔ Completa","Falta: "&amp;IF(C99="","fecha · ","")&amp;IF(D99="","ubicación · ","")&amp;IF(E99="","referencia · ","")&amp;IF(H99="","criticidad · ","")&amp;IF(I99="","origen del agua · ","")&amp;IF(AND(LEFT(I99,7)="Sale de",J99="",K99=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C99" s="17" t="n"/>
@@ -3872,8 +3991,9 @@
       <c r="N99" s="21" t="n"/>
       <c r="O99" s="21" t="n"/>
       <c r="P99" s="21" t="n"/>
-      <c r="Q99" s="18" t="n"/>
-      <c r="R99" s="19" t="n"/>
+      <c r="Q99" s="21" t="n"/>
+      <c r="R99" s="18" t="n"/>
+      <c r="S99" s="19" t="n"/>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="15" t="inlineStr">
@@ -3882,7 +4002,7 @@
         </is>
       </c>
       <c r="B100" s="16">
-        <f>IF(COUNTA(C100:R100)=0,"",IF(AND(C100&lt;&gt;"",D100&lt;&gt;"",E100&lt;&gt;"",H100&lt;&gt;"",I100&lt;&gt;"",NOT(AND(LEFT(I100,7)="Sale de",J100="",K100=""))),"✔ Completa","Falta: "&amp;IF(C100="","fecha · ","")&amp;IF(D100="","ubicación · ","")&amp;IF(E100="","referencia · ","")&amp;IF(H100="","criticidad · ","")&amp;IF(I100="","origen del agua · ","")&amp;IF(AND(LEFT(I100,7)="Sale de",J100="",K100=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C100:S100)=0,"",IF(AND(C100&lt;&gt;"",D100&lt;&gt;"",E100&lt;&gt;"",H100&lt;&gt;"",I100&lt;&gt;"",NOT(AND(LEFT(I100,7)="Sale de",J100="",K100=""))),"✔ Completa","Falta: "&amp;IF(C100="","fecha · ","")&amp;IF(D100="","ubicación · ","")&amp;IF(E100="","referencia · ","")&amp;IF(H100="","criticidad · ","")&amp;IF(I100="","origen del agua · ","")&amp;IF(AND(LEFT(I100,7)="Sale de",J100="",K100=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C100" s="17" t="n"/>
@@ -3899,8 +4019,9 @@
       <c r="N100" s="21" t="n"/>
       <c r="O100" s="21" t="n"/>
       <c r="P100" s="21" t="n"/>
-      <c r="Q100" s="18" t="n"/>
-      <c r="R100" s="19" t="n"/>
+      <c r="Q100" s="21" t="n"/>
+      <c r="R100" s="18" t="n"/>
+      <c r="S100" s="19" t="n"/>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="15" t="inlineStr">
@@ -3909,7 +4030,7 @@
         </is>
       </c>
       <c r="B101" s="16">
-        <f>IF(COUNTA(C101:R101)=0,"",IF(AND(C101&lt;&gt;"",D101&lt;&gt;"",E101&lt;&gt;"",H101&lt;&gt;"",I101&lt;&gt;"",NOT(AND(LEFT(I101,7)="Sale de",J101="",K101=""))),"✔ Completa","Falta: "&amp;IF(C101="","fecha · ","")&amp;IF(D101="","ubicación · ","")&amp;IF(E101="","referencia · ","")&amp;IF(H101="","criticidad · ","")&amp;IF(I101="","origen del agua · ","")&amp;IF(AND(LEFT(I101,7)="Sale de",J101="",K101=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C101:S101)=0,"",IF(AND(C101&lt;&gt;"",D101&lt;&gt;"",E101&lt;&gt;"",H101&lt;&gt;"",I101&lt;&gt;"",NOT(AND(LEFT(I101,7)="Sale de",J101="",K101=""))),"✔ Completa","Falta: "&amp;IF(C101="","fecha · ","")&amp;IF(D101="","ubicación · ","")&amp;IF(E101="","referencia · ","")&amp;IF(H101="","criticidad · ","")&amp;IF(I101="","origen del agua · ","")&amp;IF(AND(LEFT(I101,7)="Sale de",J101="",K101=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C101" s="17" t="n"/>
@@ -3926,8 +4047,9 @@
       <c r="N101" s="21" t="n"/>
       <c r="O101" s="21" t="n"/>
       <c r="P101" s="21" t="n"/>
-      <c r="Q101" s="18" t="n"/>
-      <c r="R101" s="19" t="n"/>
+      <c r="Q101" s="21" t="n"/>
+      <c r="R101" s="18" t="n"/>
+      <c r="S101" s="19" t="n"/>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="15" t="inlineStr">
@@ -3936,7 +4058,7 @@
         </is>
       </c>
       <c r="B102" s="16">
-        <f>IF(COUNTA(C102:R102)=0,"",IF(AND(C102&lt;&gt;"",D102&lt;&gt;"",E102&lt;&gt;"",H102&lt;&gt;"",I102&lt;&gt;"",NOT(AND(LEFT(I102,7)="Sale de",J102="",K102=""))),"✔ Completa","Falta: "&amp;IF(C102="","fecha · ","")&amp;IF(D102="","ubicación · ","")&amp;IF(E102="","referencia · ","")&amp;IF(H102="","criticidad · ","")&amp;IF(I102="","origen del agua · ","")&amp;IF(AND(LEFT(I102,7)="Sale de",J102="",K102=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C102:S102)=0,"",IF(AND(C102&lt;&gt;"",D102&lt;&gt;"",E102&lt;&gt;"",H102&lt;&gt;"",I102&lt;&gt;"",NOT(AND(LEFT(I102,7)="Sale de",J102="",K102=""))),"✔ Completa","Falta: "&amp;IF(C102="","fecha · ","")&amp;IF(D102="","ubicación · ","")&amp;IF(E102="","referencia · ","")&amp;IF(H102="","criticidad · ","")&amp;IF(I102="","origen del agua · ","")&amp;IF(AND(LEFT(I102,7)="Sale de",J102="",K102=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C102" s="17" t="n"/>
@@ -3953,8 +4075,9 @@
       <c r="N102" s="21" t="n"/>
       <c r="O102" s="21" t="n"/>
       <c r="P102" s="21" t="n"/>
-      <c r="Q102" s="18" t="n"/>
-      <c r="R102" s="19" t="n"/>
+      <c r="Q102" s="21" t="n"/>
+      <c r="R102" s="18" t="n"/>
+      <c r="S102" s="19" t="n"/>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="15" t="inlineStr">
@@ -3963,7 +4086,7 @@
         </is>
       </c>
       <c r="B103" s="16">
-        <f>IF(COUNTA(C103:R103)=0,"",IF(AND(C103&lt;&gt;"",D103&lt;&gt;"",E103&lt;&gt;"",H103&lt;&gt;"",I103&lt;&gt;"",NOT(AND(LEFT(I103,7)="Sale de",J103="",K103=""))),"✔ Completa","Falta: "&amp;IF(C103="","fecha · ","")&amp;IF(D103="","ubicación · ","")&amp;IF(E103="","referencia · ","")&amp;IF(H103="","criticidad · ","")&amp;IF(I103="","origen del agua · ","")&amp;IF(AND(LEFT(I103,7)="Sale de",J103="",K103=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C103:S103)=0,"",IF(AND(C103&lt;&gt;"",D103&lt;&gt;"",E103&lt;&gt;"",H103&lt;&gt;"",I103&lt;&gt;"",NOT(AND(LEFT(I103,7)="Sale de",J103="",K103=""))),"✔ Completa","Falta: "&amp;IF(C103="","fecha · ","")&amp;IF(D103="","ubicación · ","")&amp;IF(E103="","referencia · ","")&amp;IF(H103="","criticidad · ","")&amp;IF(I103="","origen del agua · ","")&amp;IF(AND(LEFT(I103,7)="Sale de",J103="",K103=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C103" s="17" t="n"/>
@@ -3980,8 +4103,9 @@
       <c r="N103" s="21" t="n"/>
       <c r="O103" s="21" t="n"/>
       <c r="P103" s="21" t="n"/>
-      <c r="Q103" s="18" t="n"/>
-      <c r="R103" s="19" t="n"/>
+      <c r="Q103" s="21" t="n"/>
+      <c r="R103" s="18" t="n"/>
+      <c r="S103" s="19" t="n"/>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="15" t="inlineStr">
@@ -3990,7 +4114,7 @@
         </is>
       </c>
       <c r="B104" s="16">
-        <f>IF(COUNTA(C104:R104)=0,"",IF(AND(C104&lt;&gt;"",D104&lt;&gt;"",E104&lt;&gt;"",H104&lt;&gt;"",I104&lt;&gt;"",NOT(AND(LEFT(I104,7)="Sale de",J104="",K104=""))),"✔ Completa","Falta: "&amp;IF(C104="","fecha · ","")&amp;IF(D104="","ubicación · ","")&amp;IF(E104="","referencia · ","")&amp;IF(H104="","criticidad · ","")&amp;IF(I104="","origen del agua · ","")&amp;IF(AND(LEFT(I104,7)="Sale de",J104="",K104=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C104:S104)=0,"",IF(AND(C104&lt;&gt;"",D104&lt;&gt;"",E104&lt;&gt;"",H104&lt;&gt;"",I104&lt;&gt;"",NOT(AND(LEFT(I104,7)="Sale de",J104="",K104=""))),"✔ Completa","Falta: "&amp;IF(C104="","fecha · ","")&amp;IF(D104="","ubicación · ","")&amp;IF(E104="","referencia · ","")&amp;IF(H104="","criticidad · ","")&amp;IF(I104="","origen del agua · ","")&amp;IF(AND(LEFT(I104,7)="Sale de",J104="",K104=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C104" s="17" t="n"/>
@@ -4007,8 +4131,9 @@
       <c r="N104" s="21" t="n"/>
       <c r="O104" s="21" t="n"/>
       <c r="P104" s="21" t="n"/>
-      <c r="Q104" s="18" t="n"/>
-      <c r="R104" s="19" t="n"/>
+      <c r="Q104" s="21" t="n"/>
+      <c r="R104" s="18" t="n"/>
+      <c r="S104" s="19" t="n"/>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
@@ -4017,7 +4142,7 @@
         </is>
       </c>
       <c r="B105" s="16">
-        <f>IF(COUNTA(C105:R105)=0,"",IF(AND(C105&lt;&gt;"",D105&lt;&gt;"",E105&lt;&gt;"",H105&lt;&gt;"",I105&lt;&gt;"",NOT(AND(LEFT(I105,7)="Sale de",J105="",K105=""))),"✔ Completa","Falta: "&amp;IF(C105="","fecha · ","")&amp;IF(D105="","ubicación · ","")&amp;IF(E105="","referencia · ","")&amp;IF(H105="","criticidad · ","")&amp;IF(I105="","origen del agua · ","")&amp;IF(AND(LEFT(I105,7)="Sale de",J105="",K105=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C105:S105)=0,"",IF(AND(C105&lt;&gt;"",D105&lt;&gt;"",E105&lt;&gt;"",H105&lt;&gt;"",I105&lt;&gt;"",NOT(AND(LEFT(I105,7)="Sale de",J105="",K105=""))),"✔ Completa","Falta: "&amp;IF(C105="","fecha · ","")&amp;IF(D105="","ubicación · ","")&amp;IF(E105="","referencia · ","")&amp;IF(H105="","criticidad · ","")&amp;IF(I105="","origen del agua · ","")&amp;IF(AND(LEFT(I105,7)="Sale de",J105="",K105=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C105" s="17" t="n"/>
@@ -4034,8 +4159,9 @@
       <c r="N105" s="21" t="n"/>
       <c r="O105" s="21" t="n"/>
       <c r="P105" s="21" t="n"/>
-      <c r="Q105" s="18" t="n"/>
-      <c r="R105" s="19" t="n"/>
+      <c r="Q105" s="21" t="n"/>
+      <c r="R105" s="18" t="n"/>
+      <c r="S105" s="19" t="n"/>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="15" t="inlineStr">
@@ -4044,7 +4170,7 @@
         </is>
       </c>
       <c r="B106" s="16">
-        <f>IF(COUNTA(C106:R106)=0,"",IF(AND(C106&lt;&gt;"",D106&lt;&gt;"",E106&lt;&gt;"",H106&lt;&gt;"",I106&lt;&gt;"",NOT(AND(LEFT(I106,7)="Sale de",J106="",K106=""))),"✔ Completa","Falta: "&amp;IF(C106="","fecha · ","")&amp;IF(D106="","ubicación · ","")&amp;IF(E106="","referencia · ","")&amp;IF(H106="","criticidad · ","")&amp;IF(I106="","origen del agua · ","")&amp;IF(AND(LEFT(I106,7)="Sale de",J106="",K106=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C106:S106)=0,"",IF(AND(C106&lt;&gt;"",D106&lt;&gt;"",E106&lt;&gt;"",H106&lt;&gt;"",I106&lt;&gt;"",NOT(AND(LEFT(I106,7)="Sale de",J106="",K106=""))),"✔ Completa","Falta: "&amp;IF(C106="","fecha · ","")&amp;IF(D106="","ubicación · ","")&amp;IF(E106="","referencia · ","")&amp;IF(H106="","criticidad · ","")&amp;IF(I106="","origen del agua · ","")&amp;IF(AND(LEFT(I106,7)="Sale de",J106="",K106=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C106" s="17" t="n"/>
@@ -4061,8 +4187,9 @@
       <c r="N106" s="21" t="n"/>
       <c r="O106" s="21" t="n"/>
       <c r="P106" s="21" t="n"/>
-      <c r="Q106" s="18" t="n"/>
-      <c r="R106" s="19" t="n"/>
+      <c r="Q106" s="21" t="n"/>
+      <c r="R106" s="18" t="n"/>
+      <c r="S106" s="19" t="n"/>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="15" t="inlineStr">
@@ -4071,7 +4198,7 @@
         </is>
       </c>
       <c r="B107" s="16">
-        <f>IF(COUNTA(C107:R107)=0,"",IF(AND(C107&lt;&gt;"",D107&lt;&gt;"",E107&lt;&gt;"",H107&lt;&gt;"",I107&lt;&gt;"",NOT(AND(LEFT(I107,7)="Sale de",J107="",K107=""))),"✔ Completa","Falta: "&amp;IF(C107="","fecha · ","")&amp;IF(D107="","ubicación · ","")&amp;IF(E107="","referencia · ","")&amp;IF(H107="","criticidad · ","")&amp;IF(I107="","origen del agua · ","")&amp;IF(AND(LEFT(I107,7)="Sale de",J107="",K107=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C107:S107)=0,"",IF(AND(C107&lt;&gt;"",D107&lt;&gt;"",E107&lt;&gt;"",H107&lt;&gt;"",I107&lt;&gt;"",NOT(AND(LEFT(I107,7)="Sale de",J107="",K107=""))),"✔ Completa","Falta: "&amp;IF(C107="","fecha · ","")&amp;IF(D107="","ubicación · ","")&amp;IF(E107="","referencia · ","")&amp;IF(H107="","criticidad · ","")&amp;IF(I107="","origen del agua · ","")&amp;IF(AND(LEFT(I107,7)="Sale de",J107="",K107=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C107" s="17" t="n"/>
@@ -4088,8 +4215,9 @@
       <c r="N107" s="21" t="n"/>
       <c r="O107" s="21" t="n"/>
       <c r="P107" s="21" t="n"/>
-      <c r="Q107" s="18" t="n"/>
-      <c r="R107" s="19" t="n"/>
+      <c r="Q107" s="21" t="n"/>
+      <c r="R107" s="18" t="n"/>
+      <c r="S107" s="19" t="n"/>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="15" t="inlineStr">
@@ -4098,7 +4226,7 @@
         </is>
       </c>
       <c r="B108" s="16">
-        <f>IF(COUNTA(C108:R108)=0,"",IF(AND(C108&lt;&gt;"",D108&lt;&gt;"",E108&lt;&gt;"",H108&lt;&gt;"",I108&lt;&gt;"",NOT(AND(LEFT(I108,7)="Sale de",J108="",K108=""))),"✔ Completa","Falta: "&amp;IF(C108="","fecha · ","")&amp;IF(D108="","ubicación · ","")&amp;IF(E108="","referencia · ","")&amp;IF(H108="","criticidad · ","")&amp;IF(I108="","origen del agua · ","")&amp;IF(AND(LEFT(I108,7)="Sale de",J108="",K108=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C108:S108)=0,"",IF(AND(C108&lt;&gt;"",D108&lt;&gt;"",E108&lt;&gt;"",H108&lt;&gt;"",I108&lt;&gt;"",NOT(AND(LEFT(I108,7)="Sale de",J108="",K108=""))),"✔ Completa","Falta: "&amp;IF(C108="","fecha · ","")&amp;IF(D108="","ubicación · ","")&amp;IF(E108="","referencia · ","")&amp;IF(H108="","criticidad · ","")&amp;IF(I108="","origen del agua · ","")&amp;IF(AND(LEFT(I108,7)="Sale de",J108="",K108=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C108" s="17" t="n"/>
@@ -4115,8 +4243,9 @@
       <c r="N108" s="21" t="n"/>
       <c r="O108" s="21" t="n"/>
       <c r="P108" s="21" t="n"/>
-      <c r="Q108" s="18" t="n"/>
-      <c r="R108" s="19" t="n"/>
+      <c r="Q108" s="21" t="n"/>
+      <c r="R108" s="18" t="n"/>
+      <c r="S108" s="19" t="n"/>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="15" t="inlineStr">
@@ -4125,7 +4254,7 @@
         </is>
       </c>
       <c r="B109" s="16">
-        <f>IF(COUNTA(C109:R109)=0,"",IF(AND(C109&lt;&gt;"",D109&lt;&gt;"",E109&lt;&gt;"",H109&lt;&gt;"",I109&lt;&gt;"",NOT(AND(LEFT(I109,7)="Sale de",J109="",K109=""))),"✔ Completa","Falta: "&amp;IF(C109="","fecha · ","")&amp;IF(D109="","ubicación · ","")&amp;IF(E109="","referencia · ","")&amp;IF(H109="","criticidad · ","")&amp;IF(I109="","origen del agua · ","")&amp;IF(AND(LEFT(I109,7)="Sale de",J109="",K109=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C109:S109)=0,"",IF(AND(C109&lt;&gt;"",D109&lt;&gt;"",E109&lt;&gt;"",H109&lt;&gt;"",I109&lt;&gt;"",NOT(AND(LEFT(I109,7)="Sale de",J109="",K109=""))),"✔ Completa","Falta: "&amp;IF(C109="","fecha · ","")&amp;IF(D109="","ubicación · ","")&amp;IF(E109="","referencia · ","")&amp;IF(H109="","criticidad · ","")&amp;IF(I109="","origen del agua · ","")&amp;IF(AND(LEFT(I109,7)="Sale de",J109="",K109=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C109" s="17" t="n"/>
@@ -4142,8 +4271,9 @@
       <c r="N109" s="21" t="n"/>
       <c r="O109" s="21" t="n"/>
       <c r="P109" s="21" t="n"/>
-      <c r="Q109" s="18" t="n"/>
-      <c r="R109" s="19" t="n"/>
+      <c r="Q109" s="21" t="n"/>
+      <c r="R109" s="18" t="n"/>
+      <c r="S109" s="19" t="n"/>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="15" t="inlineStr">
@@ -4152,7 +4282,7 @@
         </is>
       </c>
       <c r="B110" s="16">
-        <f>IF(COUNTA(C110:R110)=0,"",IF(AND(C110&lt;&gt;"",D110&lt;&gt;"",E110&lt;&gt;"",H110&lt;&gt;"",I110&lt;&gt;"",NOT(AND(LEFT(I110,7)="Sale de",J110="",K110=""))),"✔ Completa","Falta: "&amp;IF(C110="","fecha · ","")&amp;IF(D110="","ubicación · ","")&amp;IF(E110="","referencia · ","")&amp;IF(H110="","criticidad · ","")&amp;IF(I110="","origen del agua · ","")&amp;IF(AND(LEFT(I110,7)="Sale de",J110="",K110=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C110:S110)=0,"",IF(AND(C110&lt;&gt;"",D110&lt;&gt;"",E110&lt;&gt;"",H110&lt;&gt;"",I110&lt;&gt;"",NOT(AND(LEFT(I110,7)="Sale de",J110="",K110=""))),"✔ Completa","Falta: "&amp;IF(C110="","fecha · ","")&amp;IF(D110="","ubicación · ","")&amp;IF(E110="","referencia · ","")&amp;IF(H110="","criticidad · ","")&amp;IF(I110="","origen del agua · ","")&amp;IF(AND(LEFT(I110,7)="Sale de",J110="",K110=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C110" s="17" t="n"/>
@@ -4169,8 +4299,9 @@
       <c r="N110" s="21" t="n"/>
       <c r="O110" s="21" t="n"/>
       <c r="P110" s="21" t="n"/>
-      <c r="Q110" s="18" t="n"/>
-      <c r="R110" s="19" t="n"/>
+      <c r="Q110" s="21" t="n"/>
+      <c r="R110" s="18" t="n"/>
+      <c r="S110" s="19" t="n"/>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="15" t="inlineStr">
@@ -4179,7 +4310,7 @@
         </is>
       </c>
       <c r="B111" s="16">
-        <f>IF(COUNTA(C111:R111)=0,"",IF(AND(C111&lt;&gt;"",D111&lt;&gt;"",E111&lt;&gt;"",H111&lt;&gt;"",I111&lt;&gt;"",NOT(AND(LEFT(I111,7)="Sale de",J111="",K111=""))),"✔ Completa","Falta: "&amp;IF(C111="","fecha · ","")&amp;IF(D111="","ubicación · ","")&amp;IF(E111="","referencia · ","")&amp;IF(H111="","criticidad · ","")&amp;IF(I111="","origen del agua · ","")&amp;IF(AND(LEFT(I111,7)="Sale de",J111="",K111=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C111:S111)=0,"",IF(AND(C111&lt;&gt;"",D111&lt;&gt;"",E111&lt;&gt;"",H111&lt;&gt;"",I111&lt;&gt;"",NOT(AND(LEFT(I111,7)="Sale de",J111="",K111=""))),"✔ Completa","Falta: "&amp;IF(C111="","fecha · ","")&amp;IF(D111="","ubicación · ","")&amp;IF(E111="","referencia · ","")&amp;IF(H111="","criticidad · ","")&amp;IF(I111="","origen del agua · ","")&amp;IF(AND(LEFT(I111,7)="Sale de",J111="",K111=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C111" s="17" t="n"/>
@@ -4196,8 +4327,9 @@
       <c r="N111" s="21" t="n"/>
       <c r="O111" s="21" t="n"/>
       <c r="P111" s="21" t="n"/>
-      <c r="Q111" s="18" t="n"/>
-      <c r="R111" s="19" t="n"/>
+      <c r="Q111" s="21" t="n"/>
+      <c r="R111" s="18" t="n"/>
+      <c r="S111" s="19" t="n"/>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="15" t="inlineStr">
@@ -4206,7 +4338,7 @@
         </is>
       </c>
       <c r="B112" s="16">
-        <f>IF(COUNTA(C112:R112)=0,"",IF(AND(C112&lt;&gt;"",D112&lt;&gt;"",E112&lt;&gt;"",H112&lt;&gt;"",I112&lt;&gt;"",NOT(AND(LEFT(I112,7)="Sale de",J112="",K112=""))),"✔ Completa","Falta: "&amp;IF(C112="","fecha · ","")&amp;IF(D112="","ubicación · ","")&amp;IF(E112="","referencia · ","")&amp;IF(H112="","criticidad · ","")&amp;IF(I112="","origen del agua · ","")&amp;IF(AND(LEFT(I112,7)="Sale de",J112="",K112=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C112:S112)=0,"",IF(AND(C112&lt;&gt;"",D112&lt;&gt;"",E112&lt;&gt;"",H112&lt;&gt;"",I112&lt;&gt;"",NOT(AND(LEFT(I112,7)="Sale de",J112="",K112=""))),"✔ Completa","Falta: "&amp;IF(C112="","fecha · ","")&amp;IF(D112="","ubicación · ","")&amp;IF(E112="","referencia · ","")&amp;IF(H112="","criticidad · ","")&amp;IF(I112="","origen del agua · ","")&amp;IF(AND(LEFT(I112,7)="Sale de",J112="",K112=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C112" s="17" t="n"/>
@@ -4223,8 +4355,9 @@
       <c r="N112" s="21" t="n"/>
       <c r="O112" s="21" t="n"/>
       <c r="P112" s="21" t="n"/>
-      <c r="Q112" s="18" t="n"/>
-      <c r="R112" s="19" t="n"/>
+      <c r="Q112" s="21" t="n"/>
+      <c r="R112" s="18" t="n"/>
+      <c r="S112" s="19" t="n"/>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="15" t="inlineStr">
@@ -4233,7 +4366,7 @@
         </is>
       </c>
       <c r="B113" s="16">
-        <f>IF(COUNTA(C113:R113)=0,"",IF(AND(C113&lt;&gt;"",D113&lt;&gt;"",E113&lt;&gt;"",H113&lt;&gt;"",I113&lt;&gt;"",NOT(AND(LEFT(I113,7)="Sale de",J113="",K113=""))),"✔ Completa","Falta: "&amp;IF(C113="","fecha · ","")&amp;IF(D113="","ubicación · ","")&amp;IF(E113="","referencia · ","")&amp;IF(H113="","criticidad · ","")&amp;IF(I113="","origen del agua · ","")&amp;IF(AND(LEFT(I113,7)="Sale de",J113="",K113=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C113:S113)=0,"",IF(AND(C113&lt;&gt;"",D113&lt;&gt;"",E113&lt;&gt;"",H113&lt;&gt;"",I113&lt;&gt;"",NOT(AND(LEFT(I113,7)="Sale de",J113="",K113=""))),"✔ Completa","Falta: "&amp;IF(C113="","fecha · ","")&amp;IF(D113="","ubicación · ","")&amp;IF(E113="","referencia · ","")&amp;IF(H113="","criticidad · ","")&amp;IF(I113="","origen del agua · ","")&amp;IF(AND(LEFT(I113,7)="Sale de",J113="",K113=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C113" s="17" t="n"/>
@@ -4250,8 +4383,9 @@
       <c r="N113" s="21" t="n"/>
       <c r="O113" s="21" t="n"/>
       <c r="P113" s="21" t="n"/>
-      <c r="Q113" s="18" t="n"/>
-      <c r="R113" s="19" t="n"/>
+      <c r="Q113" s="21" t="n"/>
+      <c r="R113" s="18" t="n"/>
+      <c r="S113" s="19" t="n"/>
     </row>
     <row r="114" ht="20" customHeight="1">
       <c r="A114" s="15" t="inlineStr">
@@ -4260,7 +4394,7 @@
         </is>
       </c>
       <c r="B114" s="16">
-        <f>IF(COUNTA(C114:R114)=0,"",IF(AND(C114&lt;&gt;"",D114&lt;&gt;"",E114&lt;&gt;"",H114&lt;&gt;"",I114&lt;&gt;"",NOT(AND(LEFT(I114,7)="Sale de",J114="",K114=""))),"✔ Completa","Falta: "&amp;IF(C114="","fecha · ","")&amp;IF(D114="","ubicación · ","")&amp;IF(E114="","referencia · ","")&amp;IF(H114="","criticidad · ","")&amp;IF(I114="","origen del agua · ","")&amp;IF(AND(LEFT(I114,7)="Sale de",J114="",K114=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C114:S114)=0,"",IF(AND(C114&lt;&gt;"",D114&lt;&gt;"",E114&lt;&gt;"",H114&lt;&gt;"",I114&lt;&gt;"",NOT(AND(LEFT(I114,7)="Sale de",J114="",K114=""))),"✔ Completa","Falta: "&amp;IF(C114="","fecha · ","")&amp;IF(D114="","ubicación · ","")&amp;IF(E114="","referencia · ","")&amp;IF(H114="","criticidad · ","")&amp;IF(I114="","origen del agua · ","")&amp;IF(AND(LEFT(I114,7)="Sale de",J114="",K114=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C114" s="17" t="n"/>
@@ -4277,8 +4411,9 @@
       <c r="N114" s="21" t="n"/>
       <c r="O114" s="21" t="n"/>
       <c r="P114" s="21" t="n"/>
-      <c r="Q114" s="18" t="n"/>
-      <c r="R114" s="19" t="n"/>
+      <c r="Q114" s="21" t="n"/>
+      <c r="R114" s="18" t="n"/>
+      <c r="S114" s="19" t="n"/>
     </row>
     <row r="115" ht="20" customHeight="1">
       <c r="A115" s="15" t="inlineStr">
@@ -4287,7 +4422,7 @@
         </is>
       </c>
       <c r="B115" s="16">
-        <f>IF(COUNTA(C115:R115)=0,"",IF(AND(C115&lt;&gt;"",D115&lt;&gt;"",E115&lt;&gt;"",H115&lt;&gt;"",I115&lt;&gt;"",NOT(AND(LEFT(I115,7)="Sale de",J115="",K115=""))),"✔ Completa","Falta: "&amp;IF(C115="","fecha · ","")&amp;IF(D115="","ubicación · ","")&amp;IF(E115="","referencia · ","")&amp;IF(H115="","criticidad · ","")&amp;IF(I115="","origen del agua · ","")&amp;IF(AND(LEFT(I115,7)="Sale de",J115="",K115=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C115:S115)=0,"",IF(AND(C115&lt;&gt;"",D115&lt;&gt;"",E115&lt;&gt;"",H115&lt;&gt;"",I115&lt;&gt;"",NOT(AND(LEFT(I115,7)="Sale de",J115="",K115=""))),"✔ Completa","Falta: "&amp;IF(C115="","fecha · ","")&amp;IF(D115="","ubicación · ","")&amp;IF(E115="","referencia · ","")&amp;IF(H115="","criticidad · ","")&amp;IF(I115="","origen del agua · ","")&amp;IF(AND(LEFT(I115,7)="Sale de",J115="",K115=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C115" s="17" t="n"/>
@@ -4304,8 +4439,9 @@
       <c r="N115" s="21" t="n"/>
       <c r="O115" s="21" t="n"/>
       <c r="P115" s="21" t="n"/>
-      <c r="Q115" s="18" t="n"/>
-      <c r="R115" s="19" t="n"/>
+      <c r="Q115" s="21" t="n"/>
+      <c r="R115" s="18" t="n"/>
+      <c r="S115" s="19" t="n"/>
     </row>
     <row r="116" ht="20" customHeight="1">
       <c r="A116" s="15" t="inlineStr">
@@ -4314,7 +4450,7 @@
         </is>
       </c>
       <c r="B116" s="16">
-        <f>IF(COUNTA(C116:R116)=0,"",IF(AND(C116&lt;&gt;"",D116&lt;&gt;"",E116&lt;&gt;"",H116&lt;&gt;"",I116&lt;&gt;"",NOT(AND(LEFT(I116,7)="Sale de",J116="",K116=""))),"✔ Completa","Falta: "&amp;IF(C116="","fecha · ","")&amp;IF(D116="","ubicación · ","")&amp;IF(E116="","referencia · ","")&amp;IF(H116="","criticidad · ","")&amp;IF(I116="","origen del agua · ","")&amp;IF(AND(LEFT(I116,7)="Sale de",J116="",K116=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C116:S116)=0,"",IF(AND(C116&lt;&gt;"",D116&lt;&gt;"",E116&lt;&gt;"",H116&lt;&gt;"",I116&lt;&gt;"",NOT(AND(LEFT(I116,7)="Sale de",J116="",K116=""))),"✔ Completa","Falta: "&amp;IF(C116="","fecha · ","")&amp;IF(D116="","ubicación · ","")&amp;IF(E116="","referencia · ","")&amp;IF(H116="","criticidad · ","")&amp;IF(I116="","origen del agua · ","")&amp;IF(AND(LEFT(I116,7)="Sale de",J116="",K116=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C116" s="17" t="n"/>
@@ -4331,8 +4467,9 @@
       <c r="N116" s="21" t="n"/>
       <c r="O116" s="21" t="n"/>
       <c r="P116" s="21" t="n"/>
-      <c r="Q116" s="18" t="n"/>
-      <c r="R116" s="19" t="n"/>
+      <c r="Q116" s="21" t="n"/>
+      <c r="R116" s="18" t="n"/>
+      <c r="S116" s="19" t="n"/>
     </row>
     <row r="117" ht="20" customHeight="1">
       <c r="A117" s="15" t="inlineStr">
@@ -4341,7 +4478,7 @@
         </is>
       </c>
       <c r="B117" s="16">
-        <f>IF(COUNTA(C117:R117)=0,"",IF(AND(C117&lt;&gt;"",D117&lt;&gt;"",E117&lt;&gt;"",H117&lt;&gt;"",I117&lt;&gt;"",NOT(AND(LEFT(I117,7)="Sale de",J117="",K117=""))),"✔ Completa","Falta: "&amp;IF(C117="","fecha · ","")&amp;IF(D117="","ubicación · ","")&amp;IF(E117="","referencia · ","")&amp;IF(H117="","criticidad · ","")&amp;IF(I117="","origen del agua · ","")&amp;IF(AND(LEFT(I117,7)="Sale de",J117="",K117=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C117:S117)=0,"",IF(AND(C117&lt;&gt;"",D117&lt;&gt;"",E117&lt;&gt;"",H117&lt;&gt;"",I117&lt;&gt;"",NOT(AND(LEFT(I117,7)="Sale de",J117="",K117=""))),"✔ Completa","Falta: "&amp;IF(C117="","fecha · ","")&amp;IF(D117="","ubicación · ","")&amp;IF(E117="","referencia · ","")&amp;IF(H117="","criticidad · ","")&amp;IF(I117="","origen del agua · ","")&amp;IF(AND(LEFT(I117,7)="Sale de",J117="",K117=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C117" s="17" t="n"/>
@@ -4358,8 +4495,9 @@
       <c r="N117" s="21" t="n"/>
       <c r="O117" s="21" t="n"/>
       <c r="P117" s="21" t="n"/>
-      <c r="Q117" s="18" t="n"/>
-      <c r="R117" s="19" t="n"/>
+      <c r="Q117" s="21" t="n"/>
+      <c r="R117" s="18" t="n"/>
+      <c r="S117" s="19" t="n"/>
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="15" t="inlineStr">
@@ -4368,7 +4506,7 @@
         </is>
       </c>
       <c r="B118" s="16">
-        <f>IF(COUNTA(C118:R118)=0,"",IF(AND(C118&lt;&gt;"",D118&lt;&gt;"",E118&lt;&gt;"",H118&lt;&gt;"",I118&lt;&gt;"",NOT(AND(LEFT(I118,7)="Sale de",J118="",K118=""))),"✔ Completa","Falta: "&amp;IF(C118="","fecha · ","")&amp;IF(D118="","ubicación · ","")&amp;IF(E118="","referencia · ","")&amp;IF(H118="","criticidad · ","")&amp;IF(I118="","origen del agua · ","")&amp;IF(AND(LEFT(I118,7)="Sale de",J118="",K118=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C118:S118)=0,"",IF(AND(C118&lt;&gt;"",D118&lt;&gt;"",E118&lt;&gt;"",H118&lt;&gt;"",I118&lt;&gt;"",NOT(AND(LEFT(I118,7)="Sale de",J118="",K118=""))),"✔ Completa","Falta: "&amp;IF(C118="","fecha · ","")&amp;IF(D118="","ubicación · ","")&amp;IF(E118="","referencia · ","")&amp;IF(H118="","criticidad · ","")&amp;IF(I118="","origen del agua · ","")&amp;IF(AND(LEFT(I118,7)="Sale de",J118="",K118=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C118" s="17" t="n"/>
@@ -4385,8 +4523,9 @@
       <c r="N118" s="21" t="n"/>
       <c r="O118" s="21" t="n"/>
       <c r="P118" s="21" t="n"/>
-      <c r="Q118" s="18" t="n"/>
-      <c r="R118" s="19" t="n"/>
+      <c r="Q118" s="21" t="n"/>
+      <c r="R118" s="18" t="n"/>
+      <c r="S118" s="19" t="n"/>
     </row>
     <row r="119" ht="20" customHeight="1">
       <c r="A119" s="15" t="inlineStr">
@@ -4395,7 +4534,7 @@
         </is>
       </c>
       <c r="B119" s="16">
-        <f>IF(COUNTA(C119:R119)=0,"",IF(AND(C119&lt;&gt;"",D119&lt;&gt;"",E119&lt;&gt;"",H119&lt;&gt;"",I119&lt;&gt;"",NOT(AND(LEFT(I119,7)="Sale de",J119="",K119=""))),"✔ Completa","Falta: "&amp;IF(C119="","fecha · ","")&amp;IF(D119="","ubicación · ","")&amp;IF(E119="","referencia · ","")&amp;IF(H119="","criticidad · ","")&amp;IF(I119="","origen del agua · ","")&amp;IF(AND(LEFT(I119,7)="Sale de",J119="",K119=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C119:S119)=0,"",IF(AND(C119&lt;&gt;"",D119&lt;&gt;"",E119&lt;&gt;"",H119&lt;&gt;"",I119&lt;&gt;"",NOT(AND(LEFT(I119,7)="Sale de",J119="",K119=""))),"✔ Completa","Falta: "&amp;IF(C119="","fecha · ","")&amp;IF(D119="","ubicación · ","")&amp;IF(E119="","referencia · ","")&amp;IF(H119="","criticidad · ","")&amp;IF(I119="","origen del agua · ","")&amp;IF(AND(LEFT(I119,7)="Sale de",J119="",K119=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C119" s="17" t="n"/>
@@ -4412,8 +4551,9 @@
       <c r="N119" s="21" t="n"/>
       <c r="O119" s="21" t="n"/>
       <c r="P119" s="21" t="n"/>
-      <c r="Q119" s="18" t="n"/>
-      <c r="R119" s="19" t="n"/>
+      <c r="Q119" s="21" t="n"/>
+      <c r="R119" s="18" t="n"/>
+      <c r="S119" s="19" t="n"/>
     </row>
     <row r="120" ht="20" customHeight="1">
       <c r="A120" s="15" t="inlineStr">
@@ -4422,7 +4562,7 @@
         </is>
       </c>
       <c r="B120" s="16">
-        <f>IF(COUNTA(C120:R120)=0,"",IF(AND(C120&lt;&gt;"",D120&lt;&gt;"",E120&lt;&gt;"",H120&lt;&gt;"",I120&lt;&gt;"",NOT(AND(LEFT(I120,7)="Sale de",J120="",K120=""))),"✔ Completa","Falta: "&amp;IF(C120="","fecha · ","")&amp;IF(D120="","ubicación · ","")&amp;IF(E120="","referencia · ","")&amp;IF(H120="","criticidad · ","")&amp;IF(I120="","origen del agua · ","")&amp;IF(AND(LEFT(I120,7)="Sale de",J120="",K120=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C120:S120)=0,"",IF(AND(C120&lt;&gt;"",D120&lt;&gt;"",E120&lt;&gt;"",H120&lt;&gt;"",I120&lt;&gt;"",NOT(AND(LEFT(I120,7)="Sale de",J120="",K120=""))),"✔ Completa","Falta: "&amp;IF(C120="","fecha · ","")&amp;IF(D120="","ubicación · ","")&amp;IF(E120="","referencia · ","")&amp;IF(H120="","criticidad · ","")&amp;IF(I120="","origen del agua · ","")&amp;IF(AND(LEFT(I120,7)="Sale de",J120="",K120=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C120" s="17" t="n"/>
@@ -4439,8 +4579,9 @@
       <c r="N120" s="21" t="n"/>
       <c r="O120" s="21" t="n"/>
       <c r="P120" s="21" t="n"/>
-      <c r="Q120" s="18" t="n"/>
-      <c r="R120" s="19" t="n"/>
+      <c r="Q120" s="21" t="n"/>
+      <c r="R120" s="18" t="n"/>
+      <c r="S120" s="19" t="n"/>
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121" s="15" t="inlineStr">
@@ -4449,7 +4590,7 @@
         </is>
       </c>
       <c r="B121" s="16">
-        <f>IF(COUNTA(C121:R121)=0,"",IF(AND(C121&lt;&gt;"",D121&lt;&gt;"",E121&lt;&gt;"",H121&lt;&gt;"",I121&lt;&gt;"",NOT(AND(LEFT(I121,7)="Sale de",J121="",K121=""))),"✔ Completa","Falta: "&amp;IF(C121="","fecha · ","")&amp;IF(D121="","ubicación · ","")&amp;IF(E121="","referencia · ","")&amp;IF(H121="","criticidad · ","")&amp;IF(I121="","origen del agua · ","")&amp;IF(AND(LEFT(I121,7)="Sale de",J121="",K121=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C121:S121)=0,"",IF(AND(C121&lt;&gt;"",D121&lt;&gt;"",E121&lt;&gt;"",H121&lt;&gt;"",I121&lt;&gt;"",NOT(AND(LEFT(I121,7)="Sale de",J121="",K121=""))),"✔ Completa","Falta: "&amp;IF(C121="","fecha · ","")&amp;IF(D121="","ubicación · ","")&amp;IF(E121="","referencia · ","")&amp;IF(H121="","criticidad · ","")&amp;IF(I121="","origen del agua · ","")&amp;IF(AND(LEFT(I121,7)="Sale de",J121="",K121=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C121" s="17" t="n"/>
@@ -4466,8 +4607,9 @@
       <c r="N121" s="21" t="n"/>
       <c r="O121" s="21" t="n"/>
       <c r="P121" s="21" t="n"/>
-      <c r="Q121" s="18" t="n"/>
-      <c r="R121" s="19" t="n"/>
+      <c r="Q121" s="21" t="n"/>
+      <c r="R121" s="18" t="n"/>
+      <c r="S121" s="19" t="n"/>
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="15" t="inlineStr">
@@ -4476,7 +4618,7 @@
         </is>
       </c>
       <c r="B122" s="16">
-        <f>IF(COUNTA(C122:R122)=0,"",IF(AND(C122&lt;&gt;"",D122&lt;&gt;"",E122&lt;&gt;"",H122&lt;&gt;"",I122&lt;&gt;"",NOT(AND(LEFT(I122,7)="Sale de",J122="",K122=""))),"✔ Completa","Falta: "&amp;IF(C122="","fecha · ","")&amp;IF(D122="","ubicación · ","")&amp;IF(E122="","referencia · ","")&amp;IF(H122="","criticidad · ","")&amp;IF(I122="","origen del agua · ","")&amp;IF(AND(LEFT(I122,7)="Sale de",J122="",K122=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C122:S122)=0,"",IF(AND(C122&lt;&gt;"",D122&lt;&gt;"",E122&lt;&gt;"",H122&lt;&gt;"",I122&lt;&gt;"",NOT(AND(LEFT(I122,7)="Sale de",J122="",K122=""))),"✔ Completa","Falta: "&amp;IF(C122="","fecha · ","")&amp;IF(D122="","ubicación · ","")&amp;IF(E122="","referencia · ","")&amp;IF(H122="","criticidad · ","")&amp;IF(I122="","origen del agua · ","")&amp;IF(AND(LEFT(I122,7)="Sale de",J122="",K122=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C122" s="17" t="n"/>
@@ -4493,8 +4635,9 @@
       <c r="N122" s="21" t="n"/>
       <c r="O122" s="21" t="n"/>
       <c r="P122" s="21" t="n"/>
-      <c r="Q122" s="18" t="n"/>
-      <c r="R122" s="19" t="n"/>
+      <c r="Q122" s="21" t="n"/>
+      <c r="R122" s="18" t="n"/>
+      <c r="S122" s="19" t="n"/>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="15" t="inlineStr">
@@ -4503,7 +4646,7 @@
         </is>
       </c>
       <c r="B123" s="16">
-        <f>IF(COUNTA(C123:R123)=0,"",IF(AND(C123&lt;&gt;"",D123&lt;&gt;"",E123&lt;&gt;"",H123&lt;&gt;"",I123&lt;&gt;"",NOT(AND(LEFT(I123,7)="Sale de",J123="",K123=""))),"✔ Completa","Falta: "&amp;IF(C123="","fecha · ","")&amp;IF(D123="","ubicación · ","")&amp;IF(E123="","referencia · ","")&amp;IF(H123="","criticidad · ","")&amp;IF(I123="","origen del agua · ","")&amp;IF(AND(LEFT(I123,7)="Sale de",J123="",K123=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C123:S123)=0,"",IF(AND(C123&lt;&gt;"",D123&lt;&gt;"",E123&lt;&gt;"",H123&lt;&gt;"",I123&lt;&gt;"",NOT(AND(LEFT(I123,7)="Sale de",J123="",K123=""))),"✔ Completa","Falta: "&amp;IF(C123="","fecha · ","")&amp;IF(D123="","ubicación · ","")&amp;IF(E123="","referencia · ","")&amp;IF(H123="","criticidad · ","")&amp;IF(I123="","origen del agua · ","")&amp;IF(AND(LEFT(I123,7)="Sale de",J123="",K123=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C123" s="17" t="n"/>
@@ -4520,8 +4663,9 @@
       <c r="N123" s="21" t="n"/>
       <c r="O123" s="21" t="n"/>
       <c r="P123" s="21" t="n"/>
-      <c r="Q123" s="18" t="n"/>
-      <c r="R123" s="19" t="n"/>
+      <c r="Q123" s="21" t="n"/>
+      <c r="R123" s="18" t="n"/>
+      <c r="S123" s="19" t="n"/>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="15" t="inlineStr">
@@ -4530,7 +4674,7 @@
         </is>
       </c>
       <c r="B124" s="16">
-        <f>IF(COUNTA(C124:R124)=0,"",IF(AND(C124&lt;&gt;"",D124&lt;&gt;"",E124&lt;&gt;"",H124&lt;&gt;"",I124&lt;&gt;"",NOT(AND(LEFT(I124,7)="Sale de",J124="",K124=""))),"✔ Completa","Falta: "&amp;IF(C124="","fecha · ","")&amp;IF(D124="","ubicación · ","")&amp;IF(E124="","referencia · ","")&amp;IF(H124="","criticidad · ","")&amp;IF(I124="","origen del agua · ","")&amp;IF(AND(LEFT(I124,7)="Sale de",J124="",K124=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C124:S124)=0,"",IF(AND(C124&lt;&gt;"",D124&lt;&gt;"",E124&lt;&gt;"",H124&lt;&gt;"",I124&lt;&gt;"",NOT(AND(LEFT(I124,7)="Sale de",J124="",K124=""))),"✔ Completa","Falta: "&amp;IF(C124="","fecha · ","")&amp;IF(D124="","ubicación · ","")&amp;IF(E124="","referencia · ","")&amp;IF(H124="","criticidad · ","")&amp;IF(I124="","origen del agua · ","")&amp;IF(AND(LEFT(I124,7)="Sale de",J124="",K124=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C124" s="17" t="n"/>
@@ -4547,8 +4691,9 @@
       <c r="N124" s="21" t="n"/>
       <c r="O124" s="21" t="n"/>
       <c r="P124" s="21" t="n"/>
-      <c r="Q124" s="18" t="n"/>
-      <c r="R124" s="19" t="n"/>
+      <c r="Q124" s="21" t="n"/>
+      <c r="R124" s="18" t="n"/>
+      <c r="S124" s="19" t="n"/>
     </row>
     <row r="125" ht="20" customHeight="1">
       <c r="A125" s="15" t="inlineStr">
@@ -4557,7 +4702,7 @@
         </is>
       </c>
       <c r="B125" s="16">
-        <f>IF(COUNTA(C125:R125)=0,"",IF(AND(C125&lt;&gt;"",D125&lt;&gt;"",E125&lt;&gt;"",H125&lt;&gt;"",I125&lt;&gt;"",NOT(AND(LEFT(I125,7)="Sale de",J125="",K125=""))),"✔ Completa","Falta: "&amp;IF(C125="","fecha · ","")&amp;IF(D125="","ubicación · ","")&amp;IF(E125="","referencia · ","")&amp;IF(H125="","criticidad · ","")&amp;IF(I125="","origen del agua · ","")&amp;IF(AND(LEFT(I125,7)="Sale de",J125="",K125=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C125:S125)=0,"",IF(AND(C125&lt;&gt;"",D125&lt;&gt;"",E125&lt;&gt;"",H125&lt;&gt;"",I125&lt;&gt;"",NOT(AND(LEFT(I125,7)="Sale de",J125="",K125=""))),"✔ Completa","Falta: "&amp;IF(C125="","fecha · ","")&amp;IF(D125="","ubicación · ","")&amp;IF(E125="","referencia · ","")&amp;IF(H125="","criticidad · ","")&amp;IF(I125="","origen del agua · ","")&amp;IF(AND(LEFT(I125,7)="Sale de",J125="",K125=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C125" s="17" t="n"/>
@@ -4574,8 +4719,9 @@
       <c r="N125" s="21" t="n"/>
       <c r="O125" s="21" t="n"/>
       <c r="P125" s="21" t="n"/>
-      <c r="Q125" s="18" t="n"/>
-      <c r="R125" s="19" t="n"/>
+      <c r="Q125" s="21" t="n"/>
+      <c r="R125" s="18" t="n"/>
+      <c r="S125" s="19" t="n"/>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="15" t="inlineStr">
@@ -4584,7 +4730,7 @@
         </is>
       </c>
       <c r="B126" s="16">
-        <f>IF(COUNTA(C126:R126)=0,"",IF(AND(C126&lt;&gt;"",D126&lt;&gt;"",E126&lt;&gt;"",H126&lt;&gt;"",I126&lt;&gt;"",NOT(AND(LEFT(I126,7)="Sale de",J126="",K126=""))),"✔ Completa","Falta: "&amp;IF(C126="","fecha · ","")&amp;IF(D126="","ubicación · ","")&amp;IF(E126="","referencia · ","")&amp;IF(H126="","criticidad · ","")&amp;IF(I126="","origen del agua · ","")&amp;IF(AND(LEFT(I126,7)="Sale de",J126="",K126=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C126:S126)=0,"",IF(AND(C126&lt;&gt;"",D126&lt;&gt;"",E126&lt;&gt;"",H126&lt;&gt;"",I126&lt;&gt;"",NOT(AND(LEFT(I126,7)="Sale de",J126="",K126=""))),"✔ Completa","Falta: "&amp;IF(C126="","fecha · ","")&amp;IF(D126="","ubicación · ","")&amp;IF(E126="","referencia · ","")&amp;IF(H126="","criticidad · ","")&amp;IF(I126="","origen del agua · ","")&amp;IF(AND(LEFT(I126,7)="Sale de",J126="",K126=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C126" s="17" t="n"/>
@@ -4601,8 +4747,9 @@
       <c r="N126" s="21" t="n"/>
       <c r="O126" s="21" t="n"/>
       <c r="P126" s="21" t="n"/>
-      <c r="Q126" s="18" t="n"/>
-      <c r="R126" s="19" t="n"/>
+      <c r="Q126" s="21" t="n"/>
+      <c r="R126" s="18" t="n"/>
+      <c r="S126" s="19" t="n"/>
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="15" t="inlineStr">
@@ -4611,7 +4758,7 @@
         </is>
       </c>
       <c r="B127" s="16">
-        <f>IF(COUNTA(C127:R127)=0,"",IF(AND(C127&lt;&gt;"",D127&lt;&gt;"",E127&lt;&gt;"",H127&lt;&gt;"",I127&lt;&gt;"",NOT(AND(LEFT(I127,7)="Sale de",J127="",K127=""))),"✔ Completa","Falta: "&amp;IF(C127="","fecha · ","")&amp;IF(D127="","ubicación · ","")&amp;IF(E127="","referencia · ","")&amp;IF(H127="","criticidad · ","")&amp;IF(I127="","origen del agua · ","")&amp;IF(AND(LEFT(I127,7)="Sale de",J127="",K127=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C127:S127)=0,"",IF(AND(C127&lt;&gt;"",D127&lt;&gt;"",E127&lt;&gt;"",H127&lt;&gt;"",I127&lt;&gt;"",NOT(AND(LEFT(I127,7)="Sale de",J127="",K127=""))),"✔ Completa","Falta: "&amp;IF(C127="","fecha · ","")&amp;IF(D127="","ubicación · ","")&amp;IF(E127="","referencia · ","")&amp;IF(H127="","criticidad · ","")&amp;IF(I127="","origen del agua · ","")&amp;IF(AND(LEFT(I127,7)="Sale de",J127="",K127=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C127" s="17" t="n"/>
@@ -4628,8 +4775,9 @@
       <c r="N127" s="21" t="n"/>
       <c r="O127" s="21" t="n"/>
       <c r="P127" s="21" t="n"/>
-      <c r="Q127" s="18" t="n"/>
-      <c r="R127" s="19" t="n"/>
+      <c r="Q127" s="21" t="n"/>
+      <c r="R127" s="18" t="n"/>
+      <c r="S127" s="19" t="n"/>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="15" t="inlineStr">
@@ -4638,7 +4786,7 @@
         </is>
       </c>
       <c r="B128" s="16">
-        <f>IF(COUNTA(C128:R128)=0,"",IF(AND(C128&lt;&gt;"",D128&lt;&gt;"",E128&lt;&gt;"",H128&lt;&gt;"",I128&lt;&gt;"",NOT(AND(LEFT(I128,7)="Sale de",J128="",K128=""))),"✔ Completa","Falta: "&amp;IF(C128="","fecha · ","")&amp;IF(D128="","ubicación · ","")&amp;IF(E128="","referencia · ","")&amp;IF(H128="","criticidad · ","")&amp;IF(I128="","origen del agua · ","")&amp;IF(AND(LEFT(I128,7)="Sale de",J128="",K128=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C128:S128)=0,"",IF(AND(C128&lt;&gt;"",D128&lt;&gt;"",E128&lt;&gt;"",H128&lt;&gt;"",I128&lt;&gt;"",NOT(AND(LEFT(I128,7)="Sale de",J128="",K128=""))),"✔ Completa","Falta: "&amp;IF(C128="","fecha · ","")&amp;IF(D128="","ubicación · ","")&amp;IF(E128="","referencia · ","")&amp;IF(H128="","criticidad · ","")&amp;IF(I128="","origen del agua · ","")&amp;IF(AND(LEFT(I128,7)="Sale de",J128="",K128=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C128" s="17" t="n"/>
@@ -4655,8 +4803,9 @@
       <c r="N128" s="21" t="n"/>
       <c r="O128" s="21" t="n"/>
       <c r="P128" s="21" t="n"/>
-      <c r="Q128" s="18" t="n"/>
-      <c r="R128" s="19" t="n"/>
+      <c r="Q128" s="21" t="n"/>
+      <c r="R128" s="18" t="n"/>
+      <c r="S128" s="19" t="n"/>
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="15" t="inlineStr">
@@ -4665,7 +4814,7 @@
         </is>
       </c>
       <c r="B129" s="16">
-        <f>IF(COUNTA(C129:R129)=0,"",IF(AND(C129&lt;&gt;"",D129&lt;&gt;"",E129&lt;&gt;"",H129&lt;&gt;"",I129&lt;&gt;"",NOT(AND(LEFT(I129,7)="Sale de",J129="",K129=""))),"✔ Completa","Falta: "&amp;IF(C129="","fecha · ","")&amp;IF(D129="","ubicación · ","")&amp;IF(E129="","referencia · ","")&amp;IF(H129="","criticidad · ","")&amp;IF(I129="","origen del agua · ","")&amp;IF(AND(LEFT(I129,7)="Sale de",J129="",K129=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C129:S129)=0,"",IF(AND(C129&lt;&gt;"",D129&lt;&gt;"",E129&lt;&gt;"",H129&lt;&gt;"",I129&lt;&gt;"",NOT(AND(LEFT(I129,7)="Sale de",J129="",K129=""))),"✔ Completa","Falta: "&amp;IF(C129="","fecha · ","")&amp;IF(D129="","ubicación · ","")&amp;IF(E129="","referencia · ","")&amp;IF(H129="","criticidad · ","")&amp;IF(I129="","origen del agua · ","")&amp;IF(AND(LEFT(I129,7)="Sale de",J129="",K129=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C129" s="17" t="n"/>
@@ -4682,8 +4831,9 @@
       <c r="N129" s="21" t="n"/>
       <c r="O129" s="21" t="n"/>
       <c r="P129" s="21" t="n"/>
-      <c r="Q129" s="18" t="n"/>
-      <c r="R129" s="19" t="n"/>
+      <c r="Q129" s="21" t="n"/>
+      <c r="R129" s="18" t="n"/>
+      <c r="S129" s="19" t="n"/>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="15" t="inlineStr">
@@ -4692,7 +4842,7 @@
         </is>
       </c>
       <c r="B130" s="16">
-        <f>IF(COUNTA(C130:R130)=0,"",IF(AND(C130&lt;&gt;"",D130&lt;&gt;"",E130&lt;&gt;"",H130&lt;&gt;"",I130&lt;&gt;"",NOT(AND(LEFT(I130,7)="Sale de",J130="",K130=""))),"✔ Completa","Falta: "&amp;IF(C130="","fecha · ","")&amp;IF(D130="","ubicación · ","")&amp;IF(E130="","referencia · ","")&amp;IF(H130="","criticidad · ","")&amp;IF(I130="","origen del agua · ","")&amp;IF(AND(LEFT(I130,7)="Sale de",J130="",K130=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C130:S130)=0,"",IF(AND(C130&lt;&gt;"",D130&lt;&gt;"",E130&lt;&gt;"",H130&lt;&gt;"",I130&lt;&gt;"",NOT(AND(LEFT(I130,7)="Sale de",J130="",K130=""))),"✔ Completa","Falta: "&amp;IF(C130="","fecha · ","")&amp;IF(D130="","ubicación · ","")&amp;IF(E130="","referencia · ","")&amp;IF(H130="","criticidad · ","")&amp;IF(I130="","origen del agua · ","")&amp;IF(AND(LEFT(I130,7)="Sale de",J130="",K130=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C130" s="17" t="n"/>
@@ -4709,8 +4859,9 @@
       <c r="N130" s="21" t="n"/>
       <c r="O130" s="21" t="n"/>
       <c r="P130" s="21" t="n"/>
-      <c r="Q130" s="18" t="n"/>
-      <c r="R130" s="19" t="n"/>
+      <c r="Q130" s="21" t="n"/>
+      <c r="R130" s="18" t="n"/>
+      <c r="S130" s="19" t="n"/>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="15" t="inlineStr">
@@ -4719,7 +4870,7 @@
         </is>
       </c>
       <c r="B131" s="16">
-        <f>IF(COUNTA(C131:R131)=0,"",IF(AND(C131&lt;&gt;"",D131&lt;&gt;"",E131&lt;&gt;"",H131&lt;&gt;"",I131&lt;&gt;"",NOT(AND(LEFT(I131,7)="Sale de",J131="",K131=""))),"✔ Completa","Falta: "&amp;IF(C131="","fecha · ","")&amp;IF(D131="","ubicación · ","")&amp;IF(E131="","referencia · ","")&amp;IF(H131="","criticidad · ","")&amp;IF(I131="","origen del agua · ","")&amp;IF(AND(LEFT(I131,7)="Sale de",J131="",K131=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C131:S131)=0,"",IF(AND(C131&lt;&gt;"",D131&lt;&gt;"",E131&lt;&gt;"",H131&lt;&gt;"",I131&lt;&gt;"",NOT(AND(LEFT(I131,7)="Sale de",J131="",K131=""))),"✔ Completa","Falta: "&amp;IF(C131="","fecha · ","")&amp;IF(D131="","ubicación · ","")&amp;IF(E131="","referencia · ","")&amp;IF(H131="","criticidad · ","")&amp;IF(I131="","origen del agua · ","")&amp;IF(AND(LEFT(I131,7)="Sale de",J131="",K131=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C131" s="17" t="n"/>
@@ -4736,8 +4887,9 @@
       <c r="N131" s="21" t="n"/>
       <c r="O131" s="21" t="n"/>
       <c r="P131" s="21" t="n"/>
-      <c r="Q131" s="18" t="n"/>
-      <c r="R131" s="19" t="n"/>
+      <c r="Q131" s="21" t="n"/>
+      <c r="R131" s="18" t="n"/>
+      <c r="S131" s="19" t="n"/>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="15" t="inlineStr">
@@ -4746,7 +4898,7 @@
         </is>
       </c>
       <c r="B132" s="16">
-        <f>IF(COUNTA(C132:R132)=0,"",IF(AND(C132&lt;&gt;"",D132&lt;&gt;"",E132&lt;&gt;"",H132&lt;&gt;"",I132&lt;&gt;"",NOT(AND(LEFT(I132,7)="Sale de",J132="",K132=""))),"✔ Completa","Falta: "&amp;IF(C132="","fecha · ","")&amp;IF(D132="","ubicación · ","")&amp;IF(E132="","referencia · ","")&amp;IF(H132="","criticidad · ","")&amp;IF(I132="","origen del agua · ","")&amp;IF(AND(LEFT(I132,7)="Sale de",J132="",K132=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C132:S132)=0,"",IF(AND(C132&lt;&gt;"",D132&lt;&gt;"",E132&lt;&gt;"",H132&lt;&gt;"",I132&lt;&gt;"",NOT(AND(LEFT(I132,7)="Sale de",J132="",K132=""))),"✔ Completa","Falta: "&amp;IF(C132="","fecha · ","")&amp;IF(D132="","ubicación · ","")&amp;IF(E132="","referencia · ","")&amp;IF(H132="","criticidad · ","")&amp;IF(I132="","origen del agua · ","")&amp;IF(AND(LEFT(I132,7)="Sale de",J132="",K132=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C132" s="17" t="n"/>
@@ -4763,8 +4915,9 @@
       <c r="N132" s="21" t="n"/>
       <c r="O132" s="21" t="n"/>
       <c r="P132" s="21" t="n"/>
-      <c r="Q132" s="18" t="n"/>
-      <c r="R132" s="19" t="n"/>
+      <c r="Q132" s="21" t="n"/>
+      <c r="R132" s="18" t="n"/>
+      <c r="S132" s="19" t="n"/>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="15" t="inlineStr">
@@ -4773,7 +4926,7 @@
         </is>
       </c>
       <c r="B133" s="16">
-        <f>IF(COUNTA(C133:R133)=0,"",IF(AND(C133&lt;&gt;"",D133&lt;&gt;"",E133&lt;&gt;"",H133&lt;&gt;"",I133&lt;&gt;"",NOT(AND(LEFT(I133,7)="Sale de",J133="",K133=""))),"✔ Completa","Falta: "&amp;IF(C133="","fecha · ","")&amp;IF(D133="","ubicación · ","")&amp;IF(E133="","referencia · ","")&amp;IF(H133="","criticidad · ","")&amp;IF(I133="","origen del agua · ","")&amp;IF(AND(LEFT(I133,7)="Sale de",J133="",K133=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C133:S133)=0,"",IF(AND(C133&lt;&gt;"",D133&lt;&gt;"",E133&lt;&gt;"",H133&lt;&gt;"",I133&lt;&gt;"",NOT(AND(LEFT(I133,7)="Sale de",J133="",K133=""))),"✔ Completa","Falta: "&amp;IF(C133="","fecha · ","")&amp;IF(D133="","ubicación · ","")&amp;IF(E133="","referencia · ","")&amp;IF(H133="","criticidad · ","")&amp;IF(I133="","origen del agua · ","")&amp;IF(AND(LEFT(I133,7)="Sale de",J133="",K133=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C133" s="17" t="n"/>
@@ -4790,8 +4943,9 @@
       <c r="N133" s="21" t="n"/>
       <c r="O133" s="21" t="n"/>
       <c r="P133" s="21" t="n"/>
-      <c r="Q133" s="18" t="n"/>
-      <c r="R133" s="19" t="n"/>
+      <c r="Q133" s="21" t="n"/>
+      <c r="R133" s="18" t="n"/>
+      <c r="S133" s="19" t="n"/>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="15" t="inlineStr">
@@ -4800,7 +4954,7 @@
         </is>
       </c>
       <c r="B134" s="16">
-        <f>IF(COUNTA(C134:R134)=0,"",IF(AND(C134&lt;&gt;"",D134&lt;&gt;"",E134&lt;&gt;"",H134&lt;&gt;"",I134&lt;&gt;"",NOT(AND(LEFT(I134,7)="Sale de",J134="",K134=""))),"✔ Completa","Falta: "&amp;IF(C134="","fecha · ","")&amp;IF(D134="","ubicación · ","")&amp;IF(E134="","referencia · ","")&amp;IF(H134="","criticidad · ","")&amp;IF(I134="","origen del agua · ","")&amp;IF(AND(LEFT(I134,7)="Sale de",J134="",K134=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C134:S134)=0,"",IF(AND(C134&lt;&gt;"",D134&lt;&gt;"",E134&lt;&gt;"",H134&lt;&gt;"",I134&lt;&gt;"",NOT(AND(LEFT(I134,7)="Sale de",J134="",K134=""))),"✔ Completa","Falta: "&amp;IF(C134="","fecha · ","")&amp;IF(D134="","ubicación · ","")&amp;IF(E134="","referencia · ","")&amp;IF(H134="","criticidad · ","")&amp;IF(I134="","origen del agua · ","")&amp;IF(AND(LEFT(I134,7)="Sale de",J134="",K134=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C134" s="17" t="n"/>
@@ -4817,8 +4971,9 @@
       <c r="N134" s="21" t="n"/>
       <c r="O134" s="21" t="n"/>
       <c r="P134" s="21" t="n"/>
-      <c r="Q134" s="18" t="n"/>
-      <c r="R134" s="19" t="n"/>
+      <c r="Q134" s="21" t="n"/>
+      <c r="R134" s="18" t="n"/>
+      <c r="S134" s="19" t="n"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="15" t="inlineStr">
@@ -4827,7 +4982,7 @@
         </is>
       </c>
       <c r="B135" s="16">
-        <f>IF(COUNTA(C135:R135)=0,"",IF(AND(C135&lt;&gt;"",D135&lt;&gt;"",E135&lt;&gt;"",H135&lt;&gt;"",I135&lt;&gt;"",NOT(AND(LEFT(I135,7)="Sale de",J135="",K135=""))),"✔ Completa","Falta: "&amp;IF(C135="","fecha · ","")&amp;IF(D135="","ubicación · ","")&amp;IF(E135="","referencia · ","")&amp;IF(H135="","criticidad · ","")&amp;IF(I135="","origen del agua · ","")&amp;IF(AND(LEFT(I135,7)="Sale de",J135="",K135=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C135:S135)=0,"",IF(AND(C135&lt;&gt;"",D135&lt;&gt;"",E135&lt;&gt;"",H135&lt;&gt;"",I135&lt;&gt;"",NOT(AND(LEFT(I135,7)="Sale de",J135="",K135=""))),"✔ Completa","Falta: "&amp;IF(C135="","fecha · ","")&amp;IF(D135="","ubicación · ","")&amp;IF(E135="","referencia · ","")&amp;IF(H135="","criticidad · ","")&amp;IF(I135="","origen del agua · ","")&amp;IF(AND(LEFT(I135,7)="Sale de",J135="",K135=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C135" s="17" t="n"/>
@@ -4844,8 +4999,9 @@
       <c r="N135" s="21" t="n"/>
       <c r="O135" s="21" t="n"/>
       <c r="P135" s="21" t="n"/>
-      <c r="Q135" s="18" t="n"/>
-      <c r="R135" s="19" t="n"/>
+      <c r="Q135" s="21" t="n"/>
+      <c r="R135" s="18" t="n"/>
+      <c r="S135" s="19" t="n"/>
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="15" t="inlineStr">
@@ -4854,7 +5010,7 @@
         </is>
       </c>
       <c r="B136" s="16">
-        <f>IF(COUNTA(C136:R136)=0,"",IF(AND(C136&lt;&gt;"",D136&lt;&gt;"",E136&lt;&gt;"",H136&lt;&gt;"",I136&lt;&gt;"",NOT(AND(LEFT(I136,7)="Sale de",J136="",K136=""))),"✔ Completa","Falta: "&amp;IF(C136="","fecha · ","")&amp;IF(D136="","ubicación · ","")&amp;IF(E136="","referencia · ","")&amp;IF(H136="","criticidad · ","")&amp;IF(I136="","origen del agua · ","")&amp;IF(AND(LEFT(I136,7)="Sale de",J136="",K136=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C136:S136)=0,"",IF(AND(C136&lt;&gt;"",D136&lt;&gt;"",E136&lt;&gt;"",H136&lt;&gt;"",I136&lt;&gt;"",NOT(AND(LEFT(I136,7)="Sale de",J136="",K136=""))),"✔ Completa","Falta: "&amp;IF(C136="","fecha · ","")&amp;IF(D136="","ubicación · ","")&amp;IF(E136="","referencia · ","")&amp;IF(H136="","criticidad · ","")&amp;IF(I136="","origen del agua · ","")&amp;IF(AND(LEFT(I136,7)="Sale de",J136="",K136=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C136" s="17" t="n"/>
@@ -4871,8 +5027,9 @@
       <c r="N136" s="21" t="n"/>
       <c r="O136" s="21" t="n"/>
       <c r="P136" s="21" t="n"/>
-      <c r="Q136" s="18" t="n"/>
-      <c r="R136" s="19" t="n"/>
+      <c r="Q136" s="21" t="n"/>
+      <c r="R136" s="18" t="n"/>
+      <c r="S136" s="19" t="n"/>
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="15" t="inlineStr">
@@ -4881,7 +5038,7 @@
         </is>
       </c>
       <c r="B137" s="16">
-        <f>IF(COUNTA(C137:R137)=0,"",IF(AND(C137&lt;&gt;"",D137&lt;&gt;"",E137&lt;&gt;"",H137&lt;&gt;"",I137&lt;&gt;"",NOT(AND(LEFT(I137,7)="Sale de",J137="",K137=""))),"✔ Completa","Falta: "&amp;IF(C137="","fecha · ","")&amp;IF(D137="","ubicación · ","")&amp;IF(E137="","referencia · ","")&amp;IF(H137="","criticidad · ","")&amp;IF(I137="","origen del agua · ","")&amp;IF(AND(LEFT(I137,7)="Sale de",J137="",K137=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C137:S137)=0,"",IF(AND(C137&lt;&gt;"",D137&lt;&gt;"",E137&lt;&gt;"",H137&lt;&gt;"",I137&lt;&gt;"",NOT(AND(LEFT(I137,7)="Sale de",J137="",K137=""))),"✔ Completa","Falta: "&amp;IF(C137="","fecha · ","")&amp;IF(D137="","ubicación · ","")&amp;IF(E137="","referencia · ","")&amp;IF(H137="","criticidad · ","")&amp;IF(I137="","origen del agua · ","")&amp;IF(AND(LEFT(I137,7)="Sale de",J137="",K137=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C137" s="17" t="n"/>
@@ -4898,8 +5055,9 @@
       <c r="N137" s="21" t="n"/>
       <c r="O137" s="21" t="n"/>
       <c r="P137" s="21" t="n"/>
-      <c r="Q137" s="18" t="n"/>
-      <c r="R137" s="19" t="n"/>
+      <c r="Q137" s="21" t="n"/>
+      <c r="R137" s="18" t="n"/>
+      <c r="S137" s="19" t="n"/>
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="15" t="inlineStr">
@@ -4908,7 +5066,7 @@
         </is>
       </c>
       <c r="B138" s="16">
-        <f>IF(COUNTA(C138:R138)=0,"",IF(AND(C138&lt;&gt;"",D138&lt;&gt;"",E138&lt;&gt;"",H138&lt;&gt;"",I138&lt;&gt;"",NOT(AND(LEFT(I138,7)="Sale de",J138="",K138=""))),"✔ Completa","Falta: "&amp;IF(C138="","fecha · ","")&amp;IF(D138="","ubicación · ","")&amp;IF(E138="","referencia · ","")&amp;IF(H138="","criticidad · ","")&amp;IF(I138="","origen del agua · ","")&amp;IF(AND(LEFT(I138,7)="Sale de",J138="",K138=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C138:S138)=0,"",IF(AND(C138&lt;&gt;"",D138&lt;&gt;"",E138&lt;&gt;"",H138&lt;&gt;"",I138&lt;&gt;"",NOT(AND(LEFT(I138,7)="Sale de",J138="",K138=""))),"✔ Completa","Falta: "&amp;IF(C138="","fecha · ","")&amp;IF(D138="","ubicación · ","")&amp;IF(E138="","referencia · ","")&amp;IF(H138="","criticidad · ","")&amp;IF(I138="","origen del agua · ","")&amp;IF(AND(LEFT(I138,7)="Sale de",J138="",K138=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C138" s="17" t="n"/>
@@ -4925,8 +5083,9 @@
       <c r="N138" s="21" t="n"/>
       <c r="O138" s="21" t="n"/>
       <c r="P138" s="21" t="n"/>
-      <c r="Q138" s="18" t="n"/>
-      <c r="R138" s="19" t="n"/>
+      <c r="Q138" s="21" t="n"/>
+      <c r="R138" s="18" t="n"/>
+      <c r="S138" s="19" t="n"/>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="15" t="inlineStr">
@@ -4935,7 +5094,7 @@
         </is>
       </c>
       <c r="B139" s="16">
-        <f>IF(COUNTA(C139:R139)=0,"",IF(AND(C139&lt;&gt;"",D139&lt;&gt;"",E139&lt;&gt;"",H139&lt;&gt;"",I139&lt;&gt;"",NOT(AND(LEFT(I139,7)="Sale de",J139="",K139=""))),"✔ Completa","Falta: "&amp;IF(C139="","fecha · ","")&amp;IF(D139="","ubicación · ","")&amp;IF(E139="","referencia · ","")&amp;IF(H139="","criticidad · ","")&amp;IF(I139="","origen del agua · ","")&amp;IF(AND(LEFT(I139,7)="Sale de",J139="",K139=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C139:S139)=0,"",IF(AND(C139&lt;&gt;"",D139&lt;&gt;"",E139&lt;&gt;"",H139&lt;&gt;"",I139&lt;&gt;"",NOT(AND(LEFT(I139,7)="Sale de",J139="",K139=""))),"✔ Completa","Falta: "&amp;IF(C139="","fecha · ","")&amp;IF(D139="","ubicación · ","")&amp;IF(E139="","referencia · ","")&amp;IF(H139="","criticidad · ","")&amp;IF(I139="","origen del agua · ","")&amp;IF(AND(LEFT(I139,7)="Sale de",J139="",K139=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C139" s="17" t="n"/>
@@ -4952,8 +5111,9 @@
       <c r="N139" s="21" t="n"/>
       <c r="O139" s="21" t="n"/>
       <c r="P139" s="21" t="n"/>
-      <c r="Q139" s="18" t="n"/>
-      <c r="R139" s="19" t="n"/>
+      <c r="Q139" s="21" t="n"/>
+      <c r="R139" s="18" t="n"/>
+      <c r="S139" s="19" t="n"/>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="15" t="inlineStr">
@@ -4962,7 +5122,7 @@
         </is>
       </c>
       <c r="B140" s="16">
-        <f>IF(COUNTA(C140:R140)=0,"",IF(AND(C140&lt;&gt;"",D140&lt;&gt;"",E140&lt;&gt;"",H140&lt;&gt;"",I140&lt;&gt;"",NOT(AND(LEFT(I140,7)="Sale de",J140="",K140=""))),"✔ Completa","Falta: "&amp;IF(C140="","fecha · ","")&amp;IF(D140="","ubicación · ","")&amp;IF(E140="","referencia · ","")&amp;IF(H140="","criticidad · ","")&amp;IF(I140="","origen del agua · ","")&amp;IF(AND(LEFT(I140,7)="Sale de",J140="",K140=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C140:S140)=0,"",IF(AND(C140&lt;&gt;"",D140&lt;&gt;"",E140&lt;&gt;"",H140&lt;&gt;"",I140&lt;&gt;"",NOT(AND(LEFT(I140,7)="Sale de",J140="",K140=""))),"✔ Completa","Falta: "&amp;IF(C140="","fecha · ","")&amp;IF(D140="","ubicación · ","")&amp;IF(E140="","referencia · ","")&amp;IF(H140="","criticidad · ","")&amp;IF(I140="","origen del agua · ","")&amp;IF(AND(LEFT(I140,7)="Sale de",J140="",K140=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C140" s="17" t="n"/>
@@ -4979,8 +5139,9 @@
       <c r="N140" s="21" t="n"/>
       <c r="O140" s="21" t="n"/>
       <c r="P140" s="21" t="n"/>
-      <c r="Q140" s="18" t="n"/>
-      <c r="R140" s="19" t="n"/>
+      <c r="Q140" s="21" t="n"/>
+      <c r="R140" s="18" t="n"/>
+      <c r="S140" s="19" t="n"/>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="15" t="inlineStr">
@@ -4989,7 +5150,7 @@
         </is>
       </c>
       <c r="B141" s="16">
-        <f>IF(COUNTA(C141:R141)=0,"",IF(AND(C141&lt;&gt;"",D141&lt;&gt;"",E141&lt;&gt;"",H141&lt;&gt;"",I141&lt;&gt;"",NOT(AND(LEFT(I141,7)="Sale de",J141="",K141=""))),"✔ Completa","Falta: "&amp;IF(C141="","fecha · ","")&amp;IF(D141="","ubicación · ","")&amp;IF(E141="","referencia · ","")&amp;IF(H141="","criticidad · ","")&amp;IF(I141="","origen del agua · ","")&amp;IF(AND(LEFT(I141,7)="Sale de",J141="",K141=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C141:S141)=0,"",IF(AND(C141&lt;&gt;"",D141&lt;&gt;"",E141&lt;&gt;"",H141&lt;&gt;"",I141&lt;&gt;"",NOT(AND(LEFT(I141,7)="Sale de",J141="",K141=""))),"✔ Completa","Falta: "&amp;IF(C141="","fecha · ","")&amp;IF(D141="","ubicación · ","")&amp;IF(E141="","referencia · ","")&amp;IF(H141="","criticidad · ","")&amp;IF(I141="","origen del agua · ","")&amp;IF(AND(LEFT(I141,7)="Sale de",J141="",K141=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C141" s="17" t="n"/>
@@ -5006,8 +5167,9 @@
       <c r="N141" s="21" t="n"/>
       <c r="O141" s="21" t="n"/>
       <c r="P141" s="21" t="n"/>
-      <c r="Q141" s="18" t="n"/>
-      <c r="R141" s="19" t="n"/>
+      <c r="Q141" s="21" t="n"/>
+      <c r="R141" s="18" t="n"/>
+      <c r="S141" s="19" t="n"/>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="15" t="inlineStr">
@@ -5016,7 +5178,7 @@
         </is>
       </c>
       <c r="B142" s="16">
-        <f>IF(COUNTA(C142:R142)=0,"",IF(AND(C142&lt;&gt;"",D142&lt;&gt;"",E142&lt;&gt;"",H142&lt;&gt;"",I142&lt;&gt;"",NOT(AND(LEFT(I142,7)="Sale de",J142="",K142=""))),"✔ Completa","Falta: "&amp;IF(C142="","fecha · ","")&amp;IF(D142="","ubicación · ","")&amp;IF(E142="","referencia · ","")&amp;IF(H142="","criticidad · ","")&amp;IF(I142="","origen del agua · ","")&amp;IF(AND(LEFT(I142,7)="Sale de",J142="",K142=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C142:S142)=0,"",IF(AND(C142&lt;&gt;"",D142&lt;&gt;"",E142&lt;&gt;"",H142&lt;&gt;"",I142&lt;&gt;"",NOT(AND(LEFT(I142,7)="Sale de",J142="",K142=""))),"✔ Completa","Falta: "&amp;IF(C142="","fecha · ","")&amp;IF(D142="","ubicación · ","")&amp;IF(E142="","referencia · ","")&amp;IF(H142="","criticidad · ","")&amp;IF(I142="","origen del agua · ","")&amp;IF(AND(LEFT(I142,7)="Sale de",J142="",K142=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C142" s="17" t="n"/>
@@ -5033,8 +5195,9 @@
       <c r="N142" s="21" t="n"/>
       <c r="O142" s="21" t="n"/>
       <c r="P142" s="21" t="n"/>
-      <c r="Q142" s="18" t="n"/>
-      <c r="R142" s="19" t="n"/>
+      <c r="Q142" s="21" t="n"/>
+      <c r="R142" s="18" t="n"/>
+      <c r="S142" s="19" t="n"/>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="15" t="inlineStr">
@@ -5043,7 +5206,7 @@
         </is>
       </c>
       <c r="B143" s="16">
-        <f>IF(COUNTA(C143:R143)=0,"",IF(AND(C143&lt;&gt;"",D143&lt;&gt;"",E143&lt;&gt;"",H143&lt;&gt;"",I143&lt;&gt;"",NOT(AND(LEFT(I143,7)="Sale de",J143="",K143=""))),"✔ Completa","Falta: "&amp;IF(C143="","fecha · ","")&amp;IF(D143="","ubicación · ","")&amp;IF(E143="","referencia · ","")&amp;IF(H143="","criticidad · ","")&amp;IF(I143="","origen del agua · ","")&amp;IF(AND(LEFT(I143,7)="Sale de",J143="",K143=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C143:S143)=0,"",IF(AND(C143&lt;&gt;"",D143&lt;&gt;"",E143&lt;&gt;"",H143&lt;&gt;"",I143&lt;&gt;"",NOT(AND(LEFT(I143,7)="Sale de",J143="",K143=""))),"✔ Completa","Falta: "&amp;IF(C143="","fecha · ","")&amp;IF(D143="","ubicación · ","")&amp;IF(E143="","referencia · ","")&amp;IF(H143="","criticidad · ","")&amp;IF(I143="","origen del agua · ","")&amp;IF(AND(LEFT(I143,7)="Sale de",J143="",K143=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C143" s="17" t="n"/>
@@ -5060,8 +5223,9 @@
       <c r="N143" s="21" t="n"/>
       <c r="O143" s="21" t="n"/>
       <c r="P143" s="21" t="n"/>
-      <c r="Q143" s="18" t="n"/>
-      <c r="R143" s="19" t="n"/>
+      <c r="Q143" s="21" t="n"/>
+      <c r="R143" s="18" t="n"/>
+      <c r="S143" s="19" t="n"/>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="15" t="inlineStr">
@@ -5070,7 +5234,7 @@
         </is>
       </c>
       <c r="B144" s="16">
-        <f>IF(COUNTA(C144:R144)=0,"",IF(AND(C144&lt;&gt;"",D144&lt;&gt;"",E144&lt;&gt;"",H144&lt;&gt;"",I144&lt;&gt;"",NOT(AND(LEFT(I144,7)="Sale de",J144="",K144=""))),"✔ Completa","Falta: "&amp;IF(C144="","fecha · ","")&amp;IF(D144="","ubicación · ","")&amp;IF(E144="","referencia · ","")&amp;IF(H144="","criticidad · ","")&amp;IF(I144="","origen del agua · ","")&amp;IF(AND(LEFT(I144,7)="Sale de",J144="",K144=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C144:S144)=0,"",IF(AND(C144&lt;&gt;"",D144&lt;&gt;"",E144&lt;&gt;"",H144&lt;&gt;"",I144&lt;&gt;"",NOT(AND(LEFT(I144,7)="Sale de",J144="",K144=""))),"✔ Completa","Falta: "&amp;IF(C144="","fecha · ","")&amp;IF(D144="","ubicación · ","")&amp;IF(E144="","referencia · ","")&amp;IF(H144="","criticidad · ","")&amp;IF(I144="","origen del agua · ","")&amp;IF(AND(LEFT(I144,7)="Sale de",J144="",K144=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C144" s="17" t="n"/>
@@ -5087,8 +5251,9 @@
       <c r="N144" s="21" t="n"/>
       <c r="O144" s="21" t="n"/>
       <c r="P144" s="21" t="n"/>
-      <c r="Q144" s="18" t="n"/>
-      <c r="R144" s="19" t="n"/>
+      <c r="Q144" s="21" t="n"/>
+      <c r="R144" s="18" t="n"/>
+      <c r="S144" s="19" t="n"/>
     </row>
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="15" t="inlineStr">
@@ -5097,7 +5262,7 @@
         </is>
       </c>
       <c r="B145" s="16">
-        <f>IF(COUNTA(C145:R145)=0,"",IF(AND(C145&lt;&gt;"",D145&lt;&gt;"",E145&lt;&gt;"",H145&lt;&gt;"",I145&lt;&gt;"",NOT(AND(LEFT(I145,7)="Sale de",J145="",K145=""))),"✔ Completa","Falta: "&amp;IF(C145="","fecha · ","")&amp;IF(D145="","ubicación · ","")&amp;IF(E145="","referencia · ","")&amp;IF(H145="","criticidad · ","")&amp;IF(I145="","origen del agua · ","")&amp;IF(AND(LEFT(I145,7)="Sale de",J145="",K145=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C145:S145)=0,"",IF(AND(C145&lt;&gt;"",D145&lt;&gt;"",E145&lt;&gt;"",H145&lt;&gt;"",I145&lt;&gt;"",NOT(AND(LEFT(I145,7)="Sale de",J145="",K145=""))),"✔ Completa","Falta: "&amp;IF(C145="","fecha · ","")&amp;IF(D145="","ubicación · ","")&amp;IF(E145="","referencia · ","")&amp;IF(H145="","criticidad · ","")&amp;IF(I145="","origen del agua · ","")&amp;IF(AND(LEFT(I145,7)="Sale de",J145="",K145=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C145" s="17" t="n"/>
@@ -5114,8 +5279,9 @@
       <c r="N145" s="21" t="n"/>
       <c r="O145" s="21" t="n"/>
       <c r="P145" s="21" t="n"/>
-      <c r="Q145" s="18" t="n"/>
-      <c r="R145" s="19" t="n"/>
+      <c r="Q145" s="21" t="n"/>
+      <c r="R145" s="18" t="n"/>
+      <c r="S145" s="19" t="n"/>
     </row>
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="15" t="inlineStr">
@@ -5124,7 +5290,7 @@
         </is>
       </c>
       <c r="B146" s="16">
-        <f>IF(COUNTA(C146:R146)=0,"",IF(AND(C146&lt;&gt;"",D146&lt;&gt;"",E146&lt;&gt;"",H146&lt;&gt;"",I146&lt;&gt;"",NOT(AND(LEFT(I146,7)="Sale de",J146="",K146=""))),"✔ Completa","Falta: "&amp;IF(C146="","fecha · ","")&amp;IF(D146="","ubicación · ","")&amp;IF(E146="","referencia · ","")&amp;IF(H146="","criticidad · ","")&amp;IF(I146="","origen del agua · ","")&amp;IF(AND(LEFT(I146,7)="Sale de",J146="",K146=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C146:S146)=0,"",IF(AND(C146&lt;&gt;"",D146&lt;&gt;"",E146&lt;&gt;"",H146&lt;&gt;"",I146&lt;&gt;"",NOT(AND(LEFT(I146,7)="Sale de",J146="",K146=""))),"✔ Completa","Falta: "&amp;IF(C146="","fecha · ","")&amp;IF(D146="","ubicación · ","")&amp;IF(E146="","referencia · ","")&amp;IF(H146="","criticidad · ","")&amp;IF(I146="","origen del agua · ","")&amp;IF(AND(LEFT(I146,7)="Sale de",J146="",K146=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C146" s="17" t="n"/>
@@ -5141,8 +5307,9 @@
       <c r="N146" s="21" t="n"/>
       <c r="O146" s="21" t="n"/>
       <c r="P146" s="21" t="n"/>
-      <c r="Q146" s="18" t="n"/>
-      <c r="R146" s="19" t="n"/>
+      <c r="Q146" s="21" t="n"/>
+      <c r="R146" s="18" t="n"/>
+      <c r="S146" s="19" t="n"/>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="15" t="inlineStr">
@@ -5151,7 +5318,7 @@
         </is>
       </c>
       <c r="B147" s="16">
-        <f>IF(COUNTA(C147:R147)=0,"",IF(AND(C147&lt;&gt;"",D147&lt;&gt;"",E147&lt;&gt;"",H147&lt;&gt;"",I147&lt;&gt;"",NOT(AND(LEFT(I147,7)="Sale de",J147="",K147=""))),"✔ Completa","Falta: "&amp;IF(C147="","fecha · ","")&amp;IF(D147="","ubicación · ","")&amp;IF(E147="","referencia · ","")&amp;IF(H147="","criticidad · ","")&amp;IF(I147="","origen del agua · ","")&amp;IF(AND(LEFT(I147,7)="Sale de",J147="",K147=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C147:S147)=0,"",IF(AND(C147&lt;&gt;"",D147&lt;&gt;"",E147&lt;&gt;"",H147&lt;&gt;"",I147&lt;&gt;"",NOT(AND(LEFT(I147,7)="Sale de",J147="",K147=""))),"✔ Completa","Falta: "&amp;IF(C147="","fecha · ","")&amp;IF(D147="","ubicación · ","")&amp;IF(E147="","referencia · ","")&amp;IF(H147="","criticidad · ","")&amp;IF(I147="","origen del agua · ","")&amp;IF(AND(LEFT(I147,7)="Sale de",J147="",K147=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C147" s="17" t="n"/>
@@ -5168,8 +5335,9 @@
       <c r="N147" s="21" t="n"/>
       <c r="O147" s="21" t="n"/>
       <c r="P147" s="21" t="n"/>
-      <c r="Q147" s="18" t="n"/>
-      <c r="R147" s="19" t="n"/>
+      <c r="Q147" s="21" t="n"/>
+      <c r="R147" s="18" t="n"/>
+      <c r="S147" s="19" t="n"/>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="15" t="inlineStr">
@@ -5178,7 +5346,7 @@
         </is>
       </c>
       <c r="B148" s="16">
-        <f>IF(COUNTA(C148:R148)=0,"",IF(AND(C148&lt;&gt;"",D148&lt;&gt;"",E148&lt;&gt;"",H148&lt;&gt;"",I148&lt;&gt;"",NOT(AND(LEFT(I148,7)="Sale de",J148="",K148=""))),"✔ Completa","Falta: "&amp;IF(C148="","fecha · ","")&amp;IF(D148="","ubicación · ","")&amp;IF(E148="","referencia · ","")&amp;IF(H148="","criticidad · ","")&amp;IF(I148="","origen del agua · ","")&amp;IF(AND(LEFT(I148,7)="Sale de",J148="",K148=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C148:S148)=0,"",IF(AND(C148&lt;&gt;"",D148&lt;&gt;"",E148&lt;&gt;"",H148&lt;&gt;"",I148&lt;&gt;"",NOT(AND(LEFT(I148,7)="Sale de",J148="",K148=""))),"✔ Completa","Falta: "&amp;IF(C148="","fecha · ","")&amp;IF(D148="","ubicación · ","")&amp;IF(E148="","referencia · ","")&amp;IF(H148="","criticidad · ","")&amp;IF(I148="","origen del agua · ","")&amp;IF(AND(LEFT(I148,7)="Sale de",J148="",K148=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C148" s="17" t="n"/>
@@ -5195,8 +5363,9 @@
       <c r="N148" s="21" t="n"/>
       <c r="O148" s="21" t="n"/>
       <c r="P148" s="21" t="n"/>
-      <c r="Q148" s="18" t="n"/>
-      <c r="R148" s="19" t="n"/>
+      <c r="Q148" s="21" t="n"/>
+      <c r="R148" s="18" t="n"/>
+      <c r="S148" s="19" t="n"/>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="15" t="inlineStr">
@@ -5205,7 +5374,7 @@
         </is>
       </c>
       <c r="B149" s="16">
-        <f>IF(COUNTA(C149:R149)=0,"",IF(AND(C149&lt;&gt;"",D149&lt;&gt;"",E149&lt;&gt;"",H149&lt;&gt;"",I149&lt;&gt;"",NOT(AND(LEFT(I149,7)="Sale de",J149="",K149=""))),"✔ Completa","Falta: "&amp;IF(C149="","fecha · ","")&amp;IF(D149="","ubicación · ","")&amp;IF(E149="","referencia · ","")&amp;IF(H149="","criticidad · ","")&amp;IF(I149="","origen del agua · ","")&amp;IF(AND(LEFT(I149,7)="Sale de",J149="",K149=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C149:S149)=0,"",IF(AND(C149&lt;&gt;"",D149&lt;&gt;"",E149&lt;&gt;"",H149&lt;&gt;"",I149&lt;&gt;"",NOT(AND(LEFT(I149,7)="Sale de",J149="",K149=""))),"✔ Completa","Falta: "&amp;IF(C149="","fecha · ","")&amp;IF(D149="","ubicación · ","")&amp;IF(E149="","referencia · ","")&amp;IF(H149="","criticidad · ","")&amp;IF(I149="","origen del agua · ","")&amp;IF(AND(LEFT(I149,7)="Sale de",J149="",K149=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C149" s="17" t="n"/>
@@ -5222,8 +5391,9 @@
       <c r="N149" s="21" t="n"/>
       <c r="O149" s="21" t="n"/>
       <c r="P149" s="21" t="n"/>
-      <c r="Q149" s="18" t="n"/>
-      <c r="R149" s="19" t="n"/>
+      <c r="Q149" s="21" t="n"/>
+      <c r="R149" s="18" t="n"/>
+      <c r="S149" s="19" t="n"/>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="15" t="inlineStr">
@@ -5232,7 +5402,7 @@
         </is>
       </c>
       <c r="B150" s="16">
-        <f>IF(COUNTA(C150:R150)=0,"",IF(AND(C150&lt;&gt;"",D150&lt;&gt;"",E150&lt;&gt;"",H150&lt;&gt;"",I150&lt;&gt;"",NOT(AND(LEFT(I150,7)="Sale de",J150="",K150=""))),"✔ Completa","Falta: "&amp;IF(C150="","fecha · ","")&amp;IF(D150="","ubicación · ","")&amp;IF(E150="","referencia · ","")&amp;IF(H150="","criticidad · ","")&amp;IF(I150="","origen del agua · ","")&amp;IF(AND(LEFT(I150,7)="Sale de",J150="",K150=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C150:S150)=0,"",IF(AND(C150&lt;&gt;"",D150&lt;&gt;"",E150&lt;&gt;"",H150&lt;&gt;"",I150&lt;&gt;"",NOT(AND(LEFT(I150,7)="Sale de",J150="",K150=""))),"✔ Completa","Falta: "&amp;IF(C150="","fecha · ","")&amp;IF(D150="","ubicación · ","")&amp;IF(E150="","referencia · ","")&amp;IF(H150="","criticidad · ","")&amp;IF(I150="","origen del agua · ","")&amp;IF(AND(LEFT(I150,7)="Sale de",J150="",K150=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C150" s="17" t="n"/>
@@ -5249,8 +5419,9 @@
       <c r="N150" s="21" t="n"/>
       <c r="O150" s="21" t="n"/>
       <c r="P150" s="21" t="n"/>
-      <c r="Q150" s="18" t="n"/>
-      <c r="R150" s="19" t="n"/>
+      <c r="Q150" s="21" t="n"/>
+      <c r="R150" s="18" t="n"/>
+      <c r="S150" s="19" t="n"/>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="15" t="inlineStr">
@@ -5259,7 +5430,7 @@
         </is>
       </c>
       <c r="B151" s="16">
-        <f>IF(COUNTA(C151:R151)=0,"",IF(AND(C151&lt;&gt;"",D151&lt;&gt;"",E151&lt;&gt;"",H151&lt;&gt;"",I151&lt;&gt;"",NOT(AND(LEFT(I151,7)="Sale de",J151="",K151=""))),"✔ Completa","Falta: "&amp;IF(C151="","fecha · ","")&amp;IF(D151="","ubicación · ","")&amp;IF(E151="","referencia · ","")&amp;IF(H151="","criticidad · ","")&amp;IF(I151="","origen del agua · ","")&amp;IF(AND(LEFT(I151,7)="Sale de",J151="",K151=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C151:S151)=0,"",IF(AND(C151&lt;&gt;"",D151&lt;&gt;"",E151&lt;&gt;"",H151&lt;&gt;"",I151&lt;&gt;"",NOT(AND(LEFT(I151,7)="Sale de",J151="",K151=""))),"✔ Completa","Falta: "&amp;IF(C151="","fecha · ","")&amp;IF(D151="","ubicación · ","")&amp;IF(E151="","referencia · ","")&amp;IF(H151="","criticidad · ","")&amp;IF(I151="","origen del agua · ","")&amp;IF(AND(LEFT(I151,7)="Sale de",J151="",K151=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C151" s="17" t="n"/>
@@ -5276,8 +5447,9 @@
       <c r="N151" s="21" t="n"/>
       <c r="O151" s="21" t="n"/>
       <c r="P151" s="21" t="n"/>
-      <c r="Q151" s="18" t="n"/>
-      <c r="R151" s="19" t="n"/>
+      <c r="Q151" s="21" t="n"/>
+      <c r="R151" s="18" t="n"/>
+      <c r="S151" s="19" t="n"/>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="15" t="inlineStr">
@@ -5286,7 +5458,7 @@
         </is>
       </c>
       <c r="B152" s="16">
-        <f>IF(COUNTA(C152:R152)=0,"",IF(AND(C152&lt;&gt;"",D152&lt;&gt;"",E152&lt;&gt;"",H152&lt;&gt;"",I152&lt;&gt;"",NOT(AND(LEFT(I152,7)="Sale de",J152="",K152=""))),"✔ Completa","Falta: "&amp;IF(C152="","fecha · ","")&amp;IF(D152="","ubicación · ","")&amp;IF(E152="","referencia · ","")&amp;IF(H152="","criticidad · ","")&amp;IF(I152="","origen del agua · ","")&amp;IF(AND(LEFT(I152,7)="Sale de",J152="",K152=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C152:S152)=0,"",IF(AND(C152&lt;&gt;"",D152&lt;&gt;"",E152&lt;&gt;"",H152&lt;&gt;"",I152&lt;&gt;"",NOT(AND(LEFT(I152,7)="Sale de",J152="",K152=""))),"✔ Completa","Falta: "&amp;IF(C152="","fecha · ","")&amp;IF(D152="","ubicación · ","")&amp;IF(E152="","referencia · ","")&amp;IF(H152="","criticidad · ","")&amp;IF(I152="","origen del agua · ","")&amp;IF(AND(LEFT(I152,7)="Sale de",J152="",K152=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C152" s="17" t="n"/>
@@ -5303,8 +5475,9 @@
       <c r="N152" s="21" t="n"/>
       <c r="O152" s="21" t="n"/>
       <c r="P152" s="21" t="n"/>
-      <c r="Q152" s="18" t="n"/>
-      <c r="R152" s="19" t="n"/>
+      <c r="Q152" s="21" t="n"/>
+      <c r="R152" s="18" t="n"/>
+      <c r="S152" s="19" t="n"/>
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="15" t="inlineStr">
@@ -5313,7 +5486,7 @@
         </is>
       </c>
       <c r="B153" s="16">
-        <f>IF(COUNTA(C153:R153)=0,"",IF(AND(C153&lt;&gt;"",D153&lt;&gt;"",E153&lt;&gt;"",H153&lt;&gt;"",I153&lt;&gt;"",NOT(AND(LEFT(I153,7)="Sale de",J153="",K153=""))),"✔ Completa","Falta: "&amp;IF(C153="","fecha · ","")&amp;IF(D153="","ubicación · ","")&amp;IF(E153="","referencia · ","")&amp;IF(H153="","criticidad · ","")&amp;IF(I153="","origen del agua · ","")&amp;IF(AND(LEFT(I153,7)="Sale de",J153="",K153=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C153:S153)=0,"",IF(AND(C153&lt;&gt;"",D153&lt;&gt;"",E153&lt;&gt;"",H153&lt;&gt;"",I153&lt;&gt;"",NOT(AND(LEFT(I153,7)="Sale de",J153="",K153=""))),"✔ Completa","Falta: "&amp;IF(C153="","fecha · ","")&amp;IF(D153="","ubicación · ","")&amp;IF(E153="","referencia · ","")&amp;IF(H153="","criticidad · ","")&amp;IF(I153="","origen del agua · ","")&amp;IF(AND(LEFT(I153,7)="Sale de",J153="",K153=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C153" s="17" t="n"/>
@@ -5330,8 +5503,9 @@
       <c r="N153" s="21" t="n"/>
       <c r="O153" s="21" t="n"/>
       <c r="P153" s="21" t="n"/>
-      <c r="Q153" s="18" t="n"/>
-      <c r="R153" s="19" t="n"/>
+      <c r="Q153" s="21" t="n"/>
+      <c r="R153" s="18" t="n"/>
+      <c r="S153" s="19" t="n"/>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="15" t="inlineStr">
@@ -5340,7 +5514,7 @@
         </is>
       </c>
       <c r="B154" s="16">
-        <f>IF(COUNTA(C154:R154)=0,"",IF(AND(C154&lt;&gt;"",D154&lt;&gt;"",E154&lt;&gt;"",H154&lt;&gt;"",I154&lt;&gt;"",NOT(AND(LEFT(I154,7)="Sale de",J154="",K154=""))),"✔ Completa","Falta: "&amp;IF(C154="","fecha · ","")&amp;IF(D154="","ubicación · ","")&amp;IF(E154="","referencia · ","")&amp;IF(H154="","criticidad · ","")&amp;IF(I154="","origen del agua · ","")&amp;IF(AND(LEFT(I154,7)="Sale de",J154="",K154=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C154:S154)=0,"",IF(AND(C154&lt;&gt;"",D154&lt;&gt;"",E154&lt;&gt;"",H154&lt;&gt;"",I154&lt;&gt;"",NOT(AND(LEFT(I154,7)="Sale de",J154="",K154=""))),"✔ Completa","Falta: "&amp;IF(C154="","fecha · ","")&amp;IF(D154="","ubicación · ","")&amp;IF(E154="","referencia · ","")&amp;IF(H154="","criticidad · ","")&amp;IF(I154="","origen del agua · ","")&amp;IF(AND(LEFT(I154,7)="Sale de",J154="",K154=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C154" s="17" t="n"/>
@@ -5357,8 +5531,9 @@
       <c r="N154" s="21" t="n"/>
       <c r="O154" s="21" t="n"/>
       <c r="P154" s="21" t="n"/>
-      <c r="Q154" s="18" t="n"/>
-      <c r="R154" s="19" t="n"/>
+      <c r="Q154" s="21" t="n"/>
+      <c r="R154" s="18" t="n"/>
+      <c r="S154" s="19" t="n"/>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="15" t="inlineStr">
@@ -5367,7 +5542,7 @@
         </is>
       </c>
       <c r="B155" s="16">
-        <f>IF(COUNTA(C155:R155)=0,"",IF(AND(C155&lt;&gt;"",D155&lt;&gt;"",E155&lt;&gt;"",H155&lt;&gt;"",I155&lt;&gt;"",NOT(AND(LEFT(I155,7)="Sale de",J155="",K155=""))),"✔ Completa","Falta: "&amp;IF(C155="","fecha · ","")&amp;IF(D155="","ubicación · ","")&amp;IF(E155="","referencia · ","")&amp;IF(H155="","criticidad · ","")&amp;IF(I155="","origen del agua · ","")&amp;IF(AND(LEFT(I155,7)="Sale de",J155="",K155=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C155:S155)=0,"",IF(AND(C155&lt;&gt;"",D155&lt;&gt;"",E155&lt;&gt;"",H155&lt;&gt;"",I155&lt;&gt;"",NOT(AND(LEFT(I155,7)="Sale de",J155="",K155=""))),"✔ Completa","Falta: "&amp;IF(C155="","fecha · ","")&amp;IF(D155="","ubicación · ","")&amp;IF(E155="","referencia · ","")&amp;IF(H155="","criticidad · ","")&amp;IF(I155="","origen del agua · ","")&amp;IF(AND(LEFT(I155,7)="Sale de",J155="",K155=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C155" s="17" t="n"/>
@@ -5384,8 +5559,9 @@
       <c r="N155" s="21" t="n"/>
       <c r="O155" s="21" t="n"/>
       <c r="P155" s="21" t="n"/>
-      <c r="Q155" s="18" t="n"/>
-      <c r="R155" s="19" t="n"/>
+      <c r="Q155" s="21" t="n"/>
+      <c r="R155" s="18" t="n"/>
+      <c r="S155" s="19" t="n"/>
     </row>
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="15" t="inlineStr">
@@ -5394,7 +5570,7 @@
         </is>
       </c>
       <c r="B156" s="16">
-        <f>IF(COUNTA(C156:R156)=0,"",IF(AND(C156&lt;&gt;"",D156&lt;&gt;"",E156&lt;&gt;"",H156&lt;&gt;"",I156&lt;&gt;"",NOT(AND(LEFT(I156,7)="Sale de",J156="",K156=""))),"✔ Completa","Falta: "&amp;IF(C156="","fecha · ","")&amp;IF(D156="","ubicación · ","")&amp;IF(E156="","referencia · ","")&amp;IF(H156="","criticidad · ","")&amp;IF(I156="","origen del agua · ","")&amp;IF(AND(LEFT(I156,7)="Sale de",J156="",K156=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C156:S156)=0,"",IF(AND(C156&lt;&gt;"",D156&lt;&gt;"",E156&lt;&gt;"",H156&lt;&gt;"",I156&lt;&gt;"",NOT(AND(LEFT(I156,7)="Sale de",J156="",K156=""))),"✔ Completa","Falta: "&amp;IF(C156="","fecha · ","")&amp;IF(D156="","ubicación · ","")&amp;IF(E156="","referencia · ","")&amp;IF(H156="","criticidad · ","")&amp;IF(I156="","origen del agua · ","")&amp;IF(AND(LEFT(I156,7)="Sale de",J156="",K156=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C156" s="17" t="n"/>
@@ -5411,8 +5587,9 @@
       <c r="N156" s="21" t="n"/>
       <c r="O156" s="21" t="n"/>
       <c r="P156" s="21" t="n"/>
-      <c r="Q156" s="18" t="n"/>
-      <c r="R156" s="19" t="n"/>
+      <c r="Q156" s="21" t="n"/>
+      <c r="R156" s="18" t="n"/>
+      <c r="S156" s="19" t="n"/>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="15" t="inlineStr">
@@ -5421,7 +5598,7 @@
         </is>
       </c>
       <c r="B157" s="16">
-        <f>IF(COUNTA(C157:R157)=0,"",IF(AND(C157&lt;&gt;"",D157&lt;&gt;"",E157&lt;&gt;"",H157&lt;&gt;"",I157&lt;&gt;"",NOT(AND(LEFT(I157,7)="Sale de",J157="",K157=""))),"✔ Completa","Falta: "&amp;IF(C157="","fecha · ","")&amp;IF(D157="","ubicación · ","")&amp;IF(E157="","referencia · ","")&amp;IF(H157="","criticidad · ","")&amp;IF(I157="","origen del agua · ","")&amp;IF(AND(LEFT(I157,7)="Sale de",J157="",K157=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C157:S157)=0,"",IF(AND(C157&lt;&gt;"",D157&lt;&gt;"",E157&lt;&gt;"",H157&lt;&gt;"",I157&lt;&gt;"",NOT(AND(LEFT(I157,7)="Sale de",J157="",K157=""))),"✔ Completa","Falta: "&amp;IF(C157="","fecha · ","")&amp;IF(D157="","ubicación · ","")&amp;IF(E157="","referencia · ","")&amp;IF(H157="","criticidad · ","")&amp;IF(I157="","origen del agua · ","")&amp;IF(AND(LEFT(I157,7)="Sale de",J157="",K157=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C157" s="17" t="n"/>
@@ -5438,8 +5615,9 @@
       <c r="N157" s="21" t="n"/>
       <c r="O157" s="21" t="n"/>
       <c r="P157" s="21" t="n"/>
-      <c r="Q157" s="18" t="n"/>
-      <c r="R157" s="19" t="n"/>
+      <c r="Q157" s="21" t="n"/>
+      <c r="R157" s="18" t="n"/>
+      <c r="S157" s="19" t="n"/>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="15" t="inlineStr">
@@ -5448,7 +5626,7 @@
         </is>
       </c>
       <c r="B158" s="16">
-        <f>IF(COUNTA(C158:R158)=0,"",IF(AND(C158&lt;&gt;"",D158&lt;&gt;"",E158&lt;&gt;"",H158&lt;&gt;"",I158&lt;&gt;"",NOT(AND(LEFT(I158,7)="Sale de",J158="",K158=""))),"✔ Completa","Falta: "&amp;IF(C158="","fecha · ","")&amp;IF(D158="","ubicación · ","")&amp;IF(E158="","referencia · ","")&amp;IF(H158="","criticidad · ","")&amp;IF(I158="","origen del agua · ","")&amp;IF(AND(LEFT(I158,7)="Sale de",J158="",K158=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C158:S158)=0,"",IF(AND(C158&lt;&gt;"",D158&lt;&gt;"",E158&lt;&gt;"",H158&lt;&gt;"",I158&lt;&gt;"",NOT(AND(LEFT(I158,7)="Sale de",J158="",K158=""))),"✔ Completa","Falta: "&amp;IF(C158="","fecha · ","")&amp;IF(D158="","ubicación · ","")&amp;IF(E158="","referencia · ","")&amp;IF(H158="","criticidad · ","")&amp;IF(I158="","origen del agua · ","")&amp;IF(AND(LEFT(I158,7)="Sale de",J158="",K158=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C158" s="17" t="n"/>
@@ -5465,8 +5643,9 @@
       <c r="N158" s="21" t="n"/>
       <c r="O158" s="21" t="n"/>
       <c r="P158" s="21" t="n"/>
-      <c r="Q158" s="18" t="n"/>
-      <c r="R158" s="19" t="n"/>
+      <c r="Q158" s="21" t="n"/>
+      <c r="R158" s="18" t="n"/>
+      <c r="S158" s="19" t="n"/>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="15" t="inlineStr">
@@ -5475,7 +5654,7 @@
         </is>
       </c>
       <c r="B159" s="16">
-        <f>IF(COUNTA(C159:R159)=0,"",IF(AND(C159&lt;&gt;"",D159&lt;&gt;"",E159&lt;&gt;"",H159&lt;&gt;"",I159&lt;&gt;"",NOT(AND(LEFT(I159,7)="Sale de",J159="",K159=""))),"✔ Completa","Falta: "&amp;IF(C159="","fecha · ","")&amp;IF(D159="","ubicación · ","")&amp;IF(E159="","referencia · ","")&amp;IF(H159="","criticidad · ","")&amp;IF(I159="","origen del agua · ","")&amp;IF(AND(LEFT(I159,7)="Sale de",J159="",K159=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C159:S159)=0,"",IF(AND(C159&lt;&gt;"",D159&lt;&gt;"",E159&lt;&gt;"",H159&lt;&gt;"",I159&lt;&gt;"",NOT(AND(LEFT(I159,7)="Sale de",J159="",K159=""))),"✔ Completa","Falta: "&amp;IF(C159="","fecha · ","")&amp;IF(D159="","ubicación · ","")&amp;IF(E159="","referencia · ","")&amp;IF(H159="","criticidad · ","")&amp;IF(I159="","origen del agua · ","")&amp;IF(AND(LEFT(I159,7)="Sale de",J159="",K159=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C159" s="17" t="n"/>
@@ -5492,8 +5671,9 @@
       <c r="N159" s="21" t="n"/>
       <c r="O159" s="21" t="n"/>
       <c r="P159" s="21" t="n"/>
-      <c r="Q159" s="18" t="n"/>
-      <c r="R159" s="19" t="n"/>
+      <c r="Q159" s="21" t="n"/>
+      <c r="R159" s="18" t="n"/>
+      <c r="S159" s="19" t="n"/>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="15" t="inlineStr">
@@ -5502,7 +5682,7 @@
         </is>
       </c>
       <c r="B160" s="16">
-        <f>IF(COUNTA(C160:R160)=0,"",IF(AND(C160&lt;&gt;"",D160&lt;&gt;"",E160&lt;&gt;"",H160&lt;&gt;"",I160&lt;&gt;"",NOT(AND(LEFT(I160,7)="Sale de",J160="",K160=""))),"✔ Completa","Falta: "&amp;IF(C160="","fecha · ","")&amp;IF(D160="","ubicación · ","")&amp;IF(E160="","referencia · ","")&amp;IF(H160="","criticidad · ","")&amp;IF(I160="","origen del agua · ","")&amp;IF(AND(LEFT(I160,7)="Sale de",J160="",K160=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C160:S160)=0,"",IF(AND(C160&lt;&gt;"",D160&lt;&gt;"",E160&lt;&gt;"",H160&lt;&gt;"",I160&lt;&gt;"",NOT(AND(LEFT(I160,7)="Sale de",J160="",K160=""))),"✔ Completa","Falta: "&amp;IF(C160="","fecha · ","")&amp;IF(D160="","ubicación · ","")&amp;IF(E160="","referencia · ","")&amp;IF(H160="","criticidad · ","")&amp;IF(I160="","origen del agua · ","")&amp;IF(AND(LEFT(I160,7)="Sale de",J160="",K160=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C160" s="17" t="n"/>
@@ -5519,8 +5699,9 @@
       <c r="N160" s="21" t="n"/>
       <c r="O160" s="21" t="n"/>
       <c r="P160" s="21" t="n"/>
-      <c r="Q160" s="18" t="n"/>
-      <c r="R160" s="19" t="n"/>
+      <c r="Q160" s="21" t="n"/>
+      <c r="R160" s="18" t="n"/>
+      <c r="S160" s="19" t="n"/>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="15" t="inlineStr">
@@ -5529,7 +5710,7 @@
         </is>
       </c>
       <c r="B161" s="16">
-        <f>IF(COUNTA(C161:R161)=0,"",IF(AND(C161&lt;&gt;"",D161&lt;&gt;"",E161&lt;&gt;"",H161&lt;&gt;"",I161&lt;&gt;"",NOT(AND(LEFT(I161,7)="Sale de",J161="",K161=""))),"✔ Completa","Falta: "&amp;IF(C161="","fecha · ","")&amp;IF(D161="","ubicación · ","")&amp;IF(E161="","referencia · ","")&amp;IF(H161="","criticidad · ","")&amp;IF(I161="","origen del agua · ","")&amp;IF(AND(LEFT(I161,7)="Sale de",J161="",K161=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C161:S161)=0,"",IF(AND(C161&lt;&gt;"",D161&lt;&gt;"",E161&lt;&gt;"",H161&lt;&gt;"",I161&lt;&gt;"",NOT(AND(LEFT(I161,7)="Sale de",J161="",K161=""))),"✔ Completa","Falta: "&amp;IF(C161="","fecha · ","")&amp;IF(D161="","ubicación · ","")&amp;IF(E161="","referencia · ","")&amp;IF(H161="","criticidad · ","")&amp;IF(I161="","origen del agua · ","")&amp;IF(AND(LEFT(I161,7)="Sale de",J161="",K161=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C161" s="17" t="n"/>
@@ -5546,8 +5727,9 @@
       <c r="N161" s="21" t="n"/>
       <c r="O161" s="21" t="n"/>
       <c r="P161" s="21" t="n"/>
-      <c r="Q161" s="18" t="n"/>
-      <c r="R161" s="19" t="n"/>
+      <c r="Q161" s="21" t="n"/>
+      <c r="R161" s="18" t="n"/>
+      <c r="S161" s="19" t="n"/>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="15" t="inlineStr">
@@ -5556,7 +5738,7 @@
         </is>
       </c>
       <c r="B162" s="16">
-        <f>IF(COUNTA(C162:R162)=0,"",IF(AND(C162&lt;&gt;"",D162&lt;&gt;"",E162&lt;&gt;"",H162&lt;&gt;"",I162&lt;&gt;"",NOT(AND(LEFT(I162,7)="Sale de",J162="",K162=""))),"✔ Completa","Falta: "&amp;IF(C162="","fecha · ","")&amp;IF(D162="","ubicación · ","")&amp;IF(E162="","referencia · ","")&amp;IF(H162="","criticidad · ","")&amp;IF(I162="","origen del agua · ","")&amp;IF(AND(LEFT(I162,7)="Sale de",J162="",K162=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C162:S162)=0,"",IF(AND(C162&lt;&gt;"",D162&lt;&gt;"",E162&lt;&gt;"",H162&lt;&gt;"",I162&lt;&gt;"",NOT(AND(LEFT(I162,7)="Sale de",J162="",K162=""))),"✔ Completa","Falta: "&amp;IF(C162="","fecha · ","")&amp;IF(D162="","ubicación · ","")&amp;IF(E162="","referencia · ","")&amp;IF(H162="","criticidad · ","")&amp;IF(I162="","origen del agua · ","")&amp;IF(AND(LEFT(I162,7)="Sale de",J162="",K162=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C162" s="17" t="n"/>
@@ -5573,8 +5755,9 @@
       <c r="N162" s="21" t="n"/>
       <c r="O162" s="21" t="n"/>
       <c r="P162" s="21" t="n"/>
-      <c r="Q162" s="18" t="n"/>
-      <c r="R162" s="19" t="n"/>
+      <c r="Q162" s="21" t="n"/>
+      <c r="R162" s="18" t="n"/>
+      <c r="S162" s="19" t="n"/>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="15" t="inlineStr">
@@ -5583,7 +5766,7 @@
         </is>
       </c>
       <c r="B163" s="16">
-        <f>IF(COUNTA(C163:R163)=0,"",IF(AND(C163&lt;&gt;"",D163&lt;&gt;"",E163&lt;&gt;"",H163&lt;&gt;"",I163&lt;&gt;"",NOT(AND(LEFT(I163,7)="Sale de",J163="",K163=""))),"✔ Completa","Falta: "&amp;IF(C163="","fecha · ","")&amp;IF(D163="","ubicación · ","")&amp;IF(E163="","referencia · ","")&amp;IF(H163="","criticidad · ","")&amp;IF(I163="","origen del agua · ","")&amp;IF(AND(LEFT(I163,7)="Sale de",J163="",K163=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C163:S163)=0,"",IF(AND(C163&lt;&gt;"",D163&lt;&gt;"",E163&lt;&gt;"",H163&lt;&gt;"",I163&lt;&gt;"",NOT(AND(LEFT(I163,7)="Sale de",J163="",K163=""))),"✔ Completa","Falta: "&amp;IF(C163="","fecha · ","")&amp;IF(D163="","ubicación · ","")&amp;IF(E163="","referencia · ","")&amp;IF(H163="","criticidad · ","")&amp;IF(I163="","origen del agua · ","")&amp;IF(AND(LEFT(I163,7)="Sale de",J163="",K163=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C163" s="17" t="n"/>
@@ -5600,8 +5783,9 @@
       <c r="N163" s="21" t="n"/>
       <c r="O163" s="21" t="n"/>
       <c r="P163" s="21" t="n"/>
-      <c r="Q163" s="18" t="n"/>
-      <c r="R163" s="19" t="n"/>
+      <c r="Q163" s="21" t="n"/>
+      <c r="R163" s="18" t="n"/>
+      <c r="S163" s="19" t="n"/>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="15" t="inlineStr">
@@ -5610,7 +5794,7 @@
         </is>
       </c>
       <c r="B164" s="16">
-        <f>IF(COUNTA(C164:R164)=0,"",IF(AND(C164&lt;&gt;"",D164&lt;&gt;"",E164&lt;&gt;"",H164&lt;&gt;"",I164&lt;&gt;"",NOT(AND(LEFT(I164,7)="Sale de",J164="",K164=""))),"✔ Completa","Falta: "&amp;IF(C164="","fecha · ","")&amp;IF(D164="","ubicación · ","")&amp;IF(E164="","referencia · ","")&amp;IF(H164="","criticidad · ","")&amp;IF(I164="","origen del agua · ","")&amp;IF(AND(LEFT(I164,7)="Sale de",J164="",K164=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C164:S164)=0,"",IF(AND(C164&lt;&gt;"",D164&lt;&gt;"",E164&lt;&gt;"",H164&lt;&gt;"",I164&lt;&gt;"",NOT(AND(LEFT(I164,7)="Sale de",J164="",K164=""))),"✔ Completa","Falta: "&amp;IF(C164="","fecha · ","")&amp;IF(D164="","ubicación · ","")&amp;IF(E164="","referencia · ","")&amp;IF(H164="","criticidad · ","")&amp;IF(I164="","origen del agua · ","")&amp;IF(AND(LEFT(I164,7)="Sale de",J164="",K164=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C164" s="17" t="n"/>
@@ -5627,8 +5811,9 @@
       <c r="N164" s="21" t="n"/>
       <c r="O164" s="21" t="n"/>
       <c r="P164" s="21" t="n"/>
-      <c r="Q164" s="18" t="n"/>
-      <c r="R164" s="19" t="n"/>
+      <c r="Q164" s="21" t="n"/>
+      <c r="R164" s="18" t="n"/>
+      <c r="S164" s="19" t="n"/>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="15" t="inlineStr">
@@ -5637,7 +5822,7 @@
         </is>
       </c>
       <c r="B165" s="16">
-        <f>IF(COUNTA(C165:R165)=0,"",IF(AND(C165&lt;&gt;"",D165&lt;&gt;"",E165&lt;&gt;"",H165&lt;&gt;"",I165&lt;&gt;"",NOT(AND(LEFT(I165,7)="Sale de",J165="",K165=""))),"✔ Completa","Falta: "&amp;IF(C165="","fecha · ","")&amp;IF(D165="","ubicación · ","")&amp;IF(E165="","referencia · ","")&amp;IF(H165="","criticidad · ","")&amp;IF(I165="","origen del agua · ","")&amp;IF(AND(LEFT(I165,7)="Sale de",J165="",K165=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C165:S165)=0,"",IF(AND(C165&lt;&gt;"",D165&lt;&gt;"",E165&lt;&gt;"",H165&lt;&gt;"",I165&lt;&gt;"",NOT(AND(LEFT(I165,7)="Sale de",J165="",K165=""))),"✔ Completa","Falta: "&amp;IF(C165="","fecha · ","")&amp;IF(D165="","ubicación · ","")&amp;IF(E165="","referencia · ","")&amp;IF(H165="","criticidad · ","")&amp;IF(I165="","origen del agua · ","")&amp;IF(AND(LEFT(I165,7)="Sale de",J165="",K165=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C165" s="17" t="n"/>
@@ -5654,8 +5839,9 @@
       <c r="N165" s="21" t="n"/>
       <c r="O165" s="21" t="n"/>
       <c r="P165" s="21" t="n"/>
-      <c r="Q165" s="18" t="n"/>
-      <c r="R165" s="19" t="n"/>
+      <c r="Q165" s="21" t="n"/>
+      <c r="R165" s="18" t="n"/>
+      <c r="S165" s="19" t="n"/>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="15" t="inlineStr">
@@ -5664,7 +5850,7 @@
         </is>
       </c>
       <c r="B166" s="16">
-        <f>IF(COUNTA(C166:R166)=0,"",IF(AND(C166&lt;&gt;"",D166&lt;&gt;"",E166&lt;&gt;"",H166&lt;&gt;"",I166&lt;&gt;"",NOT(AND(LEFT(I166,7)="Sale de",J166="",K166=""))),"✔ Completa","Falta: "&amp;IF(C166="","fecha · ","")&amp;IF(D166="","ubicación · ","")&amp;IF(E166="","referencia · ","")&amp;IF(H166="","criticidad · ","")&amp;IF(I166="","origen del agua · ","")&amp;IF(AND(LEFT(I166,7)="Sale de",J166="",K166=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C166:S166)=0,"",IF(AND(C166&lt;&gt;"",D166&lt;&gt;"",E166&lt;&gt;"",H166&lt;&gt;"",I166&lt;&gt;"",NOT(AND(LEFT(I166,7)="Sale de",J166="",K166=""))),"✔ Completa","Falta: "&amp;IF(C166="","fecha · ","")&amp;IF(D166="","ubicación · ","")&amp;IF(E166="","referencia · ","")&amp;IF(H166="","criticidad · ","")&amp;IF(I166="","origen del agua · ","")&amp;IF(AND(LEFT(I166,7)="Sale de",J166="",K166=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C166" s="17" t="n"/>
@@ -5681,8 +5867,9 @@
       <c r="N166" s="21" t="n"/>
       <c r="O166" s="21" t="n"/>
       <c r="P166" s="21" t="n"/>
-      <c r="Q166" s="18" t="n"/>
-      <c r="R166" s="19" t="n"/>
+      <c r="Q166" s="21" t="n"/>
+      <c r="R166" s="18" t="n"/>
+      <c r="S166" s="19" t="n"/>
     </row>
     <row r="167" ht="20" customHeight="1">
       <c r="A167" s="15" t="inlineStr">
@@ -5691,7 +5878,7 @@
         </is>
       </c>
       <c r="B167" s="16">
-        <f>IF(COUNTA(C167:R167)=0,"",IF(AND(C167&lt;&gt;"",D167&lt;&gt;"",E167&lt;&gt;"",H167&lt;&gt;"",I167&lt;&gt;"",NOT(AND(LEFT(I167,7)="Sale de",J167="",K167=""))),"✔ Completa","Falta: "&amp;IF(C167="","fecha · ","")&amp;IF(D167="","ubicación · ","")&amp;IF(E167="","referencia · ","")&amp;IF(H167="","criticidad · ","")&amp;IF(I167="","origen del agua · ","")&amp;IF(AND(LEFT(I167,7)="Sale de",J167="",K167=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C167:S167)=0,"",IF(AND(C167&lt;&gt;"",D167&lt;&gt;"",E167&lt;&gt;"",H167&lt;&gt;"",I167&lt;&gt;"",NOT(AND(LEFT(I167,7)="Sale de",J167="",K167=""))),"✔ Completa","Falta: "&amp;IF(C167="","fecha · ","")&amp;IF(D167="","ubicación · ","")&amp;IF(E167="","referencia · ","")&amp;IF(H167="","criticidad · ","")&amp;IF(I167="","origen del agua · ","")&amp;IF(AND(LEFT(I167,7)="Sale de",J167="",K167=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C167" s="17" t="n"/>
@@ -5708,8 +5895,9 @@
       <c r="N167" s="21" t="n"/>
       <c r="O167" s="21" t="n"/>
       <c r="P167" s="21" t="n"/>
-      <c r="Q167" s="18" t="n"/>
-      <c r="R167" s="19" t="n"/>
+      <c r="Q167" s="21" t="n"/>
+      <c r="R167" s="18" t="n"/>
+      <c r="S167" s="19" t="n"/>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="15" t="inlineStr">
@@ -5718,7 +5906,7 @@
         </is>
       </c>
       <c r="B168" s="16">
-        <f>IF(COUNTA(C168:R168)=0,"",IF(AND(C168&lt;&gt;"",D168&lt;&gt;"",E168&lt;&gt;"",H168&lt;&gt;"",I168&lt;&gt;"",NOT(AND(LEFT(I168,7)="Sale de",J168="",K168=""))),"✔ Completa","Falta: "&amp;IF(C168="","fecha · ","")&amp;IF(D168="","ubicación · ","")&amp;IF(E168="","referencia · ","")&amp;IF(H168="","criticidad · ","")&amp;IF(I168="","origen del agua · ","")&amp;IF(AND(LEFT(I168,7)="Sale de",J168="",K168=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C168:S168)=0,"",IF(AND(C168&lt;&gt;"",D168&lt;&gt;"",E168&lt;&gt;"",H168&lt;&gt;"",I168&lt;&gt;"",NOT(AND(LEFT(I168,7)="Sale de",J168="",K168=""))),"✔ Completa","Falta: "&amp;IF(C168="","fecha · ","")&amp;IF(D168="","ubicación · ","")&amp;IF(E168="","referencia · ","")&amp;IF(H168="","criticidad · ","")&amp;IF(I168="","origen del agua · ","")&amp;IF(AND(LEFT(I168,7)="Sale de",J168="",K168=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C168" s="17" t="n"/>
@@ -5735,8 +5923,9 @@
       <c r="N168" s="21" t="n"/>
       <c r="O168" s="21" t="n"/>
       <c r="P168" s="21" t="n"/>
-      <c r="Q168" s="18" t="n"/>
-      <c r="R168" s="19" t="n"/>
+      <c r="Q168" s="21" t="n"/>
+      <c r="R168" s="18" t="n"/>
+      <c r="S168" s="19" t="n"/>
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="15" t="inlineStr">
@@ -5745,7 +5934,7 @@
         </is>
       </c>
       <c r="B169" s="16">
-        <f>IF(COUNTA(C169:R169)=0,"",IF(AND(C169&lt;&gt;"",D169&lt;&gt;"",E169&lt;&gt;"",H169&lt;&gt;"",I169&lt;&gt;"",NOT(AND(LEFT(I169,7)="Sale de",J169="",K169=""))),"✔ Completa","Falta: "&amp;IF(C169="","fecha · ","")&amp;IF(D169="","ubicación · ","")&amp;IF(E169="","referencia · ","")&amp;IF(H169="","criticidad · ","")&amp;IF(I169="","origen del agua · ","")&amp;IF(AND(LEFT(I169,7)="Sale de",J169="",K169=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C169:S169)=0,"",IF(AND(C169&lt;&gt;"",D169&lt;&gt;"",E169&lt;&gt;"",H169&lt;&gt;"",I169&lt;&gt;"",NOT(AND(LEFT(I169,7)="Sale de",J169="",K169=""))),"✔ Completa","Falta: "&amp;IF(C169="","fecha · ","")&amp;IF(D169="","ubicación · ","")&amp;IF(E169="","referencia · ","")&amp;IF(H169="","criticidad · ","")&amp;IF(I169="","origen del agua · ","")&amp;IF(AND(LEFT(I169,7)="Sale de",J169="",K169=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C169" s="17" t="n"/>
@@ -5762,8 +5951,9 @@
       <c r="N169" s="21" t="n"/>
       <c r="O169" s="21" t="n"/>
       <c r="P169" s="21" t="n"/>
-      <c r="Q169" s="18" t="n"/>
-      <c r="R169" s="19" t="n"/>
+      <c r="Q169" s="21" t="n"/>
+      <c r="R169" s="18" t="n"/>
+      <c r="S169" s="19" t="n"/>
     </row>
     <row r="170" ht="20" customHeight="1">
       <c r="A170" s="15" t="inlineStr">
@@ -5772,7 +5962,7 @@
         </is>
       </c>
       <c r="B170" s="16">
-        <f>IF(COUNTA(C170:R170)=0,"",IF(AND(C170&lt;&gt;"",D170&lt;&gt;"",E170&lt;&gt;"",H170&lt;&gt;"",I170&lt;&gt;"",NOT(AND(LEFT(I170,7)="Sale de",J170="",K170=""))),"✔ Completa","Falta: "&amp;IF(C170="","fecha · ","")&amp;IF(D170="","ubicación · ","")&amp;IF(E170="","referencia · ","")&amp;IF(H170="","criticidad · ","")&amp;IF(I170="","origen del agua · ","")&amp;IF(AND(LEFT(I170,7)="Sale de",J170="",K170=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C170:S170)=0,"",IF(AND(C170&lt;&gt;"",D170&lt;&gt;"",E170&lt;&gt;"",H170&lt;&gt;"",I170&lt;&gt;"",NOT(AND(LEFT(I170,7)="Sale de",J170="",K170=""))),"✔ Completa","Falta: "&amp;IF(C170="","fecha · ","")&amp;IF(D170="","ubicación · ","")&amp;IF(E170="","referencia · ","")&amp;IF(H170="","criticidad · ","")&amp;IF(I170="","origen del agua · ","")&amp;IF(AND(LEFT(I170,7)="Sale de",J170="",K170=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C170" s="17" t="n"/>
@@ -5789,8 +5979,9 @@
       <c r="N170" s="21" t="n"/>
       <c r="O170" s="21" t="n"/>
       <c r="P170" s="21" t="n"/>
-      <c r="Q170" s="18" t="n"/>
-      <c r="R170" s="19" t="n"/>
+      <c r="Q170" s="21" t="n"/>
+      <c r="R170" s="18" t="n"/>
+      <c r="S170" s="19" t="n"/>
     </row>
     <row r="171" ht="20" customHeight="1">
       <c r="A171" s="15" t="inlineStr">
@@ -5799,7 +5990,7 @@
         </is>
       </c>
       <c r="B171" s="16">
-        <f>IF(COUNTA(C171:R171)=0,"",IF(AND(C171&lt;&gt;"",D171&lt;&gt;"",E171&lt;&gt;"",H171&lt;&gt;"",I171&lt;&gt;"",NOT(AND(LEFT(I171,7)="Sale de",J171="",K171=""))),"✔ Completa","Falta: "&amp;IF(C171="","fecha · ","")&amp;IF(D171="","ubicación · ","")&amp;IF(E171="","referencia · ","")&amp;IF(H171="","criticidad · ","")&amp;IF(I171="","origen del agua · ","")&amp;IF(AND(LEFT(I171,7)="Sale de",J171="",K171=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C171:S171)=0,"",IF(AND(C171&lt;&gt;"",D171&lt;&gt;"",E171&lt;&gt;"",H171&lt;&gt;"",I171&lt;&gt;"",NOT(AND(LEFT(I171,7)="Sale de",J171="",K171=""))),"✔ Completa","Falta: "&amp;IF(C171="","fecha · ","")&amp;IF(D171="","ubicación · ","")&amp;IF(E171="","referencia · ","")&amp;IF(H171="","criticidad · ","")&amp;IF(I171="","origen del agua · ","")&amp;IF(AND(LEFT(I171,7)="Sale de",J171="",K171=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C171" s="17" t="n"/>
@@ -5816,8 +6007,9 @@
       <c r="N171" s="21" t="n"/>
       <c r="O171" s="21" t="n"/>
       <c r="P171" s="21" t="n"/>
-      <c r="Q171" s="18" t="n"/>
-      <c r="R171" s="19" t="n"/>
+      <c r="Q171" s="21" t="n"/>
+      <c r="R171" s="18" t="n"/>
+      <c r="S171" s="19" t="n"/>
     </row>
     <row r="172" ht="20" customHeight="1">
       <c r="A172" s="15" t="inlineStr">
@@ -5826,7 +6018,7 @@
         </is>
       </c>
       <c r="B172" s="16">
-        <f>IF(COUNTA(C172:R172)=0,"",IF(AND(C172&lt;&gt;"",D172&lt;&gt;"",E172&lt;&gt;"",H172&lt;&gt;"",I172&lt;&gt;"",NOT(AND(LEFT(I172,7)="Sale de",J172="",K172=""))),"✔ Completa","Falta: "&amp;IF(C172="","fecha · ","")&amp;IF(D172="","ubicación · ","")&amp;IF(E172="","referencia · ","")&amp;IF(H172="","criticidad · ","")&amp;IF(I172="","origen del agua · ","")&amp;IF(AND(LEFT(I172,7)="Sale de",J172="",K172=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C172:S172)=0,"",IF(AND(C172&lt;&gt;"",D172&lt;&gt;"",E172&lt;&gt;"",H172&lt;&gt;"",I172&lt;&gt;"",NOT(AND(LEFT(I172,7)="Sale de",J172="",K172=""))),"✔ Completa","Falta: "&amp;IF(C172="","fecha · ","")&amp;IF(D172="","ubicación · ","")&amp;IF(E172="","referencia · ","")&amp;IF(H172="","criticidad · ","")&amp;IF(I172="","origen del agua · ","")&amp;IF(AND(LEFT(I172,7)="Sale de",J172="",K172=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C172" s="17" t="n"/>
@@ -5843,8 +6035,9 @@
       <c r="N172" s="21" t="n"/>
       <c r="O172" s="21" t="n"/>
       <c r="P172" s="21" t="n"/>
-      <c r="Q172" s="18" t="n"/>
-      <c r="R172" s="19" t="n"/>
+      <c r="Q172" s="21" t="n"/>
+      <c r="R172" s="18" t="n"/>
+      <c r="S172" s="19" t="n"/>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="15" t="inlineStr">
@@ -5853,7 +6046,7 @@
         </is>
       </c>
       <c r="B173" s="16">
-        <f>IF(COUNTA(C173:R173)=0,"",IF(AND(C173&lt;&gt;"",D173&lt;&gt;"",E173&lt;&gt;"",H173&lt;&gt;"",I173&lt;&gt;"",NOT(AND(LEFT(I173,7)="Sale de",J173="",K173=""))),"✔ Completa","Falta: "&amp;IF(C173="","fecha · ","")&amp;IF(D173="","ubicación · ","")&amp;IF(E173="","referencia · ","")&amp;IF(H173="","criticidad · ","")&amp;IF(I173="","origen del agua · ","")&amp;IF(AND(LEFT(I173,7)="Sale de",J173="",K173=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C173:S173)=0,"",IF(AND(C173&lt;&gt;"",D173&lt;&gt;"",E173&lt;&gt;"",H173&lt;&gt;"",I173&lt;&gt;"",NOT(AND(LEFT(I173,7)="Sale de",J173="",K173=""))),"✔ Completa","Falta: "&amp;IF(C173="","fecha · ","")&amp;IF(D173="","ubicación · ","")&amp;IF(E173="","referencia · ","")&amp;IF(H173="","criticidad · ","")&amp;IF(I173="","origen del agua · ","")&amp;IF(AND(LEFT(I173,7)="Sale de",J173="",K173=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C173" s="17" t="n"/>
@@ -5870,8 +6063,9 @@
       <c r="N173" s="21" t="n"/>
       <c r="O173" s="21" t="n"/>
       <c r="P173" s="21" t="n"/>
-      <c r="Q173" s="18" t="n"/>
-      <c r="R173" s="19" t="n"/>
+      <c r="Q173" s="21" t="n"/>
+      <c r="R173" s="18" t="n"/>
+      <c r="S173" s="19" t="n"/>
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="15" t="inlineStr">
@@ -5880,7 +6074,7 @@
         </is>
       </c>
       <c r="B174" s="16">
-        <f>IF(COUNTA(C174:R174)=0,"",IF(AND(C174&lt;&gt;"",D174&lt;&gt;"",E174&lt;&gt;"",H174&lt;&gt;"",I174&lt;&gt;"",NOT(AND(LEFT(I174,7)="Sale de",J174="",K174=""))),"✔ Completa","Falta: "&amp;IF(C174="","fecha · ","")&amp;IF(D174="","ubicación · ","")&amp;IF(E174="","referencia · ","")&amp;IF(H174="","criticidad · ","")&amp;IF(I174="","origen del agua · ","")&amp;IF(AND(LEFT(I174,7)="Sale de",J174="",K174=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C174:S174)=0,"",IF(AND(C174&lt;&gt;"",D174&lt;&gt;"",E174&lt;&gt;"",H174&lt;&gt;"",I174&lt;&gt;"",NOT(AND(LEFT(I174,7)="Sale de",J174="",K174=""))),"✔ Completa","Falta: "&amp;IF(C174="","fecha · ","")&amp;IF(D174="","ubicación · ","")&amp;IF(E174="","referencia · ","")&amp;IF(H174="","criticidad · ","")&amp;IF(I174="","origen del agua · ","")&amp;IF(AND(LEFT(I174,7)="Sale de",J174="",K174=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C174" s="17" t="n"/>
@@ -5897,8 +6091,9 @@
       <c r="N174" s="21" t="n"/>
       <c r="O174" s="21" t="n"/>
       <c r="P174" s="21" t="n"/>
-      <c r="Q174" s="18" t="n"/>
-      <c r="R174" s="19" t="n"/>
+      <c r="Q174" s="21" t="n"/>
+      <c r="R174" s="18" t="n"/>
+      <c r="S174" s="19" t="n"/>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="15" t="inlineStr">
@@ -5907,7 +6102,7 @@
         </is>
       </c>
       <c r="B175" s="16">
-        <f>IF(COUNTA(C175:R175)=0,"",IF(AND(C175&lt;&gt;"",D175&lt;&gt;"",E175&lt;&gt;"",H175&lt;&gt;"",I175&lt;&gt;"",NOT(AND(LEFT(I175,7)="Sale de",J175="",K175=""))),"✔ Completa","Falta: "&amp;IF(C175="","fecha · ","")&amp;IF(D175="","ubicación · ","")&amp;IF(E175="","referencia · ","")&amp;IF(H175="","criticidad · ","")&amp;IF(I175="","origen del agua · ","")&amp;IF(AND(LEFT(I175,7)="Sale de",J175="",K175=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C175:S175)=0,"",IF(AND(C175&lt;&gt;"",D175&lt;&gt;"",E175&lt;&gt;"",H175&lt;&gt;"",I175&lt;&gt;"",NOT(AND(LEFT(I175,7)="Sale de",J175="",K175=""))),"✔ Completa","Falta: "&amp;IF(C175="","fecha · ","")&amp;IF(D175="","ubicación · ","")&amp;IF(E175="","referencia · ","")&amp;IF(H175="","criticidad · ","")&amp;IF(I175="","origen del agua · ","")&amp;IF(AND(LEFT(I175,7)="Sale de",J175="",K175=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C175" s="17" t="n"/>
@@ -5924,8 +6119,9 @@
       <c r="N175" s="21" t="n"/>
       <c r="O175" s="21" t="n"/>
       <c r="P175" s="21" t="n"/>
-      <c r="Q175" s="18" t="n"/>
-      <c r="R175" s="19" t="n"/>
+      <c r="Q175" s="21" t="n"/>
+      <c r="R175" s="18" t="n"/>
+      <c r="S175" s="19" t="n"/>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="15" t="inlineStr">
@@ -5934,7 +6130,7 @@
         </is>
       </c>
       <c r="B176" s="16">
-        <f>IF(COUNTA(C176:R176)=0,"",IF(AND(C176&lt;&gt;"",D176&lt;&gt;"",E176&lt;&gt;"",H176&lt;&gt;"",I176&lt;&gt;"",NOT(AND(LEFT(I176,7)="Sale de",J176="",K176=""))),"✔ Completa","Falta: "&amp;IF(C176="","fecha · ","")&amp;IF(D176="","ubicación · ","")&amp;IF(E176="","referencia · ","")&amp;IF(H176="","criticidad · ","")&amp;IF(I176="","origen del agua · ","")&amp;IF(AND(LEFT(I176,7)="Sale de",J176="",K176=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C176:S176)=0,"",IF(AND(C176&lt;&gt;"",D176&lt;&gt;"",E176&lt;&gt;"",H176&lt;&gt;"",I176&lt;&gt;"",NOT(AND(LEFT(I176,7)="Sale de",J176="",K176=""))),"✔ Completa","Falta: "&amp;IF(C176="","fecha · ","")&amp;IF(D176="","ubicación · ","")&amp;IF(E176="","referencia · ","")&amp;IF(H176="","criticidad · ","")&amp;IF(I176="","origen del agua · ","")&amp;IF(AND(LEFT(I176,7)="Sale de",J176="",K176=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C176" s="17" t="n"/>
@@ -5951,8 +6147,9 @@
       <c r="N176" s="21" t="n"/>
       <c r="O176" s="21" t="n"/>
       <c r="P176" s="21" t="n"/>
-      <c r="Q176" s="18" t="n"/>
-      <c r="R176" s="19" t="n"/>
+      <c r="Q176" s="21" t="n"/>
+      <c r="R176" s="18" t="n"/>
+      <c r="S176" s="19" t="n"/>
     </row>
     <row r="177" ht="20" customHeight="1">
       <c r="A177" s="15" t="inlineStr">
@@ -5961,7 +6158,7 @@
         </is>
       </c>
       <c r="B177" s="16">
-        <f>IF(COUNTA(C177:R177)=0,"",IF(AND(C177&lt;&gt;"",D177&lt;&gt;"",E177&lt;&gt;"",H177&lt;&gt;"",I177&lt;&gt;"",NOT(AND(LEFT(I177,7)="Sale de",J177="",K177=""))),"✔ Completa","Falta: "&amp;IF(C177="","fecha · ","")&amp;IF(D177="","ubicación · ","")&amp;IF(E177="","referencia · ","")&amp;IF(H177="","criticidad · ","")&amp;IF(I177="","origen del agua · ","")&amp;IF(AND(LEFT(I177,7)="Sale de",J177="",K177=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C177:S177)=0,"",IF(AND(C177&lt;&gt;"",D177&lt;&gt;"",E177&lt;&gt;"",H177&lt;&gt;"",I177&lt;&gt;"",NOT(AND(LEFT(I177,7)="Sale de",J177="",K177=""))),"✔ Completa","Falta: "&amp;IF(C177="","fecha · ","")&amp;IF(D177="","ubicación · ","")&amp;IF(E177="","referencia · ","")&amp;IF(H177="","criticidad · ","")&amp;IF(I177="","origen del agua · ","")&amp;IF(AND(LEFT(I177,7)="Sale de",J177="",K177=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C177" s="17" t="n"/>
@@ -5978,8 +6175,9 @@
       <c r="N177" s="21" t="n"/>
       <c r="O177" s="21" t="n"/>
       <c r="P177" s="21" t="n"/>
-      <c r="Q177" s="18" t="n"/>
-      <c r="R177" s="19" t="n"/>
+      <c r="Q177" s="21" t="n"/>
+      <c r="R177" s="18" t="n"/>
+      <c r="S177" s="19" t="n"/>
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="15" t="inlineStr">
@@ -5988,7 +6186,7 @@
         </is>
       </c>
       <c r="B178" s="16">
-        <f>IF(COUNTA(C178:R178)=0,"",IF(AND(C178&lt;&gt;"",D178&lt;&gt;"",E178&lt;&gt;"",H178&lt;&gt;"",I178&lt;&gt;"",NOT(AND(LEFT(I178,7)="Sale de",J178="",K178=""))),"✔ Completa","Falta: "&amp;IF(C178="","fecha · ","")&amp;IF(D178="","ubicación · ","")&amp;IF(E178="","referencia · ","")&amp;IF(H178="","criticidad · ","")&amp;IF(I178="","origen del agua · ","")&amp;IF(AND(LEFT(I178,7)="Sale de",J178="",K178=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C178:S178)=0,"",IF(AND(C178&lt;&gt;"",D178&lt;&gt;"",E178&lt;&gt;"",H178&lt;&gt;"",I178&lt;&gt;"",NOT(AND(LEFT(I178,7)="Sale de",J178="",K178=""))),"✔ Completa","Falta: "&amp;IF(C178="","fecha · ","")&amp;IF(D178="","ubicación · ","")&amp;IF(E178="","referencia · ","")&amp;IF(H178="","criticidad · ","")&amp;IF(I178="","origen del agua · ","")&amp;IF(AND(LEFT(I178,7)="Sale de",J178="",K178=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C178" s="17" t="n"/>
@@ -6005,8 +6203,9 @@
       <c r="N178" s="21" t="n"/>
       <c r="O178" s="21" t="n"/>
       <c r="P178" s="21" t="n"/>
-      <c r="Q178" s="18" t="n"/>
-      <c r="R178" s="19" t="n"/>
+      <c r="Q178" s="21" t="n"/>
+      <c r="R178" s="18" t="n"/>
+      <c r="S178" s="19" t="n"/>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="15" t="inlineStr">
@@ -6015,7 +6214,7 @@
         </is>
       </c>
       <c r="B179" s="16">
-        <f>IF(COUNTA(C179:R179)=0,"",IF(AND(C179&lt;&gt;"",D179&lt;&gt;"",E179&lt;&gt;"",H179&lt;&gt;"",I179&lt;&gt;"",NOT(AND(LEFT(I179,7)="Sale de",J179="",K179=""))),"✔ Completa","Falta: "&amp;IF(C179="","fecha · ","")&amp;IF(D179="","ubicación · ","")&amp;IF(E179="","referencia · ","")&amp;IF(H179="","criticidad · ","")&amp;IF(I179="","origen del agua · ","")&amp;IF(AND(LEFT(I179,7)="Sale de",J179="",K179=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C179:S179)=0,"",IF(AND(C179&lt;&gt;"",D179&lt;&gt;"",E179&lt;&gt;"",H179&lt;&gt;"",I179&lt;&gt;"",NOT(AND(LEFT(I179,7)="Sale de",J179="",K179=""))),"✔ Completa","Falta: "&amp;IF(C179="","fecha · ","")&amp;IF(D179="","ubicación · ","")&amp;IF(E179="","referencia · ","")&amp;IF(H179="","criticidad · ","")&amp;IF(I179="","origen del agua · ","")&amp;IF(AND(LEFT(I179,7)="Sale de",J179="",K179=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C179" s="17" t="n"/>
@@ -6032,8 +6231,9 @@
       <c r="N179" s="21" t="n"/>
       <c r="O179" s="21" t="n"/>
       <c r="P179" s="21" t="n"/>
-      <c r="Q179" s="18" t="n"/>
-      <c r="R179" s="19" t="n"/>
+      <c r="Q179" s="21" t="n"/>
+      <c r="R179" s="18" t="n"/>
+      <c r="S179" s="19" t="n"/>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="15" t="inlineStr">
@@ -6042,7 +6242,7 @@
         </is>
       </c>
       <c r="B180" s="16">
-        <f>IF(COUNTA(C180:R180)=0,"",IF(AND(C180&lt;&gt;"",D180&lt;&gt;"",E180&lt;&gt;"",H180&lt;&gt;"",I180&lt;&gt;"",NOT(AND(LEFT(I180,7)="Sale de",J180="",K180=""))),"✔ Completa","Falta: "&amp;IF(C180="","fecha · ","")&amp;IF(D180="","ubicación · ","")&amp;IF(E180="","referencia · ","")&amp;IF(H180="","criticidad · ","")&amp;IF(I180="","origen del agua · ","")&amp;IF(AND(LEFT(I180,7)="Sale de",J180="",K180=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C180:S180)=0,"",IF(AND(C180&lt;&gt;"",D180&lt;&gt;"",E180&lt;&gt;"",H180&lt;&gt;"",I180&lt;&gt;"",NOT(AND(LEFT(I180,7)="Sale de",J180="",K180=""))),"✔ Completa","Falta: "&amp;IF(C180="","fecha · ","")&amp;IF(D180="","ubicación · ","")&amp;IF(E180="","referencia · ","")&amp;IF(H180="","criticidad · ","")&amp;IF(I180="","origen del agua · ","")&amp;IF(AND(LEFT(I180,7)="Sale de",J180="",K180=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C180" s="17" t="n"/>
@@ -6059,8 +6259,9 @@
       <c r="N180" s="21" t="n"/>
       <c r="O180" s="21" t="n"/>
       <c r="P180" s="21" t="n"/>
-      <c r="Q180" s="18" t="n"/>
-      <c r="R180" s="19" t="n"/>
+      <c r="Q180" s="21" t="n"/>
+      <c r="R180" s="18" t="n"/>
+      <c r="S180" s="19" t="n"/>
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="15" t="inlineStr">
@@ -6069,7 +6270,7 @@
         </is>
       </c>
       <c r="B181" s="16">
-        <f>IF(COUNTA(C181:R181)=0,"",IF(AND(C181&lt;&gt;"",D181&lt;&gt;"",E181&lt;&gt;"",H181&lt;&gt;"",I181&lt;&gt;"",NOT(AND(LEFT(I181,7)="Sale de",J181="",K181=""))),"✔ Completa","Falta: "&amp;IF(C181="","fecha · ","")&amp;IF(D181="","ubicación · ","")&amp;IF(E181="","referencia · ","")&amp;IF(H181="","criticidad · ","")&amp;IF(I181="","origen del agua · ","")&amp;IF(AND(LEFT(I181,7)="Sale de",J181="",K181=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C181:S181)=0,"",IF(AND(C181&lt;&gt;"",D181&lt;&gt;"",E181&lt;&gt;"",H181&lt;&gt;"",I181&lt;&gt;"",NOT(AND(LEFT(I181,7)="Sale de",J181="",K181=""))),"✔ Completa","Falta: "&amp;IF(C181="","fecha · ","")&amp;IF(D181="","ubicación · ","")&amp;IF(E181="","referencia · ","")&amp;IF(H181="","criticidad · ","")&amp;IF(I181="","origen del agua · ","")&amp;IF(AND(LEFT(I181,7)="Sale de",J181="",K181=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C181" s="17" t="n"/>
@@ -6086,8 +6287,9 @@
       <c r="N181" s="21" t="n"/>
       <c r="O181" s="21" t="n"/>
       <c r="P181" s="21" t="n"/>
-      <c r="Q181" s="18" t="n"/>
-      <c r="R181" s="19" t="n"/>
+      <c r="Q181" s="21" t="n"/>
+      <c r="R181" s="18" t="n"/>
+      <c r="S181" s="19" t="n"/>
     </row>
     <row r="182" ht="20" customHeight="1">
       <c r="A182" s="15" t="inlineStr">
@@ -6096,7 +6298,7 @@
         </is>
       </c>
       <c r="B182" s="16">
-        <f>IF(COUNTA(C182:R182)=0,"",IF(AND(C182&lt;&gt;"",D182&lt;&gt;"",E182&lt;&gt;"",H182&lt;&gt;"",I182&lt;&gt;"",NOT(AND(LEFT(I182,7)="Sale de",J182="",K182=""))),"✔ Completa","Falta: "&amp;IF(C182="","fecha · ","")&amp;IF(D182="","ubicación · ","")&amp;IF(E182="","referencia · ","")&amp;IF(H182="","criticidad · ","")&amp;IF(I182="","origen del agua · ","")&amp;IF(AND(LEFT(I182,7)="Sale de",J182="",K182=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C182:S182)=0,"",IF(AND(C182&lt;&gt;"",D182&lt;&gt;"",E182&lt;&gt;"",H182&lt;&gt;"",I182&lt;&gt;"",NOT(AND(LEFT(I182,7)="Sale de",J182="",K182=""))),"✔ Completa","Falta: "&amp;IF(C182="","fecha · ","")&amp;IF(D182="","ubicación · ","")&amp;IF(E182="","referencia · ","")&amp;IF(H182="","criticidad · ","")&amp;IF(I182="","origen del agua · ","")&amp;IF(AND(LEFT(I182,7)="Sale de",J182="",K182=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C182" s="17" t="n"/>
@@ -6113,8 +6315,9 @@
       <c r="N182" s="21" t="n"/>
       <c r="O182" s="21" t="n"/>
       <c r="P182" s="21" t="n"/>
-      <c r="Q182" s="18" t="n"/>
-      <c r="R182" s="19" t="n"/>
+      <c r="Q182" s="21" t="n"/>
+      <c r="R182" s="18" t="n"/>
+      <c r="S182" s="19" t="n"/>
     </row>
     <row r="183" ht="20" customHeight="1">
       <c r="A183" s="15" t="inlineStr">
@@ -6123,7 +6326,7 @@
         </is>
       </c>
       <c r="B183" s="16">
-        <f>IF(COUNTA(C183:R183)=0,"",IF(AND(C183&lt;&gt;"",D183&lt;&gt;"",E183&lt;&gt;"",H183&lt;&gt;"",I183&lt;&gt;"",NOT(AND(LEFT(I183,7)="Sale de",J183="",K183=""))),"✔ Completa","Falta: "&amp;IF(C183="","fecha · ","")&amp;IF(D183="","ubicación · ","")&amp;IF(E183="","referencia · ","")&amp;IF(H183="","criticidad · ","")&amp;IF(I183="","origen del agua · ","")&amp;IF(AND(LEFT(I183,7)="Sale de",J183="",K183=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C183:S183)=0,"",IF(AND(C183&lt;&gt;"",D183&lt;&gt;"",E183&lt;&gt;"",H183&lt;&gt;"",I183&lt;&gt;"",NOT(AND(LEFT(I183,7)="Sale de",J183="",K183=""))),"✔ Completa","Falta: "&amp;IF(C183="","fecha · ","")&amp;IF(D183="","ubicación · ","")&amp;IF(E183="","referencia · ","")&amp;IF(H183="","criticidad · ","")&amp;IF(I183="","origen del agua · ","")&amp;IF(AND(LEFT(I183,7)="Sale de",J183="",K183=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C183" s="17" t="n"/>
@@ -6140,8 +6343,9 @@
       <c r="N183" s="21" t="n"/>
       <c r="O183" s="21" t="n"/>
       <c r="P183" s="21" t="n"/>
-      <c r="Q183" s="18" t="n"/>
-      <c r="R183" s="19" t="n"/>
+      <c r="Q183" s="21" t="n"/>
+      <c r="R183" s="18" t="n"/>
+      <c r="S183" s="19" t="n"/>
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="15" t="inlineStr">
@@ -6150,7 +6354,7 @@
         </is>
       </c>
       <c r="B184" s="16">
-        <f>IF(COUNTA(C184:R184)=0,"",IF(AND(C184&lt;&gt;"",D184&lt;&gt;"",E184&lt;&gt;"",H184&lt;&gt;"",I184&lt;&gt;"",NOT(AND(LEFT(I184,7)="Sale de",J184="",K184=""))),"✔ Completa","Falta: "&amp;IF(C184="","fecha · ","")&amp;IF(D184="","ubicación · ","")&amp;IF(E184="","referencia · ","")&amp;IF(H184="","criticidad · ","")&amp;IF(I184="","origen del agua · ","")&amp;IF(AND(LEFT(I184,7)="Sale de",J184="",K184=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C184:S184)=0,"",IF(AND(C184&lt;&gt;"",D184&lt;&gt;"",E184&lt;&gt;"",H184&lt;&gt;"",I184&lt;&gt;"",NOT(AND(LEFT(I184,7)="Sale de",J184="",K184=""))),"✔ Completa","Falta: "&amp;IF(C184="","fecha · ","")&amp;IF(D184="","ubicación · ","")&amp;IF(E184="","referencia · ","")&amp;IF(H184="","criticidad · ","")&amp;IF(I184="","origen del agua · ","")&amp;IF(AND(LEFT(I184,7)="Sale de",J184="",K184=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C184" s="17" t="n"/>
@@ -6167,8 +6371,9 @@
       <c r="N184" s="21" t="n"/>
       <c r="O184" s="21" t="n"/>
       <c r="P184" s="21" t="n"/>
-      <c r="Q184" s="18" t="n"/>
-      <c r="R184" s="19" t="n"/>
+      <c r="Q184" s="21" t="n"/>
+      <c r="R184" s="18" t="n"/>
+      <c r="S184" s="19" t="n"/>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="15" t="inlineStr">
@@ -6177,7 +6382,7 @@
         </is>
       </c>
       <c r="B185" s="16">
-        <f>IF(COUNTA(C185:R185)=0,"",IF(AND(C185&lt;&gt;"",D185&lt;&gt;"",E185&lt;&gt;"",H185&lt;&gt;"",I185&lt;&gt;"",NOT(AND(LEFT(I185,7)="Sale de",J185="",K185=""))),"✔ Completa","Falta: "&amp;IF(C185="","fecha · ","")&amp;IF(D185="","ubicación · ","")&amp;IF(E185="","referencia · ","")&amp;IF(H185="","criticidad · ","")&amp;IF(I185="","origen del agua · ","")&amp;IF(AND(LEFT(I185,7)="Sale de",J185="",K185=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C185:S185)=0,"",IF(AND(C185&lt;&gt;"",D185&lt;&gt;"",E185&lt;&gt;"",H185&lt;&gt;"",I185&lt;&gt;"",NOT(AND(LEFT(I185,7)="Sale de",J185="",K185=""))),"✔ Completa","Falta: "&amp;IF(C185="","fecha · ","")&amp;IF(D185="","ubicación · ","")&amp;IF(E185="","referencia · ","")&amp;IF(H185="","criticidad · ","")&amp;IF(I185="","origen del agua · ","")&amp;IF(AND(LEFT(I185,7)="Sale de",J185="",K185=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C185" s="17" t="n"/>
@@ -6194,8 +6399,9 @@
       <c r="N185" s="21" t="n"/>
       <c r="O185" s="21" t="n"/>
       <c r="P185" s="21" t="n"/>
-      <c r="Q185" s="18" t="n"/>
-      <c r="R185" s="19" t="n"/>
+      <c r="Q185" s="21" t="n"/>
+      <c r="R185" s="18" t="n"/>
+      <c r="S185" s="19" t="n"/>
     </row>
     <row r="186" ht="20" customHeight="1">
       <c r="A186" s="15" t="inlineStr">
@@ -6204,7 +6410,7 @@
         </is>
       </c>
       <c r="B186" s="16">
-        <f>IF(COUNTA(C186:R186)=0,"",IF(AND(C186&lt;&gt;"",D186&lt;&gt;"",E186&lt;&gt;"",H186&lt;&gt;"",I186&lt;&gt;"",NOT(AND(LEFT(I186,7)="Sale de",J186="",K186=""))),"✔ Completa","Falta: "&amp;IF(C186="","fecha · ","")&amp;IF(D186="","ubicación · ","")&amp;IF(E186="","referencia · ","")&amp;IF(H186="","criticidad · ","")&amp;IF(I186="","origen del agua · ","")&amp;IF(AND(LEFT(I186,7)="Sale de",J186="",K186=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C186:S186)=0,"",IF(AND(C186&lt;&gt;"",D186&lt;&gt;"",E186&lt;&gt;"",H186&lt;&gt;"",I186&lt;&gt;"",NOT(AND(LEFT(I186,7)="Sale de",J186="",K186=""))),"✔ Completa","Falta: "&amp;IF(C186="","fecha · ","")&amp;IF(D186="","ubicación · ","")&amp;IF(E186="","referencia · ","")&amp;IF(H186="","criticidad · ","")&amp;IF(I186="","origen del agua · ","")&amp;IF(AND(LEFT(I186,7)="Sale de",J186="",K186=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C186" s="17" t="n"/>
@@ -6221,8 +6427,9 @@
       <c r="N186" s="21" t="n"/>
       <c r="O186" s="21" t="n"/>
       <c r="P186" s="21" t="n"/>
-      <c r="Q186" s="18" t="n"/>
-      <c r="R186" s="19" t="n"/>
+      <c r="Q186" s="21" t="n"/>
+      <c r="R186" s="18" t="n"/>
+      <c r="S186" s="19" t="n"/>
     </row>
     <row r="187" ht="20" customHeight="1">
       <c r="A187" s="15" t="inlineStr">
@@ -6231,7 +6438,7 @@
         </is>
       </c>
       <c r="B187" s="16">
-        <f>IF(COUNTA(C187:R187)=0,"",IF(AND(C187&lt;&gt;"",D187&lt;&gt;"",E187&lt;&gt;"",H187&lt;&gt;"",I187&lt;&gt;"",NOT(AND(LEFT(I187,7)="Sale de",J187="",K187=""))),"✔ Completa","Falta: "&amp;IF(C187="","fecha · ","")&amp;IF(D187="","ubicación · ","")&amp;IF(E187="","referencia · ","")&amp;IF(H187="","criticidad · ","")&amp;IF(I187="","origen del agua · ","")&amp;IF(AND(LEFT(I187,7)="Sale de",J187="",K187=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C187:S187)=0,"",IF(AND(C187&lt;&gt;"",D187&lt;&gt;"",E187&lt;&gt;"",H187&lt;&gt;"",I187&lt;&gt;"",NOT(AND(LEFT(I187,7)="Sale de",J187="",K187=""))),"✔ Completa","Falta: "&amp;IF(C187="","fecha · ","")&amp;IF(D187="","ubicación · ","")&amp;IF(E187="","referencia · ","")&amp;IF(H187="","criticidad · ","")&amp;IF(I187="","origen del agua · ","")&amp;IF(AND(LEFT(I187,7)="Sale de",J187="",K187=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C187" s="17" t="n"/>
@@ -6248,8 +6455,9 @@
       <c r="N187" s="21" t="n"/>
       <c r="O187" s="21" t="n"/>
       <c r="P187" s="21" t="n"/>
-      <c r="Q187" s="18" t="n"/>
-      <c r="R187" s="19" t="n"/>
+      <c r="Q187" s="21" t="n"/>
+      <c r="R187" s="18" t="n"/>
+      <c r="S187" s="19" t="n"/>
     </row>
     <row r="188" ht="20" customHeight="1">
       <c r="A188" s="15" t="inlineStr">
@@ -6258,7 +6466,7 @@
         </is>
       </c>
       <c r="B188" s="16">
-        <f>IF(COUNTA(C188:R188)=0,"",IF(AND(C188&lt;&gt;"",D188&lt;&gt;"",E188&lt;&gt;"",H188&lt;&gt;"",I188&lt;&gt;"",NOT(AND(LEFT(I188,7)="Sale de",J188="",K188=""))),"✔ Completa","Falta: "&amp;IF(C188="","fecha · ","")&amp;IF(D188="","ubicación · ","")&amp;IF(E188="","referencia · ","")&amp;IF(H188="","criticidad · ","")&amp;IF(I188="","origen del agua · ","")&amp;IF(AND(LEFT(I188,7)="Sale de",J188="",K188=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C188:S188)=0,"",IF(AND(C188&lt;&gt;"",D188&lt;&gt;"",E188&lt;&gt;"",H188&lt;&gt;"",I188&lt;&gt;"",NOT(AND(LEFT(I188,7)="Sale de",J188="",K188=""))),"✔ Completa","Falta: "&amp;IF(C188="","fecha · ","")&amp;IF(D188="","ubicación · ","")&amp;IF(E188="","referencia · ","")&amp;IF(H188="","criticidad · ","")&amp;IF(I188="","origen del agua · ","")&amp;IF(AND(LEFT(I188,7)="Sale de",J188="",K188=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C188" s="17" t="n"/>
@@ -6275,8 +6483,9 @@
       <c r="N188" s="21" t="n"/>
       <c r="O188" s="21" t="n"/>
       <c r="P188" s="21" t="n"/>
-      <c r="Q188" s="18" t="n"/>
-      <c r="R188" s="19" t="n"/>
+      <c r="Q188" s="21" t="n"/>
+      <c r="R188" s="18" t="n"/>
+      <c r="S188" s="19" t="n"/>
     </row>
     <row r="189" ht="20" customHeight="1">
       <c r="A189" s="15" t="inlineStr">
@@ -6285,7 +6494,7 @@
         </is>
       </c>
       <c r="B189" s="16">
-        <f>IF(COUNTA(C189:R189)=0,"",IF(AND(C189&lt;&gt;"",D189&lt;&gt;"",E189&lt;&gt;"",H189&lt;&gt;"",I189&lt;&gt;"",NOT(AND(LEFT(I189,7)="Sale de",J189="",K189=""))),"✔ Completa","Falta: "&amp;IF(C189="","fecha · ","")&amp;IF(D189="","ubicación · ","")&amp;IF(E189="","referencia · ","")&amp;IF(H189="","criticidad · ","")&amp;IF(I189="","origen del agua · ","")&amp;IF(AND(LEFT(I189,7)="Sale de",J189="",K189=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C189:S189)=0,"",IF(AND(C189&lt;&gt;"",D189&lt;&gt;"",E189&lt;&gt;"",H189&lt;&gt;"",I189&lt;&gt;"",NOT(AND(LEFT(I189,7)="Sale de",J189="",K189=""))),"✔ Completa","Falta: "&amp;IF(C189="","fecha · ","")&amp;IF(D189="","ubicación · ","")&amp;IF(E189="","referencia · ","")&amp;IF(H189="","criticidad · ","")&amp;IF(I189="","origen del agua · ","")&amp;IF(AND(LEFT(I189,7)="Sale de",J189="",K189=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C189" s="17" t="n"/>
@@ -6302,8 +6511,9 @@
       <c r="N189" s="21" t="n"/>
       <c r="O189" s="21" t="n"/>
       <c r="P189" s="21" t="n"/>
-      <c r="Q189" s="18" t="n"/>
-      <c r="R189" s="19" t="n"/>
+      <c r="Q189" s="21" t="n"/>
+      <c r="R189" s="18" t="n"/>
+      <c r="S189" s="19" t="n"/>
     </row>
     <row r="190" ht="20" customHeight="1">
       <c r="A190" s="15" t="inlineStr">
@@ -6312,7 +6522,7 @@
         </is>
       </c>
       <c r="B190" s="16">
-        <f>IF(COUNTA(C190:R190)=0,"",IF(AND(C190&lt;&gt;"",D190&lt;&gt;"",E190&lt;&gt;"",H190&lt;&gt;"",I190&lt;&gt;"",NOT(AND(LEFT(I190,7)="Sale de",J190="",K190=""))),"✔ Completa","Falta: "&amp;IF(C190="","fecha · ","")&amp;IF(D190="","ubicación · ","")&amp;IF(E190="","referencia · ","")&amp;IF(H190="","criticidad · ","")&amp;IF(I190="","origen del agua · ","")&amp;IF(AND(LEFT(I190,7)="Sale de",J190="",K190=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C190:S190)=0,"",IF(AND(C190&lt;&gt;"",D190&lt;&gt;"",E190&lt;&gt;"",H190&lt;&gt;"",I190&lt;&gt;"",NOT(AND(LEFT(I190,7)="Sale de",J190="",K190=""))),"✔ Completa","Falta: "&amp;IF(C190="","fecha · ","")&amp;IF(D190="","ubicación · ","")&amp;IF(E190="","referencia · ","")&amp;IF(H190="","criticidad · ","")&amp;IF(I190="","origen del agua · ","")&amp;IF(AND(LEFT(I190,7)="Sale de",J190="",K190=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C190" s="17" t="n"/>
@@ -6329,8 +6539,9 @@
       <c r="N190" s="21" t="n"/>
       <c r="O190" s="21" t="n"/>
       <c r="P190" s="21" t="n"/>
-      <c r="Q190" s="18" t="n"/>
-      <c r="R190" s="19" t="n"/>
+      <c r="Q190" s="21" t="n"/>
+      <c r="R190" s="18" t="n"/>
+      <c r="S190" s="19" t="n"/>
     </row>
     <row r="191" ht="20" customHeight="1">
       <c r="A191" s="15" t="inlineStr">
@@ -6339,7 +6550,7 @@
         </is>
       </c>
       <c r="B191" s="16">
-        <f>IF(COUNTA(C191:R191)=0,"",IF(AND(C191&lt;&gt;"",D191&lt;&gt;"",E191&lt;&gt;"",H191&lt;&gt;"",I191&lt;&gt;"",NOT(AND(LEFT(I191,7)="Sale de",J191="",K191=""))),"✔ Completa","Falta: "&amp;IF(C191="","fecha · ","")&amp;IF(D191="","ubicación · ","")&amp;IF(E191="","referencia · ","")&amp;IF(H191="","criticidad · ","")&amp;IF(I191="","origen del agua · ","")&amp;IF(AND(LEFT(I191,7)="Sale de",J191="",K191=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C191:S191)=0,"",IF(AND(C191&lt;&gt;"",D191&lt;&gt;"",E191&lt;&gt;"",H191&lt;&gt;"",I191&lt;&gt;"",NOT(AND(LEFT(I191,7)="Sale de",J191="",K191=""))),"✔ Completa","Falta: "&amp;IF(C191="","fecha · ","")&amp;IF(D191="","ubicación · ","")&amp;IF(E191="","referencia · ","")&amp;IF(H191="","criticidad · ","")&amp;IF(I191="","origen del agua · ","")&amp;IF(AND(LEFT(I191,7)="Sale de",J191="",K191=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C191" s="17" t="n"/>
@@ -6356,8 +6567,9 @@
       <c r="N191" s="21" t="n"/>
       <c r="O191" s="21" t="n"/>
       <c r="P191" s="21" t="n"/>
-      <c r="Q191" s="18" t="n"/>
-      <c r="R191" s="19" t="n"/>
+      <c r="Q191" s="21" t="n"/>
+      <c r="R191" s="18" t="n"/>
+      <c r="S191" s="19" t="n"/>
     </row>
     <row r="192" ht="20" customHeight="1">
       <c r="A192" s="15" t="inlineStr">
@@ -6366,7 +6578,7 @@
         </is>
       </c>
       <c r="B192" s="16">
-        <f>IF(COUNTA(C192:R192)=0,"",IF(AND(C192&lt;&gt;"",D192&lt;&gt;"",E192&lt;&gt;"",H192&lt;&gt;"",I192&lt;&gt;"",NOT(AND(LEFT(I192,7)="Sale de",J192="",K192=""))),"✔ Completa","Falta: "&amp;IF(C192="","fecha · ","")&amp;IF(D192="","ubicación · ","")&amp;IF(E192="","referencia · ","")&amp;IF(H192="","criticidad · ","")&amp;IF(I192="","origen del agua · ","")&amp;IF(AND(LEFT(I192,7)="Sale de",J192="",K192=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C192:S192)=0,"",IF(AND(C192&lt;&gt;"",D192&lt;&gt;"",E192&lt;&gt;"",H192&lt;&gt;"",I192&lt;&gt;"",NOT(AND(LEFT(I192,7)="Sale de",J192="",K192=""))),"✔ Completa","Falta: "&amp;IF(C192="","fecha · ","")&amp;IF(D192="","ubicación · ","")&amp;IF(E192="","referencia · ","")&amp;IF(H192="","criticidad · ","")&amp;IF(I192="","origen del agua · ","")&amp;IF(AND(LEFT(I192,7)="Sale de",J192="",K192=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C192" s="17" t="n"/>
@@ -6383,8 +6595,9 @@
       <c r="N192" s="21" t="n"/>
       <c r="O192" s="21" t="n"/>
       <c r="P192" s="21" t="n"/>
-      <c r="Q192" s="18" t="n"/>
-      <c r="R192" s="19" t="n"/>
+      <c r="Q192" s="21" t="n"/>
+      <c r="R192" s="18" t="n"/>
+      <c r="S192" s="19" t="n"/>
     </row>
     <row r="193" ht="20" customHeight="1">
       <c r="A193" s="15" t="inlineStr">
@@ -6393,7 +6606,7 @@
         </is>
       </c>
       <c r="B193" s="16">
-        <f>IF(COUNTA(C193:R193)=0,"",IF(AND(C193&lt;&gt;"",D193&lt;&gt;"",E193&lt;&gt;"",H193&lt;&gt;"",I193&lt;&gt;"",NOT(AND(LEFT(I193,7)="Sale de",J193="",K193=""))),"✔ Completa","Falta: "&amp;IF(C193="","fecha · ","")&amp;IF(D193="","ubicación · ","")&amp;IF(E193="","referencia · ","")&amp;IF(H193="","criticidad · ","")&amp;IF(I193="","origen del agua · ","")&amp;IF(AND(LEFT(I193,7)="Sale de",J193="",K193=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C193:S193)=0,"",IF(AND(C193&lt;&gt;"",D193&lt;&gt;"",E193&lt;&gt;"",H193&lt;&gt;"",I193&lt;&gt;"",NOT(AND(LEFT(I193,7)="Sale de",J193="",K193=""))),"✔ Completa","Falta: "&amp;IF(C193="","fecha · ","")&amp;IF(D193="","ubicación · ","")&amp;IF(E193="","referencia · ","")&amp;IF(H193="","criticidad · ","")&amp;IF(I193="","origen del agua · ","")&amp;IF(AND(LEFT(I193,7)="Sale de",J193="",K193=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C193" s="17" t="n"/>
@@ -6410,8 +6623,9 @@
       <c r="N193" s="21" t="n"/>
       <c r="O193" s="21" t="n"/>
       <c r="P193" s="21" t="n"/>
-      <c r="Q193" s="18" t="n"/>
-      <c r="R193" s="19" t="n"/>
+      <c r="Q193" s="21" t="n"/>
+      <c r="R193" s="18" t="n"/>
+      <c r="S193" s="19" t="n"/>
     </row>
     <row r="194" ht="20" customHeight="1">
       <c r="A194" s="15" t="inlineStr">
@@ -6420,7 +6634,7 @@
         </is>
       </c>
       <c r="B194" s="16">
-        <f>IF(COUNTA(C194:R194)=0,"",IF(AND(C194&lt;&gt;"",D194&lt;&gt;"",E194&lt;&gt;"",H194&lt;&gt;"",I194&lt;&gt;"",NOT(AND(LEFT(I194,7)="Sale de",J194="",K194=""))),"✔ Completa","Falta: "&amp;IF(C194="","fecha · ","")&amp;IF(D194="","ubicación · ","")&amp;IF(E194="","referencia · ","")&amp;IF(H194="","criticidad · ","")&amp;IF(I194="","origen del agua · ","")&amp;IF(AND(LEFT(I194,7)="Sale de",J194="",K194=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C194:S194)=0,"",IF(AND(C194&lt;&gt;"",D194&lt;&gt;"",E194&lt;&gt;"",H194&lt;&gt;"",I194&lt;&gt;"",NOT(AND(LEFT(I194,7)="Sale de",J194="",K194=""))),"✔ Completa","Falta: "&amp;IF(C194="","fecha · ","")&amp;IF(D194="","ubicación · ","")&amp;IF(E194="","referencia · ","")&amp;IF(H194="","criticidad · ","")&amp;IF(I194="","origen del agua · ","")&amp;IF(AND(LEFT(I194,7)="Sale de",J194="",K194=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C194" s="17" t="n"/>
@@ -6437,8 +6651,9 @@
       <c r="N194" s="21" t="n"/>
       <c r="O194" s="21" t="n"/>
       <c r="P194" s="21" t="n"/>
-      <c r="Q194" s="18" t="n"/>
-      <c r="R194" s="19" t="n"/>
+      <c r="Q194" s="21" t="n"/>
+      <c r="R194" s="18" t="n"/>
+      <c r="S194" s="19" t="n"/>
     </row>
     <row r="195" ht="20" customHeight="1">
       <c r="A195" s="15" t="inlineStr">
@@ -6447,7 +6662,7 @@
         </is>
       </c>
       <c r="B195" s="16">
-        <f>IF(COUNTA(C195:R195)=0,"",IF(AND(C195&lt;&gt;"",D195&lt;&gt;"",E195&lt;&gt;"",H195&lt;&gt;"",I195&lt;&gt;"",NOT(AND(LEFT(I195,7)="Sale de",J195="",K195=""))),"✔ Completa","Falta: "&amp;IF(C195="","fecha · ","")&amp;IF(D195="","ubicación · ","")&amp;IF(E195="","referencia · ","")&amp;IF(H195="","criticidad · ","")&amp;IF(I195="","origen del agua · ","")&amp;IF(AND(LEFT(I195,7)="Sale de",J195="",K195=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C195:S195)=0,"",IF(AND(C195&lt;&gt;"",D195&lt;&gt;"",E195&lt;&gt;"",H195&lt;&gt;"",I195&lt;&gt;"",NOT(AND(LEFT(I195,7)="Sale de",J195="",K195=""))),"✔ Completa","Falta: "&amp;IF(C195="","fecha · ","")&amp;IF(D195="","ubicación · ","")&amp;IF(E195="","referencia · ","")&amp;IF(H195="","criticidad · ","")&amp;IF(I195="","origen del agua · ","")&amp;IF(AND(LEFT(I195,7)="Sale de",J195="",K195=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C195" s="17" t="n"/>
@@ -6464,8 +6679,9 @@
       <c r="N195" s="21" t="n"/>
       <c r="O195" s="21" t="n"/>
       <c r="P195" s="21" t="n"/>
-      <c r="Q195" s="18" t="n"/>
-      <c r="R195" s="19" t="n"/>
+      <c r="Q195" s="21" t="n"/>
+      <c r="R195" s="18" t="n"/>
+      <c r="S195" s="19" t="n"/>
     </row>
     <row r="196" ht="20" customHeight="1">
       <c r="A196" s="15" t="inlineStr">
@@ -6474,7 +6690,7 @@
         </is>
       </c>
       <c r="B196" s="16">
-        <f>IF(COUNTA(C196:R196)=0,"",IF(AND(C196&lt;&gt;"",D196&lt;&gt;"",E196&lt;&gt;"",H196&lt;&gt;"",I196&lt;&gt;"",NOT(AND(LEFT(I196,7)="Sale de",J196="",K196=""))),"✔ Completa","Falta: "&amp;IF(C196="","fecha · ","")&amp;IF(D196="","ubicación · ","")&amp;IF(E196="","referencia · ","")&amp;IF(H196="","criticidad · ","")&amp;IF(I196="","origen del agua · ","")&amp;IF(AND(LEFT(I196,7)="Sale de",J196="",K196=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C196:S196)=0,"",IF(AND(C196&lt;&gt;"",D196&lt;&gt;"",E196&lt;&gt;"",H196&lt;&gt;"",I196&lt;&gt;"",NOT(AND(LEFT(I196,7)="Sale de",J196="",K196=""))),"✔ Completa","Falta: "&amp;IF(C196="","fecha · ","")&amp;IF(D196="","ubicación · ","")&amp;IF(E196="","referencia · ","")&amp;IF(H196="","criticidad · ","")&amp;IF(I196="","origen del agua · ","")&amp;IF(AND(LEFT(I196,7)="Sale de",J196="",K196=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C196" s="17" t="n"/>
@@ -6491,8 +6707,9 @@
       <c r="N196" s="21" t="n"/>
       <c r="O196" s="21" t="n"/>
       <c r="P196" s="21" t="n"/>
-      <c r="Q196" s="18" t="n"/>
-      <c r="R196" s="19" t="n"/>
+      <c r="Q196" s="21" t="n"/>
+      <c r="R196" s="18" t="n"/>
+      <c r="S196" s="19" t="n"/>
     </row>
     <row r="197" ht="20" customHeight="1">
       <c r="A197" s="15" t="inlineStr">
@@ -6501,7 +6718,7 @@
         </is>
       </c>
       <c r="B197" s="16">
-        <f>IF(COUNTA(C197:R197)=0,"",IF(AND(C197&lt;&gt;"",D197&lt;&gt;"",E197&lt;&gt;"",H197&lt;&gt;"",I197&lt;&gt;"",NOT(AND(LEFT(I197,7)="Sale de",J197="",K197=""))),"✔ Completa","Falta: "&amp;IF(C197="","fecha · ","")&amp;IF(D197="","ubicación · ","")&amp;IF(E197="","referencia · ","")&amp;IF(H197="","criticidad · ","")&amp;IF(I197="","origen del agua · ","")&amp;IF(AND(LEFT(I197,7)="Sale de",J197="",K197=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C197:S197)=0,"",IF(AND(C197&lt;&gt;"",D197&lt;&gt;"",E197&lt;&gt;"",H197&lt;&gt;"",I197&lt;&gt;"",NOT(AND(LEFT(I197,7)="Sale de",J197="",K197=""))),"✔ Completa","Falta: "&amp;IF(C197="","fecha · ","")&amp;IF(D197="","ubicación · ","")&amp;IF(E197="","referencia · ","")&amp;IF(H197="","criticidad · ","")&amp;IF(I197="","origen del agua · ","")&amp;IF(AND(LEFT(I197,7)="Sale de",J197="",K197=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C197" s="17" t="n"/>
@@ -6518,8 +6735,9 @@
       <c r="N197" s="21" t="n"/>
       <c r="O197" s="21" t="n"/>
       <c r="P197" s="21" t="n"/>
-      <c r="Q197" s="18" t="n"/>
-      <c r="R197" s="19" t="n"/>
+      <c r="Q197" s="21" t="n"/>
+      <c r="R197" s="18" t="n"/>
+      <c r="S197" s="19" t="n"/>
     </row>
     <row r="198" ht="20" customHeight="1">
       <c r="A198" s="15" t="inlineStr">
@@ -6528,7 +6746,7 @@
         </is>
       </c>
       <c r="B198" s="16">
-        <f>IF(COUNTA(C198:R198)=0,"",IF(AND(C198&lt;&gt;"",D198&lt;&gt;"",E198&lt;&gt;"",H198&lt;&gt;"",I198&lt;&gt;"",NOT(AND(LEFT(I198,7)="Sale de",J198="",K198=""))),"✔ Completa","Falta: "&amp;IF(C198="","fecha · ","")&amp;IF(D198="","ubicación · ","")&amp;IF(E198="","referencia · ","")&amp;IF(H198="","criticidad · ","")&amp;IF(I198="","origen del agua · ","")&amp;IF(AND(LEFT(I198,7)="Sale de",J198="",K198=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C198:S198)=0,"",IF(AND(C198&lt;&gt;"",D198&lt;&gt;"",E198&lt;&gt;"",H198&lt;&gt;"",I198&lt;&gt;"",NOT(AND(LEFT(I198,7)="Sale de",J198="",K198=""))),"✔ Completa","Falta: "&amp;IF(C198="","fecha · ","")&amp;IF(D198="","ubicación · ","")&amp;IF(E198="","referencia · ","")&amp;IF(H198="","criticidad · ","")&amp;IF(I198="","origen del agua · ","")&amp;IF(AND(LEFT(I198,7)="Sale de",J198="",K198=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C198" s="17" t="n"/>
@@ -6545,8 +6763,9 @@
       <c r="N198" s="21" t="n"/>
       <c r="O198" s="21" t="n"/>
       <c r="P198" s="21" t="n"/>
-      <c r="Q198" s="18" t="n"/>
-      <c r="R198" s="19" t="n"/>
+      <c r="Q198" s="21" t="n"/>
+      <c r="R198" s="18" t="n"/>
+      <c r="S198" s="19" t="n"/>
     </row>
     <row r="199" ht="20" customHeight="1">
       <c r="A199" s="15" t="inlineStr">
@@ -6555,7 +6774,7 @@
         </is>
       </c>
       <c r="B199" s="16">
-        <f>IF(COUNTA(C199:R199)=0,"",IF(AND(C199&lt;&gt;"",D199&lt;&gt;"",E199&lt;&gt;"",H199&lt;&gt;"",I199&lt;&gt;"",NOT(AND(LEFT(I199,7)="Sale de",J199="",K199=""))),"✔ Completa","Falta: "&amp;IF(C199="","fecha · ","")&amp;IF(D199="","ubicación · ","")&amp;IF(E199="","referencia · ","")&amp;IF(H199="","criticidad · ","")&amp;IF(I199="","origen del agua · ","")&amp;IF(AND(LEFT(I199,7)="Sale de",J199="",K199=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C199:S199)=0,"",IF(AND(C199&lt;&gt;"",D199&lt;&gt;"",E199&lt;&gt;"",H199&lt;&gt;"",I199&lt;&gt;"",NOT(AND(LEFT(I199,7)="Sale de",J199="",K199=""))),"✔ Completa","Falta: "&amp;IF(C199="","fecha · ","")&amp;IF(D199="","ubicación · ","")&amp;IF(E199="","referencia · ","")&amp;IF(H199="","criticidad · ","")&amp;IF(I199="","origen del agua · ","")&amp;IF(AND(LEFT(I199,7)="Sale de",J199="",K199=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C199" s="17" t="n"/>
@@ -6572,8 +6791,9 @@
       <c r="N199" s="21" t="n"/>
       <c r="O199" s="21" t="n"/>
       <c r="P199" s="21" t="n"/>
-      <c r="Q199" s="18" t="n"/>
-      <c r="R199" s="19" t="n"/>
+      <c r="Q199" s="21" t="n"/>
+      <c r="R199" s="18" t="n"/>
+      <c r="S199" s="19" t="n"/>
     </row>
     <row r="200" ht="20" customHeight="1">
       <c r="A200" s="15" t="inlineStr">
@@ -6582,7 +6802,7 @@
         </is>
       </c>
       <c r="B200" s="16">
-        <f>IF(COUNTA(C200:R200)=0,"",IF(AND(C200&lt;&gt;"",D200&lt;&gt;"",E200&lt;&gt;"",H200&lt;&gt;"",I200&lt;&gt;"",NOT(AND(LEFT(I200,7)="Sale de",J200="",K200=""))),"✔ Completa","Falta: "&amp;IF(C200="","fecha · ","")&amp;IF(D200="","ubicación · ","")&amp;IF(E200="","referencia · ","")&amp;IF(H200="","criticidad · ","")&amp;IF(I200="","origen del agua · ","")&amp;IF(AND(LEFT(I200,7)="Sale de",J200="",K200=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C200:S200)=0,"",IF(AND(C200&lt;&gt;"",D200&lt;&gt;"",E200&lt;&gt;"",H200&lt;&gt;"",I200&lt;&gt;"",NOT(AND(LEFT(I200,7)="Sale de",J200="",K200=""))),"✔ Completa","Falta: "&amp;IF(C200="","fecha · ","")&amp;IF(D200="","ubicación · ","")&amp;IF(E200="","referencia · ","")&amp;IF(H200="","criticidad · ","")&amp;IF(I200="","origen del agua · ","")&amp;IF(AND(LEFT(I200,7)="Sale de",J200="",K200=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C200" s="17" t="n"/>
@@ -6599,8 +6819,9 @@
       <c r="N200" s="21" t="n"/>
       <c r="O200" s="21" t="n"/>
       <c r="P200" s="21" t="n"/>
-      <c r="Q200" s="18" t="n"/>
-      <c r="R200" s="19" t="n"/>
+      <c r="Q200" s="21" t="n"/>
+      <c r="R200" s="18" t="n"/>
+      <c r="S200" s="19" t="n"/>
     </row>
     <row r="201" ht="20" customHeight="1">
       <c r="A201" s="15" t="inlineStr">
@@ -6609,7 +6830,7 @@
         </is>
       </c>
       <c r="B201" s="16">
-        <f>IF(COUNTA(C201:R201)=0,"",IF(AND(C201&lt;&gt;"",D201&lt;&gt;"",E201&lt;&gt;"",H201&lt;&gt;"",I201&lt;&gt;"",NOT(AND(LEFT(I201,7)="Sale de",J201="",K201=""))),"✔ Completa","Falta: "&amp;IF(C201="","fecha · ","")&amp;IF(D201="","ubicación · ","")&amp;IF(E201="","referencia · ","")&amp;IF(H201="","criticidad · ","")&amp;IF(I201="","origen del agua · ","")&amp;IF(AND(LEFT(I201,7)="Sale de",J201="",K201=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C201:S201)=0,"",IF(AND(C201&lt;&gt;"",D201&lt;&gt;"",E201&lt;&gt;"",H201&lt;&gt;"",I201&lt;&gt;"",NOT(AND(LEFT(I201,7)="Sale de",J201="",K201=""))),"✔ Completa","Falta: "&amp;IF(C201="","fecha · ","")&amp;IF(D201="","ubicación · ","")&amp;IF(E201="","referencia · ","")&amp;IF(H201="","criticidad · ","")&amp;IF(I201="","origen del agua · ","")&amp;IF(AND(LEFT(I201,7)="Sale de",J201="",K201=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C201" s="17" t="n"/>
@@ -6626,8 +6847,9 @@
       <c r="N201" s="21" t="n"/>
       <c r="O201" s="21" t="n"/>
       <c r="P201" s="21" t="n"/>
-      <c r="Q201" s="18" t="n"/>
-      <c r="R201" s="19" t="n"/>
+      <c r="Q201" s="21" t="n"/>
+      <c r="R201" s="18" t="n"/>
+      <c r="S201" s="19" t="n"/>
     </row>
     <row r="202" ht="20" customHeight="1">
       <c r="A202" s="15" t="inlineStr">
@@ -6636,7 +6858,7 @@
         </is>
       </c>
       <c r="B202" s="16">
-        <f>IF(COUNTA(C202:R202)=0,"",IF(AND(C202&lt;&gt;"",D202&lt;&gt;"",E202&lt;&gt;"",H202&lt;&gt;"",I202&lt;&gt;"",NOT(AND(LEFT(I202,7)="Sale de",J202="",K202=""))),"✔ Completa","Falta: "&amp;IF(C202="","fecha · ","")&amp;IF(D202="","ubicación · ","")&amp;IF(E202="","referencia · ","")&amp;IF(H202="","criticidad · ","")&amp;IF(I202="","origen del agua · ","")&amp;IF(AND(LEFT(I202,7)="Sale de",J202="",K202=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C202:S202)=0,"",IF(AND(C202&lt;&gt;"",D202&lt;&gt;"",E202&lt;&gt;"",H202&lt;&gt;"",I202&lt;&gt;"",NOT(AND(LEFT(I202,7)="Sale de",J202="",K202=""))),"✔ Completa","Falta: "&amp;IF(C202="","fecha · ","")&amp;IF(D202="","ubicación · ","")&amp;IF(E202="","referencia · ","")&amp;IF(H202="","criticidad · ","")&amp;IF(I202="","origen del agua · ","")&amp;IF(AND(LEFT(I202,7)="Sale de",J202="",K202=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C202" s="17" t="n"/>
@@ -6653,8 +6875,9 @@
       <c r="N202" s="21" t="n"/>
       <c r="O202" s="21" t="n"/>
       <c r="P202" s="21" t="n"/>
-      <c r="Q202" s="18" t="n"/>
-      <c r="R202" s="19" t="n"/>
+      <c r="Q202" s="21" t="n"/>
+      <c r="R202" s="18" t="n"/>
+      <c r="S202" s="19" t="n"/>
     </row>
     <row r="203" ht="20" customHeight="1">
       <c r="A203" s="15" t="inlineStr">
@@ -6663,7 +6886,7 @@
         </is>
       </c>
       <c r="B203" s="16">
-        <f>IF(COUNTA(C203:R203)=0,"",IF(AND(C203&lt;&gt;"",D203&lt;&gt;"",E203&lt;&gt;"",H203&lt;&gt;"",I203&lt;&gt;"",NOT(AND(LEFT(I203,7)="Sale de",J203="",K203=""))),"✔ Completa","Falta: "&amp;IF(C203="","fecha · ","")&amp;IF(D203="","ubicación · ","")&amp;IF(E203="","referencia · ","")&amp;IF(H203="","criticidad · ","")&amp;IF(I203="","origen del agua · ","")&amp;IF(AND(LEFT(I203,7)="Sale de",J203="",K203=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C203:S203)=0,"",IF(AND(C203&lt;&gt;"",D203&lt;&gt;"",E203&lt;&gt;"",H203&lt;&gt;"",I203&lt;&gt;"",NOT(AND(LEFT(I203,7)="Sale de",J203="",K203=""))),"✔ Completa","Falta: "&amp;IF(C203="","fecha · ","")&amp;IF(D203="","ubicación · ","")&amp;IF(E203="","referencia · ","")&amp;IF(H203="","criticidad · ","")&amp;IF(I203="","origen del agua · ","")&amp;IF(AND(LEFT(I203,7)="Sale de",J203="",K203=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C203" s="17" t="n"/>
@@ -6680,8 +6903,9 @@
       <c r="N203" s="21" t="n"/>
       <c r="O203" s="21" t="n"/>
       <c r="P203" s="21" t="n"/>
-      <c r="Q203" s="18" t="n"/>
-      <c r="R203" s="19" t="n"/>
+      <c r="Q203" s="21" t="n"/>
+      <c r="R203" s="18" t="n"/>
+      <c r="S203" s="19" t="n"/>
     </row>
     <row r="204" ht="20" customHeight="1">
       <c r="A204" s="15" t="inlineStr">
@@ -6690,7 +6914,7 @@
         </is>
       </c>
       <c r="B204" s="16">
-        <f>IF(COUNTA(C204:R204)=0,"",IF(AND(C204&lt;&gt;"",D204&lt;&gt;"",E204&lt;&gt;"",H204&lt;&gt;"",I204&lt;&gt;"",NOT(AND(LEFT(I204,7)="Sale de",J204="",K204=""))),"✔ Completa","Falta: "&amp;IF(C204="","fecha · ","")&amp;IF(D204="","ubicación · ","")&amp;IF(E204="","referencia · ","")&amp;IF(H204="","criticidad · ","")&amp;IF(I204="","origen del agua · ","")&amp;IF(AND(LEFT(I204,7)="Sale de",J204="",K204=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C204:S204)=0,"",IF(AND(C204&lt;&gt;"",D204&lt;&gt;"",E204&lt;&gt;"",H204&lt;&gt;"",I204&lt;&gt;"",NOT(AND(LEFT(I204,7)="Sale de",J204="",K204=""))),"✔ Completa","Falta: "&amp;IF(C204="","fecha · ","")&amp;IF(D204="","ubicación · ","")&amp;IF(E204="","referencia · ","")&amp;IF(H204="","criticidad · ","")&amp;IF(I204="","origen del agua · ","")&amp;IF(AND(LEFT(I204,7)="Sale de",J204="",K204=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C204" s="17" t="n"/>
@@ -6707,8 +6931,9 @@
       <c r="N204" s="21" t="n"/>
       <c r="O204" s="21" t="n"/>
       <c r="P204" s="21" t="n"/>
-      <c r="Q204" s="18" t="n"/>
-      <c r="R204" s="19" t="n"/>
+      <c r="Q204" s="21" t="n"/>
+      <c r="R204" s="18" t="n"/>
+      <c r="S204" s="19" t="n"/>
     </row>
     <row r="205" ht="20" customHeight="1">
       <c r="A205" s="15" t="inlineStr">
@@ -6717,7 +6942,7 @@
         </is>
       </c>
       <c r="B205" s="16">
-        <f>IF(COUNTA(C205:R205)=0,"",IF(AND(C205&lt;&gt;"",D205&lt;&gt;"",E205&lt;&gt;"",H205&lt;&gt;"",I205&lt;&gt;"",NOT(AND(LEFT(I205,7)="Sale de",J205="",K205=""))),"✔ Completa","Falta: "&amp;IF(C205="","fecha · ","")&amp;IF(D205="","ubicación · ","")&amp;IF(E205="","referencia · ","")&amp;IF(H205="","criticidad · ","")&amp;IF(I205="","origen del agua · ","")&amp;IF(AND(LEFT(I205,7)="Sale de",J205="",K205=""),"lote de origen · ","")))</f>
+        <f>IF(COUNTA(C205:S205)=0,"",IF(AND(C205&lt;&gt;"",D205&lt;&gt;"",E205&lt;&gt;"",H205&lt;&gt;"",I205&lt;&gt;"",NOT(AND(LEFT(I205,7)="Sale de",J205="",K205=""))),"✔ Completa","Falta: "&amp;IF(C205="","fecha · ","")&amp;IF(D205="","ubicación · ","")&amp;IF(E205="","referencia · ","")&amp;IF(H205="","criticidad · ","")&amp;IF(I205="","origen del agua · ","")&amp;IF(AND(LEFT(I205,7)="Sale de",J205="",K205=""),"lote de origen · ","")))</f>
         <v/>
       </c>
       <c r="C205" s="17" t="n"/>
@@ -6734,12 +6959,13 @@
       <c r="N205" s="21" t="n"/>
       <c r="O205" s="21" t="n"/>
       <c r="P205" s="21" t="n"/>
-      <c r="Q205" s="18" t="n"/>
-      <c r="R205" s="19" t="n"/>
+      <c r="Q205" s="21" t="n"/>
+      <c r="R205" s="18" t="n"/>
+      <c r="S205" s="19" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
-  <autoFilter ref="A5:R205"/>
+  <autoFilter ref="A5:S205"/>
   <conditionalFormatting sqref="H6:H205">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT($H6,4)="Rojo"</formula>
@@ -6759,7 +6985,7 @@
       <formula>LEFT($B6,5)="Falta"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation sqref="C6:C205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escriba la fecha como dd/mm/aaaa." type="date" operator="greaterThanOrEqual">
       <formula1>DATE(2025,1,1)</formula1>
     </dataValidation>
@@ -6790,6 +7016,9 @@
     <dataValidation sqref="P6:P205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Escriba solo un número." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
+    <dataValidation sqref="Q6:Q205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Escriba solo un número." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>